<commit_message>
Read all sheets from excel file into Records
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/lucasja_rose-hulman_edu/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96303D34-571E-4205-A343-0BD2D91829A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{929C0295-FFF7-4442-A7F8-B9615CC42371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="3" activeTab="3" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="3" activeTab="4" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="258">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -403,7 +403,10 @@
     <t>OS</t>
   </si>
   <si>
-    <t>RAM</t>
+    <t>RAM Amount</t>
+  </si>
+  <si>
+    <t>RAM Generation</t>
   </si>
   <si>
     <t>Storage</t>
@@ -430,10 +433,7 @@
     <t>Vanilla OS</t>
   </si>
   <si>
-    <t>4GB DDR3</t>
-  </si>
-  <si>
-    <t>256GB</t>
+    <t>DDR3</t>
   </si>
   <si>
     <t>SSD</t>
@@ -445,16 +445,13 @@
     <t>Inspiron 15-3552</t>
   </si>
   <si>
-    <t>8GB DDR3</t>
-  </si>
-  <si>
     <t>Asus Chromebox Thin Cilent 3</t>
   </si>
   <si>
     <t>Intel Celeron 3865U</t>
   </si>
   <si>
-    <t>8GB DDR4</t>
+    <t>DDR4</t>
   </si>
   <si>
     <t>intel core i3-7100</t>
@@ -514,9 +511,6 @@
     <t>Intel Core i5-8265U</t>
   </si>
   <si>
-    <t xml:space="preserve"> 8GB DDR4</t>
-  </si>
-  <si>
     <t>HP ProBook 450 G8</t>
   </si>
   <si>
@@ -526,12 +520,6 @@
     <t>Intel Core i7-6700</t>
   </si>
   <si>
-    <t>16GB DDR4</t>
-  </si>
-  <si>
-    <t>500GB</t>
-  </si>
-  <si>
     <t>HP Elitebook 850 G6</t>
   </si>
   <si>
@@ -577,18 +565,12 @@
     <t>Intel core i7-8665U</t>
   </si>
   <si>
-    <t>16gb DDR4 2400 MT/s</t>
-  </si>
-  <si>
     <t>HP 15-AC113CL</t>
   </si>
   <si>
     <t>Intel core i3-5005U</t>
   </si>
   <si>
-    <t>8gb DDR3 1600 MT/s</t>
-  </si>
-  <si>
     <t>Toshiba Satellite C55-B5296</t>
   </si>
   <si>
@@ -604,18 +586,12 @@
     <t>Intel core i7-8565U</t>
   </si>
   <si>
-    <t>16GB DDR4 2400 MT/s</t>
-  </si>
-  <si>
     <t>Dell Latitude 5420</t>
   </si>
   <si>
     <t>Intel core i5-1145G7</t>
   </si>
   <si>
-    <t>16GB DDR4 3200 MT/s</t>
-  </si>
-  <si>
     <t>Apple iPad Mini A1455</t>
   </si>
   <si>
@@ -625,10 +601,10 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>iOS 9.3.6</t>
-  </si>
-  <si>
-    <t>64GB</t>
+    <t>iOS</t>
+  </si>
+  <si>
+    <t>DDR2</t>
   </si>
   <si>
     <t>Flash Storage</t>
@@ -640,12 +616,6 @@
     <t>Apple iPad Air 2 A1566</t>
   </si>
   <si>
-    <t>iOS 15.8.5</t>
-  </si>
-  <si>
-    <t>128GB</t>
-  </si>
-  <si>
     <t>Dell OptiPlex 5060</t>
   </si>
   <si>
@@ -664,9 +634,6 @@
     <t>Wifi included</t>
   </si>
   <si>
-    <t>SFF Desktop</t>
-  </si>
-  <si>
     <t>Intel i7-6700</t>
   </si>
   <si>
@@ -685,19 +652,10 @@
     <t>Intel i7-4770</t>
   </si>
   <si>
-    <t>16GB DDR3</t>
-  </si>
-  <si>
     <t>ThinkPad P1 Gen 1</t>
   </si>
   <si>
     <t>Intel i7 10750H</t>
-  </si>
-  <si>
-    <t>512GB</t>
-  </si>
-  <si>
-    <t>Mini Desktop</t>
   </si>
   <si>
     <t>Intel i3-7100</t>
@@ -1059,7 +1017,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="49">
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1073,6 +1031,118 @@
           <color theme="4" tint="0.39997558519241921"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1113,6 +1183,142 @@
           <color theme="4" tint="0.39997558519241921"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1239,7 +1445,7 @@
     <tableColumn id="13" xr3:uid="{5BEE40AD-E450-4A13-BFB5-1D0CED084DB3}" name="ID"/>
     <tableColumn id="8" xr3:uid="{E9AB9B46-3541-4715-8E5B-024096D78342}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{F7DAC8DD-8096-40F1-8780-1DB9CB4EC72F}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="48"/>
     <tableColumn id="5" xr3:uid="{5338F6FB-43B0-44AF-AF8B-542FAC6CEDF0}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{64D6C993-8518-4A7C-9BDA-A54D7DBFBA8E}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{E5D987A3-C54A-4907-B710-79DB224E0008}" name="Current Status" totalsRowFunction="count"/>
@@ -1258,7 +1464,7 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F96A3CC8-25D1-4CF8-877D-2816B26B7DC4}" name="Item Name" totalsRowLabel="Total"/>
-    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="16"/>
+    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="45"/>
     <tableColumn id="8" xr3:uid="{7D8F815E-A974-42A8-AC0B-AB8B951599A2}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{FEA94C75-B538-448A-A9F5-46F5A27E863D}" name="Year released"/>
     <tableColumn id="4" xr3:uid="{24998D92-36B7-4553-81E7-CB33711B31BB}" name="Special Reqs/Notes"/>
@@ -1280,7 +1486,7 @@
     <tableColumn id="13" xr3:uid="{EFFF3477-1A58-41CD-BFF3-45CE299505A7}" name="ID"/>
     <tableColumn id="8" xr3:uid="{C694899F-E385-4DE2-972A-7395A9633019}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{13C54556-A90A-4F9C-800D-3D838462DF46}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="44"/>
     <tableColumn id="5" xr3:uid="{6DE19FBC-9BD8-456E-9FC5-F633F61E4A34}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{68546225-0A78-43C1-A4F9-4D2E1DC008A3}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{0D7FD365-4F73-4A57-B8A1-CFAC47267923}" name="Current Status" totalsRowFunction="count"/>
@@ -1291,19 +1497,20 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:K33" totalsRowShown="0" tableBorderDxfId="8">
-  <autoFilter ref="A2:K33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="21">
+  <autoFilter ref="A2:L33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{73648E04-2EA1-4ADB-8E24-E7DDE01C0462}" name="Item"/>
     <tableColumn id="10" xr3:uid="{2C0BEEB0-DF56-4C3E-A199-8338A12BCED4}" name="Type of Device"/>
     <tableColumn id="3" xr3:uid="{6E6AE907-D46F-4E72-8A6E-4086D6ED467F}" name="Est. Year"/>
     <tableColumn id="4" xr3:uid="{21962421-D6C5-44DF-8B4E-CE81A5E85189}" name="CPU"/>
     <tableColumn id="5" xr3:uid="{CA276052-8A68-41FA-B502-833DDEE2F0F8}" name="OS"/>
-    <tableColumn id="6" xr3:uid="{38C5F018-4493-43C4-9328-52082FCC36C1}" name="RAM"/>
+    <tableColumn id="6" xr3:uid="{38C5F018-4493-43C4-9328-52082FCC36C1}" name="RAM Amount"/>
+    <tableColumn id="2" xr3:uid="{C85B34EB-06B2-40A8-BBCB-B5F170EF3F82}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{A686D1B3-031E-4544-A98D-8F3144FA62B0}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{AB29939A-0AF4-4451-A6F4-2144F8957E73}" name="SSD/HDD"/>
-    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="19"/>
     <tableColumn id="12" xr3:uid="{67EC036F-98F6-4C6B-BDD7-99DB9B6ADF97}" name="ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1311,15 +1518,16 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:L59" totalsRowShown="0" tableBorderDxfId="2">
-  <autoFilter ref="A2:L59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="2">
+  <autoFilter ref="A2:M59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{D71C6020-33AC-4F3C-BC88-69BADE52FD9C}" name="Item"/>
     <tableColumn id="11" xr3:uid="{3694AE3D-BABD-4C86-8092-3A4D6CE18FE9}" name="Type of Device"/>
     <tableColumn id="3" xr3:uid="{DBF01EDE-E989-4722-BA17-4F2F168FA1B7}" name="Est. Year"/>
     <tableColumn id="4" xr3:uid="{8A83BF41-D4B3-47AF-9A4E-D470FED11493}" name="CPU"/>
     <tableColumn id="5" xr3:uid="{5A855548-F141-4612-89D9-87C3C3042FDB}" name="OS"/>
-    <tableColumn id="6" xr3:uid="{7C6B1539-F50D-45A7-A8CD-94746983CE20}" name="RAM"/>
+    <tableColumn id="6" xr3:uid="{7C6B1539-F50D-45A7-A8CD-94746983CE20}" name="RAM Amount"/>
+    <tableColumn id="13" xr3:uid="{D6E0079E-D628-428A-8C40-CC4B7F920E56}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{7319329B-DA0F-470E-AE1F-CAF023744072}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{96CAC308-4A56-4EA5-AF3F-FCAC656EEA09}" name="SSD/HDD"/>
     <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="1"/>
@@ -3741,12 +3949,12 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:G63">
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="47" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:G63">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="46" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3993,21 +4201,23 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE86381-3E33-4CB8-A62B-E48A74AB9667}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" customWidth="1"/>
-    <col min="9" max="9" width="18.7109375" style="19" customWidth="1"/>
-    <col min="10" max="10" width="21.28515625" customWidth="1"/>
-    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="4" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="19" customWidth="1"/>
+    <col min="11" max="11" width="21.28515625" customWidth="1"/>
+    <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="23" t="s">
         <v>114</v>
       </c>
@@ -4021,8 +4231,9 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
       <c r="K1" s="24"/>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="L1" s="24"/>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>115</v>
       </c>
@@ -4047,50 +4258,56 @@
       <c r="H2" t="s">
         <v>122</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" t="s">
         <v>123</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="19" t="s">
         <v>124</v>
       </c>
       <c r="K2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C3">
         <v>2013</v>
       </c>
       <c r="D3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E3" t="s">
-        <v>128</v>
-      </c>
-      <c r="F3" t="s">
         <v>129</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
       </c>
       <c r="G3" t="s">
         <v>130</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3">
+        <v>256</v>
+      </c>
+      <c r="I3" t="s">
         <v>131</v>
       </c>
-      <c r="I3" s="19">
+      <c r="J3" s="19">
         <v>100</v>
       </c>
-      <c r="J3" s="1"/>
-      <c r="K3">
+      <c r="K3" s="1"/>
+      <c r="L3">
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -4104,166 +4321,181 @@
         <v>133</v>
       </c>
       <c r="E4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F4" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F4">
+        <v>8</v>
       </c>
       <c r="G4" t="s">
         <v>130</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4">
+        <v>256</v>
+      </c>
+      <c r="I4" t="s">
         <v>131</v>
       </c>
-      <c r="I4" s="19">
+      <c r="J4" s="19">
         <v>200</v>
       </c>
-      <c r="J4" s="1"/>
-      <c r="K4">
+      <c r="K4" s="1"/>
+      <c r="L4">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C5">
         <v>2018</v>
       </c>
       <c r="D5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
         <v>136</v>
       </c>
-      <c r="E5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F5" t="s">
-        <v>137</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="H5">
+        <v>256</v>
+      </c>
+      <c r="I5" t="s">
         <v>131</v>
       </c>
-      <c r="I5" s="19">
+      <c r="J5" s="19">
         <v>175</v>
       </c>
-      <c r="J5" s="1"/>
-      <c r="K5">
+      <c r="K5" s="1"/>
+      <c r="L5">
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:11">
+    <row r="6" spans="1:12">
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C7">
         <v>2018</v>
       </c>
       <c r="D7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E7" t="s">
-        <v>128</v>
-      </c>
-      <c r="F7" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>130</v>
-      </c>
-      <c r="H7" t="s">
+        <v>136</v>
+      </c>
+      <c r="H7">
+        <v>256</v>
+      </c>
+      <c r="I7" t="s">
         <v>131</v>
       </c>
-      <c r="I7" s="19">
+      <c r="J7" s="19">
         <v>175</v>
       </c>
-      <c r="J7" s="1"/>
-      <c r="K7">
+      <c r="K7" s="1"/>
+      <c r="L7">
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
         <v>92</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C8">
         <v>2018</v>
       </c>
       <c r="D8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F8">
+        <v>8</v>
+      </c>
+      <c r="G8" t="s">
+        <v>136</v>
+      </c>
+      <c r="H8">
+        <v>256</v>
+      </c>
+      <c r="I8" t="s">
+        <v>131</v>
+      </c>
+      <c r="J8" s="19">
+        <v>175</v>
+      </c>
+      <c r="K8" s="1"/>
+      <c r="L8">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
         <v>139</v>
       </c>
-      <c r="E8" t="s">
-        <v>128</v>
-      </c>
-      <c r="F8" t="s">
-        <v>137</v>
-      </c>
-      <c r="G8" t="s">
-        <v>130</v>
-      </c>
-      <c r="H8" t="s">
-        <v>131</v>
-      </c>
-      <c r="I8" s="19">
-        <v>175</v>
-      </c>
-      <c r="J8" s="1"/>
-      <c r="K8">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" t="s">
-        <v>140</v>
-      </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C9">
         <v>2018</v>
       </c>
       <c r="D9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>136</v>
+      </c>
+      <c r="H9">
+        <v>256</v>
+      </c>
+      <c r="I9" t="s">
+        <v>131</v>
+      </c>
+      <c r="J9" s="19">
+        <v>150</v>
+      </c>
+      <c r="K9" s="1"/>
+      <c r="L9">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
         <v>141</v>
-      </c>
-      <c r="E9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G9" t="s">
-        <v>130</v>
-      </c>
-      <c r="H9" t="s">
-        <v>131</v>
-      </c>
-      <c r="I9" s="19">
-        <v>150</v>
-      </c>
-      <c r="J9" s="1"/>
-      <c r="K9">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" t="s">
-        <v>142</v>
       </c>
       <c r="B11" t="s">
         <v>132</v>
@@ -4272,63 +4504,69 @@
         <v>2020</v>
       </c>
       <c r="D11" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11" t="s">
         <v>143</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
+        <v>136</v>
+      </c>
+      <c r="H11">
+        <v>256</v>
+      </c>
+      <c r="I11" t="s">
+        <v>131</v>
+      </c>
+      <c r="J11" s="19">
+        <v>300</v>
+      </c>
+      <c r="K11" s="1"/>
+      <c r="L11">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
         <v>144</v>
       </c>
-      <c r="F11" t="s">
-        <v>137</v>
-      </c>
-      <c r="G11" t="s">
-        <v>130</v>
-      </c>
-      <c r="H11" t="s">
-        <v>131</v>
-      </c>
-      <c r="I11" s="19">
-        <v>300</v>
-      </c>
-      <c r="J11" s="1"/>
-      <c r="K11">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
-      <c r="A12" t="s">
-        <v>145</v>
-      </c>
       <c r="B12" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C12">
         <v>2014</v>
       </c>
       <c r="D12" t="s">
+        <v>145</v>
+      </c>
+      <c r="E12" t="s">
+        <v>129</v>
+      </c>
+      <c r="F12">
+        <v>8</v>
+      </c>
+      <c r="G12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H12">
+        <v>256</v>
+      </c>
+      <c r="I12" t="s">
+        <v>131</v>
+      </c>
+      <c r="J12" s="2">
+        <v>175</v>
+      </c>
+      <c r="L12">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
         <v>146</v>
-      </c>
-      <c r="E12" t="s">
-        <v>128</v>
-      </c>
-      <c r="F12" t="s">
-        <v>134</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="H12" t="s">
-        <v>131</v>
-      </c>
-      <c r="I12" s="2">
-        <v>175</v>
-      </c>
-      <c r="K12">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
-      <c r="A13" t="s">
-        <v>147</v>
       </c>
       <c r="B13" t="s">
         <v>132</v>
@@ -4337,31 +4575,34 @@
         <v>2018</v>
       </c>
       <c r="D13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F13" t="s">
-        <v>137</v>
+        <v>143</v>
+      </c>
+      <c r="F13">
+        <v>8</v>
       </c>
       <c r="G13" t="s">
-        <v>130</v>
-      </c>
-      <c r="H13" t="s">
+        <v>136</v>
+      </c>
+      <c r="H13">
+        <v>256</v>
+      </c>
+      <c r="I13" t="s">
         <v>131</v>
       </c>
-      <c r="I13" s="19">
+      <c r="J13" s="19">
         <v>120</v>
       </c>
-      <c r="J13" s="1"/>
-      <c r="K13">
+      <c r="K13" s="1"/>
+      <c r="L13">
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15" customHeight="1">
+    <row r="14" spans="1:12" ht="15" customHeight="1">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B14" t="s">
         <v>132</v>
@@ -4370,31 +4611,34 @@
         <v>2018</v>
       </c>
       <c r="D14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E14" t="s">
-        <v>128</v>
-      </c>
-      <c r="F14" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F14">
+        <v>8</v>
       </c>
       <c r="G14" t="s">
-        <v>130</v>
-      </c>
-      <c r="H14" t="s">
+        <v>136</v>
+      </c>
+      <c r="H14">
+        <v>256</v>
+      </c>
+      <c r="I14" t="s">
         <v>131</v>
       </c>
-      <c r="I14" s="19">
+      <c r="J14" s="19">
         <v>175</v>
       </c>
-      <c r="J14" s="1"/>
-      <c r="K14">
+      <c r="K14" s="1"/>
+      <c r="L14">
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15" customHeight="1">
+    <row r="15" spans="1:12" ht="15" customHeight="1">
       <c r="A15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B15" t="s">
         <v>132</v>
@@ -4403,29 +4647,32 @@
         <v>2013</v>
       </c>
       <c r="D15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E15" t="s">
-        <v>128</v>
-      </c>
-      <c r="F15" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F15">
+        <v>8</v>
       </c>
       <c r="G15" t="s">
         <v>130</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15">
+        <v>256</v>
+      </c>
+      <c r="I15" t="s">
         <v>131</v>
       </c>
-      <c r="I15" s="19">
+      <c r="J15" s="19">
         <v>150</v>
       </c>
-      <c r="J15" s="1"/>
-      <c r="K15">
+      <c r="K15" s="1"/>
+      <c r="L15">
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15" customHeight="1">
+    <row r="16" spans="1:12" ht="15" customHeight="1">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -4436,31 +4683,34 @@
         <v>2019</v>
       </c>
       <c r="D16" t="s">
+        <v>150</v>
+      </c>
+      <c r="E16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F16">
+        <v>8</v>
+      </c>
+      <c r="G16" t="s">
+        <v>136</v>
+      </c>
+      <c r="H16">
+        <v>256</v>
+      </c>
+      <c r="I16" t="s">
+        <v>131</v>
+      </c>
+      <c r="J16" s="19">
+        <v>265</v>
+      </c>
+      <c r="K16" s="1"/>
+      <c r="L16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="15" customHeight="1">
+      <c r="A17" t="s">
         <v>151</v>
-      </c>
-      <c r="E16" t="s">
-        <v>144</v>
-      </c>
-      <c r="F16" t="s">
-        <v>137</v>
-      </c>
-      <c r="G16" t="s">
-        <v>130</v>
-      </c>
-      <c r="H16" t="s">
-        <v>131</v>
-      </c>
-      <c r="I16" s="19">
-        <v>265</v>
-      </c>
-      <c r="J16" s="1"/>
-      <c r="K16">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="15" customHeight="1">
-      <c r="A17" t="s">
-        <v>152</v>
       </c>
       <c r="B17" t="s">
         <v>132</v>
@@ -4469,31 +4719,34 @@
         <v>2014</v>
       </c>
       <c r="D17" t="s">
+        <v>152</v>
+      </c>
+      <c r="E17" t="s">
         <v>153</v>
       </c>
-      <c r="E17" t="s">
-        <v>154</v>
-      </c>
-      <c r="F17" t="s">
-        <v>134</v>
+      <c r="F17">
+        <v>8</v>
       </c>
       <c r="G17" t="s">
         <v>130</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17">
+        <v>256</v>
+      </c>
+      <c r="I17" t="s">
         <v>131</v>
       </c>
-      <c r="I17" s="19">
+      <c r="J17" s="19">
         <v>100</v>
       </c>
-      <c r="J17" s="1"/>
-      <c r="K17">
+      <c r="K17" s="1"/>
+      <c r="L17">
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1">
+    <row r="18" spans="1:12" ht="15" customHeight="1">
       <c r="A18" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B18" t="s">
         <v>132</v>
@@ -4502,31 +4755,34 @@
         <v>2019</v>
       </c>
       <c r="D18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E18" t="s">
-        <v>128</v>
-      </c>
-      <c r="F18" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F18">
+        <v>8</v>
       </c>
       <c r="G18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H18" t="s">
+        <v>136</v>
+      </c>
+      <c r="H18">
+        <v>256</v>
+      </c>
+      <c r="I18" t="s">
         <v>131</v>
       </c>
-      <c r="I18" s="19">
+      <c r="J18" s="19">
         <v>300</v>
       </c>
-      <c r="J18" s="1"/>
-      <c r="K18">
+      <c r="K18" s="1"/>
+      <c r="L18">
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15" customHeight="1">
+    <row r="19" spans="1:12" ht="15" customHeight="1">
       <c r="A19" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B19" t="s">
         <v>132</v>
@@ -4535,31 +4791,34 @@
         <v>2019</v>
       </c>
       <c r="D19" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F19">
+        <v>8</v>
+      </c>
+      <c r="G19" t="s">
+        <v>136</v>
+      </c>
+      <c r="H19">
+        <v>256</v>
+      </c>
+      <c r="I19" t="s">
+        <v>131</v>
+      </c>
+      <c r="J19" s="19">
+        <v>300</v>
+      </c>
+      <c r="K19" s="1"/>
+      <c r="L19">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="15" customHeight="1">
+      <c r="A20" t="s">
         <v>156</v>
-      </c>
-      <c r="E19" t="s">
-        <v>144</v>
-      </c>
-      <c r="F19" t="s">
-        <v>157</v>
-      </c>
-      <c r="G19" t="s">
-        <v>130</v>
-      </c>
-      <c r="H19" t="s">
-        <v>131</v>
-      </c>
-      <c r="I19" s="19">
-        <v>300</v>
-      </c>
-      <c r="J19" s="1"/>
-      <c r="K19">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15" customHeight="1">
-      <c r="A20" t="s">
-        <v>158</v>
       </c>
       <c r="B20" t="s">
         <v>132</v>
@@ -4568,31 +4827,34 @@
         <v>2021</v>
       </c>
       <c r="D20" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E20" t="s">
-        <v>144</v>
-      </c>
-      <c r="F20" t="s">
-        <v>137</v>
+        <v>143</v>
+      </c>
+      <c r="F20">
+        <v>8</v>
       </c>
       <c r="G20" t="s">
-        <v>130</v>
-      </c>
-      <c r="H20" t="s">
+        <v>136</v>
+      </c>
+      <c r="H20">
+        <v>256</v>
+      </c>
+      <c r="I20" t="s">
         <v>131</v>
       </c>
-      <c r="I20" s="19">
+      <c r="J20" s="19">
         <v>350</v>
       </c>
-      <c r="J20" s="1"/>
-      <c r="K20">
+      <c r="K20" s="1"/>
+      <c r="L20">
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15" customHeight="1">
+    <row r="21" spans="1:12" ht="15" customHeight="1">
       <c r="A21" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B21" t="s">
         <v>132</v>
@@ -4601,64 +4863,70 @@
         <v>2021</v>
       </c>
       <c r="D21" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E21" t="s">
-        <v>144</v>
-      </c>
-      <c r="F21" t="s">
-        <v>137</v>
+        <v>143</v>
+      </c>
+      <c r="F21">
+        <v>8</v>
       </c>
       <c r="G21" t="s">
-        <v>130</v>
-      </c>
-      <c r="H21" t="s">
+        <v>136</v>
+      </c>
+      <c r="H21">
+        <v>256</v>
+      </c>
+      <c r="I21" t="s">
         <v>131</v>
       </c>
-      <c r="I21" s="19">
+      <c r="J21" s="19">
         <v>350</v>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21">
+      <c r="K21" s="1"/>
+      <c r="L21">
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15" customHeight="1">
+    <row r="22" spans="1:12" ht="15" customHeight="1">
       <c r="A22" t="s">
         <v>68</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C22">
         <v>2016</v>
       </c>
       <c r="D22" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
-      </c>
-      <c r="F22" t="s">
-        <v>161</v>
+        <v>129</v>
+      </c>
+      <c r="F22">
+        <v>16</v>
       </c>
       <c r="G22" t="s">
-        <v>162</v>
-      </c>
-      <c r="H22" t="s">
+        <v>136</v>
+      </c>
+      <c r="H22">
+        <v>256</v>
+      </c>
+      <c r="I22" t="s">
         <v>131</v>
       </c>
-      <c r="I22" s="19">
+      <c r="J22" s="19">
         <v>255</v>
       </c>
-      <c r="J22" s="1"/>
-      <c r="K22">
+      <c r="K22" s="1"/>
+      <c r="L22">
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15" customHeight="1">
+    <row r="23" spans="1:12" ht="15" customHeight="1">
       <c r="A23" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B23" t="s">
         <v>132</v>
@@ -4667,97 +4935,106 @@
         <v>2019</v>
       </c>
       <c r="D23" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E23" t="s">
-        <v>144</v>
-      </c>
-      <c r="F23" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F23">
+        <v>16</v>
       </c>
       <c r="G23" t="s">
-        <v>130</v>
-      </c>
-      <c r="H23" t="s">
+        <v>136</v>
+      </c>
+      <c r="H23">
+        <v>256</v>
+      </c>
+      <c r="I23" t="s">
         <v>131</v>
       </c>
-      <c r="I23" s="19">
+      <c r="J23" s="19">
         <v>300</v>
       </c>
-      <c r="J23" s="1"/>
-      <c r="K23">
+      <c r="K23" s="1"/>
+      <c r="L23">
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1">
+    <row r="24" spans="1:12" ht="15" customHeight="1">
       <c r="A24" t="s">
         <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C24">
         <v>2015</v>
       </c>
       <c r="D24" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E24" t="s">
-        <v>144</v>
-      </c>
-      <c r="F24" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F24">
+        <v>16</v>
       </c>
       <c r="G24" t="s">
-        <v>130</v>
-      </c>
-      <c r="H24" t="s">
+        <v>136</v>
+      </c>
+      <c r="H24">
+        <v>256</v>
+      </c>
+      <c r="I24" t="s">
         <v>131</v>
       </c>
-      <c r="I24" s="19">
+      <c r="J24" s="19">
         <v>255</v>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24">
+      <c r="K24" s="1"/>
+      <c r="L24">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15" customHeight="1">
+    <row r="25" spans="1:12" ht="15" customHeight="1">
       <c r="A25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C25">
         <v>2018</v>
       </c>
       <c r="D25" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E25" t="s">
-        <v>128</v>
-      </c>
-      <c r="F25" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F25">
+        <v>8</v>
       </c>
       <c r="G25" t="s">
-        <v>130</v>
-      </c>
-      <c r="H25" t="s">
+        <v>136</v>
+      </c>
+      <c r="H25">
+        <v>256</v>
+      </c>
+      <c r="I25" t="s">
         <v>131</v>
       </c>
-      <c r="I25" s="19">
+      <c r="J25" s="19">
         <v>175</v>
       </c>
-      <c r="J25" s="1"/>
-      <c r="K25">
+      <c r="K25" s="1"/>
+      <c r="L25">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15" customHeight="1">
+    <row r="26" spans="1:12" ht="15" customHeight="1">
       <c r="A26" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B26" t="s">
         <v>132</v>
@@ -4766,29 +5043,32 @@
         <v>2017</v>
       </c>
       <c r="D26" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E26" t="s">
-        <v>128</v>
-      </c>
-      <c r="F26" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F26">
+        <v>8</v>
       </c>
       <c r="G26" t="s">
-        <v>130</v>
-      </c>
-      <c r="H26" t="s">
+        <v>136</v>
+      </c>
+      <c r="H26">
+        <v>256</v>
+      </c>
+      <c r="I26" t="s">
         <v>131</v>
       </c>
-      <c r="I26" s="19">
+      <c r="J26" s="19">
         <v>150</v>
       </c>
-      <c r="J26" s="1"/>
-      <c r="K26">
+      <c r="K26" s="1"/>
+      <c r="L26">
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15" customHeight="1">
+    <row r="27" spans="1:12" ht="15" customHeight="1">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -4799,62 +5079,68 @@
         <v>2017</v>
       </c>
       <c r="D27" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E27" t="s">
-        <v>144</v>
-      </c>
-      <c r="F27" t="s">
-        <v>137</v>
+        <v>143</v>
+      </c>
+      <c r="F27">
+        <v>8</v>
       </c>
       <c r="G27" t="s">
-        <v>130</v>
-      </c>
-      <c r="H27" t="s">
+        <v>136</v>
+      </c>
+      <c r="H27">
+        <v>256</v>
+      </c>
+      <c r="I27" t="s">
         <v>131</v>
       </c>
-      <c r="I27" s="19">
+      <c r="J27" s="19">
         <v>200</v>
       </c>
-      <c r="J27" s="1"/>
-      <c r="K27">
+      <c r="K27" s="1"/>
+      <c r="L27">
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15" customHeight="1">
+    <row r="28" spans="1:12" ht="15" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C28">
         <v>2013</v>
       </c>
       <c r="D28" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E28" t="s">
-        <v>128</v>
-      </c>
-      <c r="F28" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F28">
+        <v>8</v>
       </c>
       <c r="G28" t="s">
         <v>130</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H28">
+        <v>256</v>
+      </c>
+      <c r="I28" t="s">
         <v>131</v>
       </c>
-      <c r="I28" s="19">
+      <c r="J28" s="19">
         <v>200</v>
       </c>
-      <c r="J28" s="1"/>
-      <c r="K28">
+      <c r="K28" s="1"/>
+      <c r="L28">
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15" customHeight="1">
+    <row r="29" spans="1:12" ht="15" customHeight="1">
       <c r="A29" t="s">
         <v>55</v>
       </c>
@@ -4865,76 +5151,159 @@
         <v>2018</v>
       </c>
       <c r="D29" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E29" t="s">
-        <v>144</v>
-      </c>
-      <c r="F29" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F29">
+        <v>16</v>
       </c>
       <c r="G29" t="s">
-        <v>130</v>
-      </c>
-      <c r="H29" t="s">
+        <v>136</v>
+      </c>
+      <c r="H29">
+        <v>256</v>
+      </c>
+      <c r="I29" t="s">
         <v>131</v>
       </c>
-      <c r="I29" s="19">
+      <c r="J29" s="19">
         <v>325</v>
       </c>
-      <c r="J29" s="1"/>
-      <c r="K29">
+      <c r="K29" s="1"/>
+      <c r="L29">
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15" customHeight="1">
-      <c r="J30" s="1"/>
-    </row>
-    <row r="31" spans="1:11" ht="15" customHeight="1">
-      <c r="J31" s="1"/>
-    </row>
-    <row r="32" spans="1:11" ht="15" customHeight="1">
-      <c r="J32" s="1"/>
-    </row>
-    <row r="33" spans="10:10" ht="15" customHeight="1">
-      <c r="J33" s="1"/>
+    <row r="30" spans="1:12" ht="15" customHeight="1">
+      <c r="K30" s="1"/>
+    </row>
+    <row r="31" spans="1:12" ht="15" customHeight="1">
+      <c r="K31" s="1"/>
+    </row>
+    <row r="32" spans="1:12" ht="15" customHeight="1">
+      <c r="K32" s="1"/>
+    </row>
+    <row r="33" spans="11:11" ht="15" customHeight="1">
+      <c r="K33" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A3:J9 A11:J14 A15:C15 E15:J15 A16:J25">
-    <cfRule type="expression" dxfId="14" priority="5">
+  <conditionalFormatting sqref="A15:C15 A3:K9 A11:K14 E15:K15 A16:K25">
+    <cfRule type="expression" dxfId="43" priority="21">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:K9 A11:K14 A15:C15 E15:K15 A16:K25">
-    <cfRule type="expression" dxfId="13" priority="6">
+  <conditionalFormatting sqref="A15:C15 A3:L9 A11:L14 E15:L15 A16:L25">
+    <cfRule type="expression" dxfId="42" priority="22">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="expression" dxfId="12" priority="4">
+    <cfRule type="expression" dxfId="41" priority="20">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="40" priority="19">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28">
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="39" priority="18">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="38" priority="17">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G28">
+    <cfRule type="expression" dxfId="37" priority="15">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28">
+    <cfRule type="expression" dxfId="36" priority="16">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G26">
+    <cfRule type="expression" dxfId="35" priority="13">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G26">
+    <cfRule type="expression" dxfId="34" priority="14">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27">
+    <cfRule type="expression" dxfId="33" priority="11">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27">
+    <cfRule type="expression" dxfId="32" priority="12">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="expression" dxfId="31" priority="9">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="expression" dxfId="30" priority="10">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="expression" dxfId="29" priority="7">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="expression" dxfId="28" priority="8">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="expression" dxfId="27" priority="5">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H27">
+    <cfRule type="expression" dxfId="26" priority="6">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H28">
+    <cfRule type="expression" dxfId="25" priority="3">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H28">
+    <cfRule type="expression" dxfId="24" priority="4">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29">
+    <cfRule type="expression" dxfId="23" priority="1">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29">
+    <cfRule type="expression" dxfId="22" priority="2">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K12:K25 K3:K4" xr:uid="{BD4480FF-AB8D-4446-AB7A-01C4C2A99ADB}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L12:L25 L3:L4" xr:uid="{BD4480FF-AB8D-4446-AB7A-01C4C2A99ADB}">
       <formula1>1</formula1>
       <formula2>2000</formula2>
     </dataValidation>
@@ -4951,7 +5320,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19592962-4FD3-47C5-914B-6346C180BC2C}">
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
@@ -4960,19 +5329,20 @@
     <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.28515625" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.28515625" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" style="16" customWidth="1"/>
-    <col min="12" max="12" width="29.140625" customWidth="1"/>
-    <col min="13" max="13" width="27.7109375" customWidth="1"/>
-    <col min="14" max="14" width="28.28515625" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="16" customWidth="1"/>
+    <col min="13" max="13" width="29.140625" customWidth="1"/>
+    <col min="14" max="14" width="27.7109375" customWidth="1"/>
+    <col min="15" max="15" width="28.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15" customHeight="1">
+    <row r="1" spans="1:15" ht="15" customHeight="1">
       <c r="B1" s="17" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -4980,18 +5350,19 @@
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="18"/>
-      <c r="M1" t="s">
-        <v>170</v>
-      </c>
+      <c r="I1" s="18"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="18"/>
       <c r="N1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
+        <v>166</v>
+      </c>
+      <c r="O1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>115</v>
       </c>
@@ -5016,135 +5387,138 @@
       <c r="H2" t="s">
         <v>122</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" t="s">
         <v>123</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L2" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="M2" t="s">
+        <v>169</v>
+      </c>
+      <c r="N2" s="2">
+        <f>SUM(J3:J38)</f>
+        <v>9870</v>
+      </c>
+      <c r="O2">
+        <f>COUNTIF(M3:M42,"*International*")</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
+        <v>170</v>
+      </c>
+      <c r="J3" s="19">
+        <v>225</v>
+      </c>
+      <c r="K3" s="2"/>
+      <c r="L3" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" t="s">
+        <v>170</v>
+      </c>
+      <c r="J4" s="19">
+        <v>225</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" t="s">
+        <v>170</v>
+      </c>
+      <c r="J5" s="19">
+        <v>225</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M5" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
+        <v>170</v>
+      </c>
+      <c r="J6" s="19">
+        <v>225</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M6" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" t="s">
+        <v>170</v>
+      </c>
+      <c r="J7" s="19">
+        <v>225</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" t="s">
+        <v>170</v>
+      </c>
+      <c r="J8" s="19">
+        <v>225</v>
+      </c>
+      <c r="K8" s="2"/>
+      <c r="L8" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="s">
+        <v>170</v>
+      </c>
+      <c r="J9" s="19">
+        <v>225</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="15">
+        <v>45970</v>
+      </c>
+      <c r="M9" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" t="s">
         <v>172</v>
-      </c>
-      <c r="L2" t="s">
-        <v>173</v>
-      </c>
-      <c r="M2" s="2">
-        <f>SUM(I3:I38)</f>
-        <v>9870</v>
-      </c>
-      <c r="N2">
-        <f>COUNTIF(L3:L42,"*International*")</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" t="s">
-        <v>174</v>
-      </c>
-      <c r="I3" s="19">
-        <v>225</v>
-      </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" t="s">
-        <v>174</v>
-      </c>
-      <c r="I4" s="19">
-        <v>225</v>
-      </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L4" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5" t="s">
-        <v>174</v>
-      </c>
-      <c r="I5" s="19">
-        <v>225</v>
-      </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L5" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6" t="s">
-        <v>174</v>
-      </c>
-      <c r="I6" s="19">
-        <v>225</v>
-      </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L6" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" t="s">
-        <v>174</v>
-      </c>
-      <c r="I7" s="19">
-        <v>225</v>
-      </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L7" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" t="s">
-        <v>174</v>
-      </c>
-      <c r="I8" s="19">
-        <v>225</v>
-      </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L8" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" t="s">
-        <v>174</v>
-      </c>
-      <c r="I9" s="19">
-        <v>225</v>
-      </c>
-      <c r="J9" s="2"/>
-      <c r="K9" s="15">
-        <v>45970</v>
-      </c>
-      <c r="L9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" t="s">
-        <v>176</v>
       </c>
       <c r="B10" t="s">
         <v>132</v>
@@ -5153,34 +5527,37 @@
         <v>2018</v>
       </c>
       <c r="D10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E10" t="s">
-        <v>144</v>
-      </c>
-      <c r="F10" t="s">
-        <v>178</v>
+        <v>143</v>
+      </c>
+      <c r="F10">
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>130</v>
-      </c>
-      <c r="H10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H10">
+        <v>256</v>
+      </c>
+      <c r="I10" t="s">
         <v>131</v>
       </c>
-      <c r="I10" s="21">
+      <c r="J10" s="21">
         <v>325</v>
       </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="15">
+      <c r="K10" s="3"/>
+      <c r="L10" s="15">
         <v>45999</v>
       </c>
-      <c r="L10" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+      <c r="M10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B11" t="s">
         <v>132</v>
@@ -5189,34 +5566,37 @@
         <v>2015</v>
       </c>
       <c r="D11" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E11" t="s">
-        <v>144</v>
-      </c>
-      <c r="F11" t="s">
-        <v>181</v>
+        <v>143</v>
+      </c>
+      <c r="F11">
+        <v>8</v>
       </c>
       <c r="G11" t="s">
         <v>130</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11">
+        <v>256</v>
+      </c>
+      <c r="I11" t="s">
         <v>131</v>
       </c>
-      <c r="I11" s="19">
+      <c r="J11" s="19">
         <v>225</v>
       </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="15">
+      <c r="K11" s="2"/>
+      <c r="L11" s="15">
         <v>45999</v>
       </c>
-      <c r="L11" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+      <c r="M11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B12" t="s">
         <v>132</v>
@@ -5225,36 +5605,39 @@
         <v>2014</v>
       </c>
       <c r="D12" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E12" t="s">
-        <v>128</v>
-      </c>
-      <c r="F12" t="s">
-        <v>181</v>
+        <v>129</v>
+      </c>
+      <c r="F12">
+        <v>8</v>
       </c>
       <c r="G12" t="s">
         <v>130</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12">
+        <v>256</v>
+      </c>
+      <c r="I12" t="s">
         <v>131</v>
       </c>
-      <c r="I12" s="19">
+      <c r="J12" s="19">
         <v>175</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="K12" s="15">
+      <c r="K12" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="L12" s="15">
         <v>45999</v>
       </c>
-      <c r="L12" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+      <c r="M12" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B13" t="s">
         <v>132</v>
@@ -5263,34 +5646,37 @@
         <v>2019</v>
       </c>
       <c r="D13" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F13" t="s">
-        <v>178</v>
+        <v>143</v>
+      </c>
+      <c r="F13">
+        <v>16</v>
       </c>
       <c r="G13" t="s">
-        <v>130</v>
-      </c>
-      <c r="H13" t="s">
+        <v>136</v>
+      </c>
+      <c r="H13">
+        <v>256</v>
+      </c>
+      <c r="I13" t="s">
         <v>131</v>
       </c>
-      <c r="I13" s="19">
+      <c r="J13" s="19">
         <v>325</v>
       </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="15">
+      <c r="K13" s="2"/>
+      <c r="L13" s="15">
         <v>45999</v>
       </c>
-      <c r="L13" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+      <c r="M13" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B14" t="s">
         <v>132</v>
@@ -5299,34 +5685,37 @@
         <v>2018</v>
       </c>
       <c r="D14" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E14" t="s">
-        <v>144</v>
-      </c>
-      <c r="F14" t="s">
-        <v>187</v>
+        <v>143</v>
+      </c>
+      <c r="F14">
+        <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>130</v>
-      </c>
-      <c r="H14" t="s">
+        <v>136</v>
+      </c>
+      <c r="H14">
+        <v>256</v>
+      </c>
+      <c r="I14" t="s">
         <v>131</v>
       </c>
-      <c r="I14" s="19">
+      <c r="J14" s="19">
         <v>325</v>
       </c>
-      <c r="J14" s="2"/>
-      <c r="K14" s="15">
+      <c r="K14" s="2"/>
+      <c r="L14" s="15">
         <v>45999</v>
       </c>
-      <c r="L14" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+      <c r="M14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B15" t="s">
         <v>132</v>
@@ -5335,476 +5724,515 @@
         <v>2021</v>
       </c>
       <c r="D15" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="E15" t="s">
-        <v>144</v>
-      </c>
-      <c r="F15" t="s">
-        <v>190</v>
+        <v>143</v>
+      </c>
+      <c r="F15">
+        <v>16</v>
       </c>
       <c r="G15" t="s">
-        <v>130</v>
-      </c>
-      <c r="H15" t="s">
+        <v>136</v>
+      </c>
+      <c r="H15">
+        <v>256</v>
+      </c>
+      <c r="I15" t="s">
         <v>131</v>
       </c>
-      <c r="I15" s="19">
+      <c r="J15" s="19">
         <v>205</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15" s="15">
+      <c r="K15" s="2"/>
+      <c r="L15" s="15">
         <v>45999</v>
       </c>
-      <c r="L15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+      <c r="M15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="C16">
         <v>2012</v>
       </c>
       <c r="D16" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="E16" t="s">
-        <v>194</v>
-      </c>
-      <c r="F16" t="s">
-        <v>193</v>
+        <v>186</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H16" t="s">
-        <v>196</v>
-      </c>
-      <c r="I16" s="19">
+        <v>187</v>
+      </c>
+      <c r="H16" s="1">
+        <v>64</v>
+      </c>
+      <c r="I16" t="s">
+        <v>188</v>
+      </c>
+      <c r="J16" s="19">
         <v>50</v>
       </c>
-      <c r="J16" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K16" s="15">
+      <c r="K16" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="L16" s="15">
         <v>45999</v>
       </c>
-      <c r="L16" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+      <c r="M16" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B17" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="C17">
         <v>2014</v>
       </c>
       <c r="D17" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="E17" t="s">
-        <v>199</v>
-      </c>
-      <c r="F17" t="s">
-        <v>193</v>
+        <v>186</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>200</v>
-      </c>
-      <c r="H17" t="s">
-        <v>196</v>
-      </c>
-      <c r="I17" s="19">
+        <v>130</v>
+      </c>
+      <c r="H17">
+        <v>128</v>
+      </c>
+      <c r="I17" t="s">
+        <v>188</v>
+      </c>
+      <c r="J17" s="19">
         <v>60</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K17" s="15">
+      <c r="K17" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="L17" s="15">
         <v>45999</v>
       </c>
-      <c r="L17" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
+      <c r="M17" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="B18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C18">
         <v>2018</v>
       </c>
       <c r="D18" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="E18" t="s">
-        <v>144</v>
-      </c>
-      <c r="F18" t="s">
-        <v>137</v>
+        <v>143</v>
+      </c>
+      <c r="F18">
+        <v>8</v>
       </c>
       <c r="G18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H18" t="s">
+        <v>136</v>
+      </c>
+      <c r="H18">
+        <v>256</v>
+      </c>
+      <c r="I18" t="s">
         <v>131</v>
       </c>
-      <c r="I18" s="19">
+      <c r="J18" s="19">
         <v>250</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="K18" s="16">
+      <c r="K18" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="L18" s="16">
         <v>46043</v>
       </c>
-      <c r="L18" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
+      <c r="M18" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
         <v>71</v>
       </c>
       <c r="B19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C19">
         <v>2013</v>
       </c>
       <c r="D19" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="E19" t="s">
-        <v>128</v>
-      </c>
-      <c r="F19" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F19">
+        <v>8</v>
       </c>
       <c r="G19" t="s">
         <v>130</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19">
+        <v>256</v>
+      </c>
+      <c r="I19" t="s">
         <v>131</v>
       </c>
-      <c r="I19" s="19">
+      <c r="J19" s="19">
         <v>290</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="K19" s="16">
+      <c r="K19" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="L19" s="16">
         <v>46043</v>
       </c>
-      <c r="L19" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="45">
+      <c r="M19" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="43.5">
       <c r="A20" t="s">
         <v>68</v>
       </c>
       <c r="B20" t="s">
-        <v>207</v>
+        <v>127</v>
       </c>
       <c r="C20">
         <v>2016</v>
       </c>
       <c r="D20" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E20" t="s">
-        <v>128</v>
-      </c>
-      <c r="F20" t="s">
-        <v>161</v>
+        <v>129</v>
+      </c>
+      <c r="F20">
+        <v>16</v>
       </c>
       <c r="G20" t="s">
-        <v>130</v>
-      </c>
-      <c r="H20" t="s">
+        <v>136</v>
+      </c>
+      <c r="H20">
+        <v>256</v>
+      </c>
+      <c r="I20" t="s">
         <v>131</v>
       </c>
-      <c r="I20" s="19">
+      <c r="J20" s="19">
         <v>300</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="K20" s="15">
+      <c r="K20" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="L20" s="15">
         <v>46056</v>
       </c>
-      <c r="L20" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
+      <c r="M20" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="B21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C21">
         <v>2013</v>
       </c>
       <c r="D21" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="E21" t="s">
-        <v>128</v>
-      </c>
-      <c r="F21" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F21">
+        <v>8</v>
       </c>
       <c r="G21" t="s">
         <v>130</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21">
+        <v>256</v>
+      </c>
+      <c r="I21" t="s">
         <v>131</v>
       </c>
-      <c r="I21" s="19">
+      <c r="J21" s="19">
         <v>200</v>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="15">
+      <c r="K21" s="1"/>
+      <c r="L21" s="15">
         <v>46056</v>
       </c>
-      <c r="L21" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
+      <c r="M21" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
         <v>71</v>
       </c>
       <c r="B22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C22">
         <v>2013</v>
       </c>
       <c r="D22" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
-      </c>
-      <c r="F22" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F22">
+        <v>8</v>
       </c>
       <c r="G22" t="s">
         <v>130</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22">
+        <v>256</v>
+      </c>
+      <c r="I22" t="s">
         <v>131</v>
       </c>
-      <c r="I22" s="19">
+      <c r="J22" s="19">
         <v>200</v>
       </c>
-      <c r="J22" s="1"/>
-      <c r="K22" s="15">
+      <c r="K22" s="1"/>
+      <c r="L22" s="15">
         <v>46056</v>
       </c>
-      <c r="L22" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12">
+      <c r="M22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
         <v>71</v>
       </c>
       <c r="B23" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23">
         <v>2013</v>
       </c>
       <c r="D23" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="E23" t="s">
-        <v>128</v>
-      </c>
-      <c r="F23" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F23">
+        <v>8</v>
       </c>
       <c r="G23" t="s">
         <v>130</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23">
+        <v>256</v>
+      </c>
+      <c r="I23" t="s">
         <v>131</v>
       </c>
-      <c r="I23" s="19">
+      <c r="J23" s="19">
         <v>200</v>
       </c>
-      <c r="J23" s="1"/>
-      <c r="K23" s="15">
+      <c r="K23" s="1"/>
+      <c r="L23" s="15">
         <v>46056</v>
       </c>
-      <c r="L23" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
+      <c r="M23" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
         <v>71</v>
       </c>
       <c r="B24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C24">
         <v>2013</v>
       </c>
       <c r="D24" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="E24" t="s">
-        <v>128</v>
-      </c>
-      <c r="F24" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F24">
+        <v>8</v>
       </c>
       <c r="G24" t="s">
         <v>130</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24">
+        <v>256</v>
+      </c>
+      <c r="I24" t="s">
         <v>131</v>
       </c>
-      <c r="I24" s="19">
+      <c r="J24" s="19">
         <v>200</v>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24" s="15">
+      <c r="K24" s="1"/>
+      <c r="L24" s="15">
         <v>46056</v>
       </c>
-      <c r="L24" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
+      <c r="M24" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
         <v>71</v>
       </c>
       <c r="B25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C25">
         <v>2013</v>
       </c>
       <c r="D25" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="E25" t="s">
-        <v>128</v>
-      </c>
-      <c r="F25" t="s">
-        <v>214</v>
+        <v>129</v>
+      </c>
+      <c r="F25">
+        <v>16</v>
       </c>
       <c r="G25" t="s">
         <v>130</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25">
+        <v>256</v>
+      </c>
+      <c r="I25" t="s">
         <v>131</v>
       </c>
-      <c r="I25" s="19">
+      <c r="J25" s="19">
         <v>200</v>
       </c>
-      <c r="J25" s="1"/>
-      <c r="K25" s="15">
+      <c r="K25" s="1"/>
+      <c r="L25" s="15">
         <v>46056</v>
       </c>
-      <c r="L25" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
+      <c r="M25" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
         <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C26">
         <v>2016</v>
       </c>
       <c r="D26" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E26" t="s">
-        <v>128</v>
-      </c>
-      <c r="F26" t="s">
-        <v>161</v>
+        <v>129</v>
+      </c>
+      <c r="F26">
+        <v>16</v>
       </c>
       <c r="G26" t="s">
-        <v>130</v>
-      </c>
-      <c r="H26" t="s">
+        <v>136</v>
+      </c>
+      <c r="H26">
+        <v>256</v>
+      </c>
+      <c r="I26" t="s">
         <v>131</v>
       </c>
-      <c r="I26" s="19">
+      <c r="J26" s="19">
         <v>300</v>
       </c>
-      <c r="J26" s="1"/>
-      <c r="K26" s="15">
+      <c r="K26" s="1"/>
+      <c r="L26" s="15">
         <v>46056</v>
       </c>
-      <c r="L26" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
+      <c r="M26" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
         <v>68</v>
       </c>
       <c r="B27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C27">
         <v>2016</v>
       </c>
       <c r="D27" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E27" t="s">
-        <v>128</v>
-      </c>
-      <c r="F27" t="s">
-        <v>134</v>
+        <v>129</v>
+      </c>
+      <c r="F27">
+        <v>8</v>
       </c>
       <c r="G27" t="s">
         <v>130</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27">
+        <v>256</v>
+      </c>
+      <c r="I27" t="s">
         <v>131</v>
       </c>
-      <c r="I27" s="19">
+      <c r="J27" s="19">
         <v>300</v>
       </c>
-      <c r="J27" s="1"/>
-      <c r="K27" s="15">
+      <c r="K27" s="1"/>
+      <c r="L27" s="15">
         <v>46056</v>
       </c>
-      <c r="L27" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12">
+      <c r="M27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="B28" t="s">
         <v>132</v>
@@ -5813,34 +6241,37 @@
         <v>2018</v>
       </c>
       <c r="D28" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E28" t="s">
-        <v>144</v>
-      </c>
-      <c r="F28" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F28">
+        <v>16</v>
       </c>
       <c r="G28" t="s">
-        <v>217</v>
-      </c>
-      <c r="H28" t="s">
+        <v>136</v>
+      </c>
+      <c r="H28">
+        <v>512</v>
+      </c>
+      <c r="I28" t="s">
         <v>131</v>
       </c>
-      <c r="I28" s="19">
+      <c r="J28" s="19">
         <v>445</v>
       </c>
-      <c r="J28" s="1"/>
-      <c r="K28" s="15">
+      <c r="K28" s="1"/>
+      <c r="L28" s="15">
         <v>46056</v>
       </c>
-      <c r="L28" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+      <c r="M28" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="B29" t="s">
         <v>132</v>
@@ -5849,176 +6280,191 @@
         <v>2018</v>
       </c>
       <c r="D29" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E29" t="s">
-        <v>144</v>
-      </c>
-      <c r="F29" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F29">
+        <v>16</v>
       </c>
       <c r="G29" t="s">
-        <v>217</v>
-      </c>
-      <c r="H29" t="s">
+        <v>136</v>
+      </c>
+      <c r="H29">
+        <v>512</v>
+      </c>
+      <c r="I29" t="s">
         <v>131</v>
       </c>
-      <c r="I29" s="19">
+      <c r="J29" s="19">
         <v>445</v>
       </c>
-      <c r="J29" s="1"/>
-      <c r="K29" s="15">
+      <c r="K29" s="1"/>
+      <c r="L29" s="15">
         <v>46056</v>
       </c>
-      <c r="L29" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12">
+      <c r="M29" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B30" t="s">
-        <v>218</v>
+        <v>127</v>
       </c>
       <c r="C30">
         <v>2018</v>
       </c>
       <c r="D30" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="E30" t="s">
-        <v>128</v>
-      </c>
-      <c r="F30" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F30">
+        <v>8</v>
       </c>
       <c r="G30" t="s">
-        <v>130</v>
-      </c>
-      <c r="H30" t="s">
+        <v>136</v>
+      </c>
+      <c r="H30">
+        <v>256</v>
+      </c>
+      <c r="I30" t="s">
         <v>131</v>
       </c>
-      <c r="I30" s="19">
+      <c r="J30" s="19">
         <v>150</v>
       </c>
-      <c r="J30" s="1"/>
-      <c r="K30" s="15">
+      <c r="K30" s="1"/>
+      <c r="L30" s="15">
         <v>46056</v>
       </c>
-      <c r="L30" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12">
+      <c r="M30" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" s="8" t="s">
         <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C31">
         <v>2016</v>
       </c>
       <c r="D31" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E31" t="s">
-        <v>128</v>
-      </c>
-      <c r="F31" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F31">
+        <v>8</v>
       </c>
       <c r="G31" t="s">
-        <v>162</v>
-      </c>
-      <c r="H31" t="s">
-        <v>220</v>
-      </c>
-      <c r="I31" s="19">
+        <v>136</v>
+      </c>
+      <c r="H31">
+        <v>500</v>
+      </c>
+      <c r="I31" t="s">
+        <v>206</v>
+      </c>
+      <c r="J31" s="19">
         <v>300</v>
       </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="16">
+      <c r="K31" s="1"/>
+      <c r="L31" s="16">
         <v>46058</v>
       </c>
-      <c r="L31" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12">
+      <c r="M31" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" t="s">
         <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C32">
         <v>2016</v>
       </c>
       <c r="D32" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E32" t="s">
-        <v>128</v>
-      </c>
-      <c r="F32" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F32">
+        <v>8</v>
       </c>
       <c r="G32" t="s">
-        <v>130</v>
-      </c>
-      <c r="H32" t="s">
+        <v>136</v>
+      </c>
+      <c r="H32">
+        <v>256</v>
+      </c>
+      <c r="I32" t="s">
         <v>131</v>
       </c>
-      <c r="I32" s="19">
+      <c r="J32" s="19">
         <v>300</v>
       </c>
-      <c r="K32" s="16">
+      <c r="L32" s="16">
         <v>46058</v>
       </c>
-      <c r="L32" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12">
+      <c r="M32" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
       <c r="A33" t="s">
         <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C33">
         <v>2016</v>
       </c>
       <c r="D33" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E33" t="s">
-        <v>128</v>
-      </c>
-      <c r="F33" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F33">
+        <v>8</v>
       </c>
       <c r="G33" t="s">
-        <v>130</v>
-      </c>
-      <c r="H33" t="s">
+        <v>136</v>
+      </c>
+      <c r="H33">
+        <v>256</v>
+      </c>
+      <c r="I33" t="s">
         <v>131</v>
       </c>
-      <c r="I33" s="19">
+      <c r="J33" s="19">
         <v>300</v>
       </c>
-      <c r="K33" s="16">
+      <c r="L33" s="16">
         <v>46058</v>
       </c>
-      <c r="L33" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12">
+      <c r="M33" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
       <c r="A34" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B34" t="s">
         <v>132</v>
@@ -6027,33 +6473,36 @@
         <v>2020</v>
       </c>
       <c r="D34" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E34" t="s">
-        <v>144</v>
-      </c>
-      <c r="F34" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F34">
+        <v>16</v>
       </c>
       <c r="G34" t="s">
-        <v>217</v>
-      </c>
-      <c r="H34" t="s">
+        <v>136</v>
+      </c>
+      <c r="H34">
+        <v>512</v>
+      </c>
+      <c r="I34" t="s">
         <v>131</v>
       </c>
-      <c r="I34" s="19">
+      <c r="J34" s="19">
         <v>445</v>
       </c>
-      <c r="K34" s="16">
+      <c r="L34" s="16">
         <v>46058</v>
       </c>
-      <c r="L34" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
+      <c r="M34" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
       <c r="A35" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B35" t="s">
         <v>132</v>
@@ -6062,33 +6511,36 @@
         <v>2020</v>
       </c>
       <c r="D35" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E35" t="s">
-        <v>144</v>
-      </c>
-      <c r="F35" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F35">
+        <v>16</v>
       </c>
       <c r="G35" t="s">
-        <v>217</v>
-      </c>
-      <c r="H35" t="s">
+        <v>136</v>
+      </c>
+      <c r="H35">
+        <v>512</v>
+      </c>
+      <c r="I35" t="s">
         <v>131</v>
       </c>
-      <c r="I35" s="19">
+      <c r="J35" s="19">
         <v>445</v>
       </c>
-      <c r="K35" s="16">
+      <c r="L35" s="16">
         <v>46058</v>
       </c>
-      <c r="L35" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
+      <c r="M35" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
       <c r="A36" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B36" t="s">
         <v>132</v>
@@ -6097,33 +6549,36 @@
         <v>2020</v>
       </c>
       <c r="D36" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E36" t="s">
-        <v>144</v>
-      </c>
-      <c r="F36" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F36">
+        <v>16</v>
       </c>
       <c r="G36" t="s">
-        <v>217</v>
-      </c>
-      <c r="H36" t="s">
+        <v>136</v>
+      </c>
+      <c r="H36">
+        <v>512</v>
+      </c>
+      <c r="I36" t="s">
         <v>131</v>
       </c>
-      <c r="I36" s="19">
+      <c r="J36" s="19">
         <v>445</v>
       </c>
-      <c r="K36" s="16">
+      <c r="L36" s="16">
         <v>46058</v>
       </c>
-      <c r="L36" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
+      <c r="M36" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
       <c r="A37" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B37" t="s">
         <v>132</v>
@@ -6132,33 +6587,36 @@
         <v>2020</v>
       </c>
       <c r="D37" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E37" t="s">
-        <v>144</v>
-      </c>
-      <c r="F37" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F37">
+        <v>16</v>
       </c>
       <c r="G37" t="s">
-        <v>217</v>
-      </c>
-      <c r="H37" t="s">
+        <v>136</v>
+      </c>
+      <c r="H37">
+        <v>512</v>
+      </c>
+      <c r="I37" t="s">
         <v>131</v>
       </c>
-      <c r="I37" s="19">
+      <c r="J37" s="19">
         <v>445</v>
       </c>
-      <c r="K37" s="16">
+      <c r="L37" s="16">
         <v>46058</v>
       </c>
-      <c r="L37" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12">
+      <c r="M37" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
       <c r="A38" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B38" t="s">
         <v>132</v>
@@ -6167,33 +6625,36 @@
         <v>2020</v>
       </c>
       <c r="D38" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E38" t="s">
-        <v>144</v>
-      </c>
-      <c r="F38" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F38">
+        <v>16</v>
       </c>
       <c r="G38" t="s">
-        <v>217</v>
-      </c>
-      <c r="H38" t="s">
+        <v>136</v>
+      </c>
+      <c r="H38">
+        <v>512</v>
+      </c>
+      <c r="I38" t="s">
         <v>131</v>
       </c>
-      <c r="I38" s="19">
+      <c r="J38" s="19">
         <v>445</v>
       </c>
-      <c r="K38" s="16">
+      <c r="L38" s="16">
         <v>46058</v>
       </c>
-      <c r="L38" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12">
+      <c r="M38" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
       <c r="A39" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B39" t="s">
         <v>132</v>
@@ -6202,33 +6663,36 @@
         <v>2020</v>
       </c>
       <c r="D39" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E39" t="s">
-        <v>144</v>
-      </c>
-      <c r="F39" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F39">
+        <v>16</v>
       </c>
       <c r="G39" t="s">
-        <v>217</v>
-      </c>
-      <c r="H39" t="s">
+        <v>136</v>
+      </c>
+      <c r="H39">
+        <v>512</v>
+      </c>
+      <c r="I39" t="s">
         <v>131</v>
       </c>
-      <c r="I39" s="19">
+      <c r="J39" s="19">
         <v>445</v>
       </c>
-      <c r="K39" s="16">
+      <c r="L39" s="16">
         <v>46058</v>
       </c>
-      <c r="L39" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="15" customHeight="1">
+      <c r="M39" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="15" customHeight="1">
       <c r="A40" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B40" t="s">
         <v>132</v>
@@ -6237,33 +6701,36 @@
         <v>2020</v>
       </c>
       <c r="D40" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E40" t="s">
-        <v>144</v>
-      </c>
-      <c r="F40" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F40">
+        <v>16</v>
       </c>
       <c r="G40" t="s">
-        <v>217</v>
-      </c>
-      <c r="H40" t="s">
+        <v>136</v>
+      </c>
+      <c r="H40">
+        <v>512</v>
+      </c>
+      <c r="I40" t="s">
         <v>131</v>
       </c>
-      <c r="I40" s="19">
+      <c r="J40" s="19">
         <v>445</v>
       </c>
-      <c r="K40" s="16">
+      <c r="L40" s="16">
         <v>46058</v>
       </c>
-      <c r="L40" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" ht="15" customHeight="1">
+      <c r="M40" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="15" customHeight="1">
       <c r="A41" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B41" t="s">
         <v>132</v>
@@ -6272,33 +6739,36 @@
         <v>2020</v>
       </c>
       <c r="D41" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E41" t="s">
-        <v>144</v>
-      </c>
-      <c r="F41" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F41">
+        <v>16</v>
       </c>
       <c r="G41" t="s">
-        <v>217</v>
-      </c>
-      <c r="H41" t="s">
+        <v>136</v>
+      </c>
+      <c r="H41">
+        <v>512</v>
+      </c>
+      <c r="I41" t="s">
         <v>131</v>
       </c>
-      <c r="I41" s="19">
+      <c r="J41" s="19">
         <v>445</v>
       </c>
-      <c r="K41" s="16">
+      <c r="L41" s="16">
         <v>46058</v>
       </c>
-      <c r="L41" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="15" customHeight="1">
+      <c r="M41" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="15" customHeight="1">
       <c r="A42" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B42" t="s">
         <v>132</v>
@@ -6307,33 +6777,36 @@
         <v>2020</v>
       </c>
       <c r="D42" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="E42" t="s">
-        <v>144</v>
-      </c>
-      <c r="F42" t="s">
-        <v>161</v>
+        <v>143</v>
+      </c>
+      <c r="F42">
+        <v>16</v>
       </c>
       <c r="G42" t="s">
-        <v>217</v>
-      </c>
-      <c r="H42" t="s">
+        <v>136</v>
+      </c>
+      <c r="H42">
+        <v>512</v>
+      </c>
+      <c r="I42" t="s">
         <v>131</v>
       </c>
-      <c r="I42" s="19">
+      <c r="J42" s="19">
         <v>445</v>
       </c>
-      <c r="K42" s="16">
+      <c r="L42" s="16">
         <v>46058</v>
       </c>
-      <c r="L42" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="15" customHeight="1">
+      <c r="M42" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="15" customHeight="1">
       <c r="A43" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B43" t="s">
         <v>132</v>
@@ -6342,128 +6815,202 @@
         <v>2018</v>
       </c>
       <c r="D43" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="E43" t="s">
-        <v>144</v>
-      </c>
-      <c r="F43" t="s">
-        <v>137</v>
+        <v>143</v>
+      </c>
+      <c r="F43">
+        <v>8</v>
       </c>
       <c r="G43" t="s">
-        <v>130</v>
-      </c>
-      <c r="H43" t="s">
+        <v>136</v>
+      </c>
+      <c r="H43">
+        <v>256</v>
+      </c>
+      <c r="I43" t="s">
         <v>131</v>
       </c>
-      <c r="I43" s="19">
+      <c r="J43" s="19">
         <v>300</v>
       </c>
-      <c r="J43" s="1"/>
-      <c r="K43" s="16">
+      <c r="K43" s="1"/>
+      <c r="L43" s="16">
         <v>46078</v>
       </c>
-      <c r="L43" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="15" customHeight="1">
+      <c r="M43" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" ht="15" customHeight="1">
       <c r="A44" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B44" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C44" s="5">
         <v>2016</v>
       </c>
       <c r="D44" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E44" t="s">
-        <v>128</v>
-      </c>
-      <c r="F44" t="s">
-        <v>137</v>
+        <v>129</v>
+      </c>
+      <c r="F44">
+        <v>8</v>
       </c>
       <c r="G44" t="s">
-        <v>130</v>
-      </c>
-      <c r="H44" t="s">
+        <v>136</v>
+      </c>
+      <c r="H44">
+        <v>256</v>
+      </c>
+      <c r="I44" t="s">
         <v>131</v>
       </c>
-      <c r="I44" s="19">
+      <c r="J44" s="19">
         <v>300</v>
       </c>
-      <c r="J44" s="1"/>
-      <c r="K44" s="16">
+      <c r="K44" s="1"/>
+      <c r="L44" s="16">
         <v>46099</v>
       </c>
-      <c r="L44" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="15" customHeight="1">
-      <c r="K45" s="15"/>
-    </row>
-    <row r="46" spans="1:12" ht="15" customHeight="1">
-      <c r="K46" s="15"/>
-    </row>
-    <row r="47" spans="1:12" ht="15" customHeight="1">
-      <c r="K47" s="15"/>
-    </row>
-    <row r="48" spans="1:12" ht="15" customHeight="1">
-      <c r="K48" s="15"/>
-    </row>
-    <row r="49" spans="11:11" ht="15" customHeight="1">
-      <c r="K49" s="15"/>
-    </row>
-    <row r="50" spans="11:11" ht="15" customHeight="1">
-      <c r="K50" s="15"/>
-    </row>
-    <row r="51" spans="11:11" ht="15" customHeight="1">
-      <c r="K51" s="15"/>
-    </row>
-    <row r="52" spans="11:11" ht="15" customHeight="1">
-      <c r="K52" s="15"/>
-    </row>
-    <row r="53" spans="11:11" ht="15" customHeight="1">
-      <c r="K53" s="15"/>
-    </row>
-    <row r="54" spans="11:11" ht="15" customHeight="1">
-      <c r="K54" s="15"/>
-    </row>
-    <row r="55" spans="11:11" ht="15" customHeight="1">
-      <c r="K55" s="15"/>
-    </row>
-    <row r="56" spans="11:11" ht="15" customHeight="1">
-      <c r="K56" s="15"/>
-    </row>
-    <row r="57" spans="11:11" ht="15" customHeight="1">
-      <c r="K57" s="15"/>
-    </row>
-    <row r="58" spans="11:11" ht="15" customHeight="1">
-      <c r="K58" s="15"/>
-    </row>
-    <row r="59" spans="11:11" ht="15" customHeight="1">
-      <c r="K59" s="15"/>
+      <c r="M44" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="15" customHeight="1">
+      <c r="L45" s="15"/>
+    </row>
+    <row r="46" spans="1:13" ht="15" customHeight="1">
+      <c r="L46" s="15"/>
+    </row>
+    <row r="47" spans="1:13" ht="15" customHeight="1">
+      <c r="L47" s="15"/>
+    </row>
+    <row r="48" spans="1:13" ht="15" customHeight="1">
+      <c r="L48" s="15"/>
+    </row>
+    <row r="49" spans="12:12" ht="15" customHeight="1">
+      <c r="L49" s="15"/>
+    </row>
+    <row r="50" spans="12:12" ht="15" customHeight="1">
+      <c r="L50" s="15"/>
+    </row>
+    <row r="51" spans="12:12" ht="15" customHeight="1">
+      <c r="L51" s="15"/>
+    </row>
+    <row r="52" spans="12:12" ht="15" customHeight="1">
+      <c r="L52" s="15"/>
+    </row>
+    <row r="53" spans="12:12" ht="15" customHeight="1">
+      <c r="L53" s="15"/>
+    </row>
+    <row r="54" spans="12:12" ht="15" customHeight="1">
+      <c r="L54" s="15"/>
+    </row>
+    <row r="55" spans="12:12" ht="15" customHeight="1">
+      <c r="L55" s="15"/>
+    </row>
+    <row r="56" spans="12:12" ht="15" customHeight="1">
+      <c r="L56" s="15"/>
+    </row>
+    <row r="57" spans="12:12" ht="15" customHeight="1">
+      <c r="L57" s="15"/>
+    </row>
+    <row r="58" spans="12:12" ht="15" customHeight="1">
+      <c r="L58" s="15"/>
+    </row>
+    <row r="59" spans="12:12" ht="15" customHeight="1">
+      <c r="L59" s="15"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A44:J44">
-    <cfRule type="expression" dxfId="5" priority="1">
+  <conditionalFormatting sqref="A44:F44 H44:K44">
+    <cfRule type="expression" dxfId="18" priority="15">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A44:K44">
-    <cfRule type="expression" dxfId="4" priority="2">
+  <conditionalFormatting sqref="A44:F44 H44:L44">
+    <cfRule type="expression" dxfId="17" priority="16">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:L43 L44 A45:L59">
-    <cfRule type="expression" priority="3">
+  <conditionalFormatting sqref="M44 A45:M59 A3:M9 A10:G15 I10:M15 A16:M43">
+    <cfRule type="expression" priority="17">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="16" priority="18">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44">
+    <cfRule type="expression" priority="13">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="14">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="expression" dxfId="13" priority="12">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" dxfId="12" priority="9">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" dxfId="11" priority="10">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="expression" dxfId="10" priority="7">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="expression" dxfId="9" priority="8">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" dxfId="8" priority="5">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" dxfId="7" priority="6">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14">
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14">
+    <cfRule type="expression" dxfId="5" priority="4">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6471,8 +7018,8 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B17 B19 B21:B29 B31:B42" xr:uid="{1DFA3251-7984-4A3C-A048-50097DB9AAD3}">
       <formula1>"Desktop,Laptop,Tablet,All-In-One"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1 K1:K42 K45:K1048576" xr:uid="{A67DFFE0-1B96-49B5-A6E2-5C17E92A136C}"/>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J32:J42" xr:uid="{BD4480FF-AB8D-4446-AB7A-01C4C2A99ADB}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1 L1:L42 L45:L1048576" xr:uid="{A67DFFE0-1B96-49B5-A6E2-5C17E92A136C}"/>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K32:K42" xr:uid="{BD4480FF-AB8D-4446-AB7A-01C4C2A99ADB}">
       <formula1>1</formula1>
       <formula2>2000</formula2>
     </dataValidation>
@@ -6495,7 +7042,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="23" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="B1" s="24"/>
     </row>
@@ -6504,12 +7051,12 @@
         <v>115</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -6517,7 +7064,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
       <c r="B4">
         <v>9</v>
@@ -6525,7 +7072,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="B5">
         <v>2</v>
@@ -6533,7 +7080,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="B6">
         <v>10</v>
@@ -6541,7 +7088,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -6549,7 +7096,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="B8">
         <v>18</v>
@@ -6557,7 +7104,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="B9">
         <v>4</v>
@@ -6565,7 +7112,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="B10">
         <v>3</v>
@@ -6573,7 +7120,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="B11">
         <v>16</v>
@@ -6581,7 +7128,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="B12">
         <v>6</v>
@@ -6589,7 +7136,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
       <c r="B13">
         <v>3</v>
@@ -6597,7 +7144,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -6605,7 +7152,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="B15">
         <v>11</v>
@@ -6613,7 +7160,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="B16">
         <v>14</v>
@@ -6621,7 +7168,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="B17">
         <v>17</v>
@@ -6629,7 +7176,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -6637,7 +7184,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -6645,7 +7192,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="B20">
         <v>4</v>
@@ -6653,7 +7200,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="B21">
         <v>2</v>
@@ -6661,7 +7208,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -6669,7 +7216,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
       <c r="B23">
         <v>12</v>
@@ -6677,7 +7224,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -6685,7 +7232,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="B25">
         <v>3</v>
@@ -6693,7 +7240,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -6701,7 +7248,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -6709,7 +7256,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="B28">
         <v>2</v>
@@ -6717,7 +7264,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="B29">
         <v>9</v>
@@ -6725,7 +7272,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="B30">
         <v>1</v>
@@ -6733,7 +7280,7 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="B31">
         <v>5</v>
@@ -6741,7 +7288,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="B32">
         <v>3</v>
@@ -6749,7 +7296,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="B33">
         <v>6</v>
@@ -6757,7 +7304,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="B34">
         <v>1</v>
@@ -6765,7 +7312,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="B35">
         <v>2</v>
@@ -6773,7 +7320,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -6781,7 +7328,7 @@
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="B37">
         <v>14</v>
@@ -6789,7 +7336,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="B38">
         <v>5</v>
@@ -6797,7 +7344,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="B39">
         <v>2</v>
@@ -6805,7 +7352,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B40">
         <v>1</v>
@@ -6813,7 +7360,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -6821,7 +7368,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -6829,7 +7376,7 @@
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="B43">
         <v>1</v>
@@ -6837,7 +7384,7 @@
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="B44">
         <v>1</v>
@@ -6845,7 +7392,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="B45">
         <v>11</v>
@@ -6853,7 +7400,7 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
       <c r="B46">
         <v>16</v>
@@ -6861,7 +7408,7 @@
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="B47">
         <v>6</v>

</xml_diff>

<commit_message>
finished Donated items import
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/lucasja_rose-hulman_edu/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucasja\git\Inventory-System\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6F62A0D-D864-413C-A038-AF10FB8B133F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1769F4D0-9B06-4025-9E21-BBB42E246945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="4" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="255">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -803,6 +803,9 @@
   </si>
   <si>
     <t>WiFi Adapters</t>
+  </si>
+  <si>
+    <t>Intel core i7-i8850H</t>
   </si>
 </sst>
 </file>
@@ -814,7 +817,7 @@
     <numFmt numFmtId="164" formatCode="00000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1005,21 +1008,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="49">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1038,9 +1027,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1050,7 +1042,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="0"/>
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1138,182 +1130,6 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
           <bgColor theme="0"/>
         </patternFill>
       </fill>
@@ -1349,62 +1165,37 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="00000"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1433,7 +1224,7 @@
     <tableColumn id="13" xr3:uid="{5BEE40AD-E450-4A13-BFB5-1D0CED084DB3}" name="ID"/>
     <tableColumn id="8" xr3:uid="{E9AB9B46-3541-4715-8E5B-024096D78342}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{F7DAC8DD-8096-40F1-8780-1DB9CB4EC72F}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="24"/>
     <tableColumn id="5" xr3:uid="{5338F6FB-43B0-44AF-AF8B-542FAC6CEDF0}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{64D6C993-8518-4A7C-9BDA-A54D7DBFBA8E}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{E5D987A3-C54A-4907-B710-79DB224E0008}" name="Current Status" totalsRowFunction="count"/>
@@ -1452,7 +1243,7 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F96A3CC8-25D1-4CF8-877D-2816B26B7DC4}" name="Item Name" totalsRowLabel="Total"/>
-    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="45"/>
+    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="23"/>
     <tableColumn id="8" xr3:uid="{7D8F815E-A974-42A8-AC0B-AB8B951599A2}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{FEA94C75-B538-448A-A9F5-46F5A27E863D}" name="Year released"/>
     <tableColumn id="4" xr3:uid="{24998D92-36B7-4553-81E7-CB33711B31BB}" name="Special Reqs/Notes"/>
@@ -1474,7 +1265,7 @@
     <tableColumn id="13" xr3:uid="{EFFF3477-1A58-41CD-BFF3-45CE299505A7}" name="ID"/>
     <tableColumn id="8" xr3:uid="{C694899F-E385-4DE2-972A-7395A9633019}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{13C54556-A90A-4F9C-800D-3D838462DF46}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="22"/>
     <tableColumn id="5" xr3:uid="{6DE19FBC-9BD8-456E-9FC5-F633F61E4A34}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{68546225-0A78-43C1-A4F9-4D2E1DC008A3}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{0D7FD365-4F73-4A57-B8A1-CFAC47267923}" name="Current Status" totalsRowFunction="count"/>
@@ -1506,7 +1297,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="18">
   <autoFilter ref="A2:M59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{D71C6020-33AC-4F3C-BC88-69BADE52FD9C}" name="Item"/>
@@ -1518,9 +1309,9 @@
     <tableColumn id="13" xr3:uid="{D6E0079E-D628-428A-8C40-CC4B7F920E56}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{7319329B-DA0F-470E-AE1F-CAF023744072}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{96CAC308-4A56-4EA5-AF3F-FCAC656EEA09}" name="SSD/HDD"/>
-    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="17"/>
     <tableColumn id="12" xr3:uid="{04505084-FFBB-491E-B658-CE08D38C3E7B}" name="Notes"/>
-    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{45D6EFC2-97A5-4C00-9305-6B4ED43BEBB2}" name="Recipient"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1856,20 +1647,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5AA6A1-7D43-4966-8813-F497D895A5C2}">
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -1882,7 +1673,7 @@
       <c r="H1" s="23"/>
       <c r="I1" s="23"/>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1914,11 +1705,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E3" s="1"/>
       <c r="I3" s="16"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1944,11 +1735,11 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1974,7 +1765,7 @@
         <v>45673</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2001,7 +1792,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -2025,7 +1816,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -2049,7 +1840,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -2073,7 +1864,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -2097,7 +1888,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -2121,7 +1912,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30">
+    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -2147,7 +1938,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -2176,7 +1967,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="45">
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -2202,7 +1993,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -2226,7 +2017,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="30">
+    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2252,7 +2043,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -2276,7 +2067,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="30">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -2302,7 +2093,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -2326,7 +2117,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="29.25">
+    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2355,11 +2146,11 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E22" s="1"/>
       <c r="I22" s="16"/>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2383,7 +2174,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2407,11 +2198,11 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E25" s="1"/>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:9" ht="30">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -2437,7 +2228,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -2461,7 +2252,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -2485,7 +2276,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -2511,34 +2302,34 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="5:5">
+    <row r="34" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E34" s="1"/>
     </row>
-    <row r="35" spans="5:5">
+    <row r="35" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="5:5">
+    <row r="36" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="5:5">
+    <row r="37" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E37" s="1"/>
     </row>
-    <row r="38" spans="5:5">
+    <row r="38" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="5:5">
+    <row r="39" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E39" s="1"/>
     </row>
   </sheetData>
@@ -2571,18 +2362,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DEA6183-B753-401C-B21E-C502785DFA3D}">
   <dimension ref="A1:G63"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" style="12" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.5546875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
         <v>56</v>
       </c>
@@ -2593,7 +2384,7 @@
       <c r="F1" s="24"/>
       <c r="G1" s="24"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2616,7 +2407,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
@@ -2637,7 +2428,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>57</v>
       </c>
@@ -2658,7 +2449,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1">
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>57</v>
       </c>
@@ -2681,7 +2472,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.5">
+    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>57</v>
       </c>
@@ -2704,7 +2495,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>57</v>
       </c>
@@ -2725,7 +2516,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30">
+    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>57</v>
       </c>
@@ -2748,7 +2539,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
@@ -2769,7 +2560,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
       <c r="B10" s="14"/>
       <c r="C10" s="9"/>
@@ -2778,7 +2569,7 @@
       <c r="F10" s="9"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>57</v>
       </c>
@@ -2799,7 +2590,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="60">
+    <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>61</v>
       </c>
@@ -2822,7 +2613,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>61</v>
       </c>
@@ -2845,7 +2636,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>61</v>
       </c>
@@ -2866,7 +2657,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>61</v>
       </c>
@@ -2887,7 +2678,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>61</v>
       </c>
@@ -2908,7 +2699,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>61</v>
       </c>
@@ -2929,7 +2720,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>61</v>
       </c>
@@ -2950,7 +2741,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>61</v>
       </c>
@@ -2971,7 +2762,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>61</v>
       </c>
@@ -2992,7 +2783,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>61</v>
       </c>
@@ -3013,7 +2804,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>64</v>
       </c>
@@ -3034,7 +2825,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>65</v>
       </c>
@@ -3057,7 +2848,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>64</v>
       </c>
@@ -3078,7 +2869,7 @@
         <v>46052</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>64</v>
       </c>
@@ -3097,7 +2888,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="13"/>
       <c r="C26" s="5"/>
@@ -3106,7 +2897,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>64</v>
       </c>
@@ -3129,7 +2920,7 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>68</v>
       </c>
@@ -3150,7 +2941,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>69</v>
       </c>
@@ -3173,7 +2964,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>71</v>
       </c>
@@ -3196,7 +2987,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>73</v>
       </c>
@@ -3217,7 +3008,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>74</v>
       </c>
@@ -3238,7 +3029,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>75</v>
       </c>
@@ -3259,7 +3050,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>73</v>
       </c>
@@ -3280,7 +3071,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>76</v>
       </c>
@@ -3301,7 +3092,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -3324,7 +3115,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>64</v>
       </c>
@@ -3347,7 +3138,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -3367,7 +3158,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -3387,7 +3178,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>64</v>
       </c>
@@ -3410,7 +3201,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -3433,10 +3224,10 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G42" s="16"/>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -3456,7 +3247,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>81</v>
       </c>
@@ -3476,7 +3267,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>81</v>
       </c>
@@ -3496,7 +3287,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>86</v>
       </c>
@@ -3519,7 +3310,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -3542,7 +3333,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -3562,7 +3353,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>89</v>
       </c>
@@ -3579,7 +3370,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>91</v>
       </c>
@@ -3599,7 +3390,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>92</v>
       </c>
@@ -3619,7 +3410,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>93</v>
       </c>
@@ -3639,7 +3430,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>94</v>
       </c>
@@ -3662,7 +3453,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>97</v>
       </c>
@@ -3682,7 +3473,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -3705,7 +3496,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>100</v>
       </c>
@@ -3725,7 +3516,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>91</v>
       </c>
@@ -3745,7 +3536,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -3765,7 +3556,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -3788,16 +3579,16 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G60" s="16"/>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G61" s="16"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G62" s="16"/>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G63" s="16"/>
     </row>
   </sheetData>
@@ -3805,13 +3596,11 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:G63">
-    <cfRule type="expression" dxfId="47" priority="2">
+    <cfRule type="expression" dxfId="15" priority="1">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A3:G63">
-    <cfRule type="expression" dxfId="46" priority="1">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -3829,20 +3618,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F948288C-1730-49D1-BD4C-FC704F167D22}">
   <dimension ref="A1:I33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
         <v>102</v>
       </c>
@@ -3855,7 +3644,7 @@
       <c r="H1" s="24"/>
       <c r="I1" s="24"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -3884,7 +3673,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>103</v>
       </c>
@@ -3913,7 +3702,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>103</v>
       </c>
@@ -3942,91 +3731,91 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="5:5">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="5:5">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="5:5">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="5:5">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="5:5">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="5:5">
+    <row r="22" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="5:5">
+    <row r="23" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="5:5">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="5:5">
+    <row r="25" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="5:5">
+    <row r="26" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="5:5">
+    <row r="27" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="5:5">
+    <row r="28" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="5:5">
+    <row r="29" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="5:5">
+    <row r="30" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="5:5">
+    <row r="31" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="5:5">
+    <row r="32" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="1"/>
     </row>
   </sheetData>
@@ -4058,22 +3847,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE86381-3E33-4CB8-A62B-E48A74AB9667}">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.33203125" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="17.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" style="19" customWidth="1"/>
-    <col min="11" max="11" width="21.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="19" customWidth="1"/>
+    <col min="11" max="11" width="21.33203125" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>107</v>
       </c>
@@ -4089,7 +3878,7 @@
       <c r="K1" s="26"/>
       <c r="L1" s="26"/>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -4127,7 +3916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -4163,7 +3952,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>125</v>
       </c>
@@ -4199,7 +3988,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>128</v>
       </c>
@@ -4235,10 +4024,10 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>128</v>
       </c>
@@ -4274,7 +4063,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>84</v>
       </c>
@@ -4310,7 +4099,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>133</v>
       </c>
@@ -4346,10 +4135,10 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -4385,7 +4174,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>138</v>
       </c>
@@ -4420,7 +4209,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>140</v>
       </c>
@@ -4456,7 +4245,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1">
+    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -4492,7 +4281,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1">
+    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -4528,7 +4317,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1">
+    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -4564,7 +4353,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15" customHeight="1">
+    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>146</v>
       </c>
@@ -4600,7 +4389,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15" customHeight="1">
+    <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>149</v>
       </c>
@@ -4636,7 +4425,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="15" customHeight="1">
+    <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>149</v>
       </c>
@@ -4672,7 +4461,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1">
+    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>151</v>
       </c>
@@ -4708,7 +4497,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15" customHeight="1">
+    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>151</v>
       </c>
@@ -4744,7 +4533,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15" customHeight="1">
+    <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>61</v>
       </c>
@@ -4780,7 +4569,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15" customHeight="1">
+    <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>154</v>
       </c>
@@ -4816,7 +4605,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15" customHeight="1">
+    <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>57</v>
       </c>
@@ -4852,7 +4641,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15" customHeight="1">
+    <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>128</v>
       </c>
@@ -4888,7 +4677,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="15" customHeight="1">
+    <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -4924,7 +4713,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="15" customHeight="1">
+    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -4960,7 +4749,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="15" customHeight="1">
+    <row r="28" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>64</v>
       </c>
@@ -4996,7 +4785,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="15" customHeight="1">
+    <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>159</v>
       </c>
@@ -5032,129 +4821,53 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="15" customHeight="1">
+    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:12" ht="15" customHeight="1">
+    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:12" ht="15" customHeight="1">
+    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="11:11" ht="15" customHeight="1">
+    <row r="33" spans="11:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K33" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A15:C15 A3:K9 A11:K14 E15:K15 A16:K25">
-    <cfRule type="expression" dxfId="43" priority="21">
+  <conditionalFormatting sqref="A27:A28">
+    <cfRule type="expression" dxfId="13" priority="17">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="18">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:K9 A11:K14 A15:C15 E15:K15 A16:K25">
+    <cfRule type="expression" dxfId="11" priority="21">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15:C15 A3:L9 A11:L14 E15:L15 A16:L25">
-    <cfRule type="expression" dxfId="42" priority="22">
+  <conditionalFormatting sqref="A3:L9 A11:L14 A15:C15 E15:L15 A16:L25">
+    <cfRule type="expression" dxfId="10" priority="22">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A27">
-    <cfRule type="expression" dxfId="41" priority="20">
+  <conditionalFormatting sqref="G26:G29">
+    <cfRule type="expression" dxfId="9" priority="9">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A27">
-    <cfRule type="expression" dxfId="40" priority="19">
+  <conditionalFormatting sqref="H26:H29">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A28">
-    <cfRule type="expression" dxfId="39" priority="18">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A28">
-    <cfRule type="expression" dxfId="38" priority="17">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G28">
-    <cfRule type="expression" dxfId="37" priority="15">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G28">
-    <cfRule type="expression" dxfId="36" priority="16">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G26">
-    <cfRule type="expression" dxfId="35" priority="13">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G26">
-    <cfRule type="expression" dxfId="34" priority="14">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
-    <cfRule type="expression" dxfId="33" priority="11">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
-    <cfRule type="expression" dxfId="32" priority="12">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
-    <cfRule type="expression" dxfId="31" priority="9">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
-    <cfRule type="expression" dxfId="30" priority="10">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H26">
-    <cfRule type="expression" dxfId="29" priority="7">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H26">
-    <cfRule type="expression" dxfId="28" priority="8">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="expression" dxfId="27" priority="5">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
-    <cfRule type="expression" dxfId="26" priority="6">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
-    <cfRule type="expression" dxfId="25" priority="3">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
-    <cfRule type="expression" dxfId="24" priority="4">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
-    <cfRule type="expression" dxfId="23" priority="1">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5177,26 +4890,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19592962-4FD3-47C5-914B-6346C180BC2C}">
   <dimension ref="A1:O59"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" customWidth="1"/>
-    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.28515625" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" style="16" customWidth="1"/>
-    <col min="13" max="13" width="29.140625" customWidth="1"/>
-    <col min="14" max="14" width="27.7109375" customWidth="1"/>
-    <col min="15" max="15" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.33203125" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" style="16" customWidth="1"/>
+    <col min="13" max="13" width="29.109375" customWidth="1"/>
+    <col min="14" max="14" width="27.6640625" customWidth="1"/>
+    <col min="15" max="15" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15" customHeight="1">
+    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="17" t="s">
         <v>161</v>
       </c>
@@ -5218,7 +4931,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -5267,12 +4980,33 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>166</v>
       </c>
       <c r="B3" t="s">
         <v>126</v>
+      </c>
+      <c r="C3">
+        <v>2019</v>
+      </c>
+      <c r="D3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H3">
+        <v>256</v>
+      </c>
+      <c r="I3" t="s">
+        <v>124</v>
       </c>
       <c r="J3" s="19">
         <v>225</v>
@@ -5285,12 +5019,33 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>166</v>
       </c>
       <c r="B4" t="s">
         <v>126</v>
+      </c>
+      <c r="C4">
+        <v>2019</v>
+      </c>
+      <c r="D4" t="s">
+        <v>254</v>
+      </c>
+      <c r="E4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F4">
+        <v>8</v>
+      </c>
+      <c r="G4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H4">
+        <v>256</v>
+      </c>
+      <c r="I4" t="s">
+        <v>124</v>
       </c>
       <c r="J4" s="19">
         <v>225</v>
@@ -5303,12 +5058,33 @@
         <v>167</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>166</v>
       </c>
       <c r="B5" t="s">
         <v>126</v>
+      </c>
+      <c r="C5">
+        <v>2019</v>
+      </c>
+      <c r="D5" t="s">
+        <v>254</v>
+      </c>
+      <c r="E5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>130</v>
+      </c>
+      <c r="H5">
+        <v>256</v>
+      </c>
+      <c r="I5" t="s">
+        <v>124</v>
       </c>
       <c r="J5" s="19">
         <v>225</v>
@@ -5321,12 +5097,33 @@
         <v>167</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>166</v>
       </c>
       <c r="B6" t="s">
         <v>126</v>
+      </c>
+      <c r="C6">
+        <v>2019</v>
+      </c>
+      <c r="D6" t="s">
+        <v>254</v>
+      </c>
+      <c r="E6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H6">
+        <v>256</v>
+      </c>
+      <c r="I6" t="s">
+        <v>124</v>
       </c>
       <c r="J6" s="19">
         <v>225</v>
@@ -5339,12 +5136,33 @@
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>166</v>
       </c>
       <c r="B7" t="s">
         <v>126</v>
+      </c>
+      <c r="C7">
+        <v>2019</v>
+      </c>
+      <c r="D7" t="s">
+        <v>254</v>
+      </c>
+      <c r="E7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>130</v>
+      </c>
+      <c r="H7">
+        <v>256</v>
+      </c>
+      <c r="I7" t="s">
+        <v>124</v>
       </c>
       <c r="J7" s="19">
         <v>225</v>
@@ -5357,12 +5175,33 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>166</v>
       </c>
       <c r="B8" t="s">
         <v>126</v>
+      </c>
+      <c r="C8">
+        <v>2019</v>
+      </c>
+      <c r="D8" t="s">
+        <v>254</v>
+      </c>
+      <c r="E8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F8">
+        <v>8</v>
+      </c>
+      <c r="G8" t="s">
+        <v>130</v>
+      </c>
+      <c r="H8">
+        <v>256</v>
+      </c>
+      <c r="I8" t="s">
+        <v>124</v>
       </c>
       <c r="J8" s="19">
         <v>225</v>
@@ -5375,12 +5214,33 @@
         <v>167</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>166</v>
       </c>
       <c r="B9" t="s">
         <v>126</v>
+      </c>
+      <c r="C9">
+        <v>2019</v>
+      </c>
+      <c r="D9" t="s">
+        <v>254</v>
+      </c>
+      <c r="E9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>130</v>
+      </c>
+      <c r="H9">
+        <v>256</v>
+      </c>
+      <c r="I9" t="s">
+        <v>124</v>
       </c>
       <c r="J9" s="19">
         <v>225</v>
@@ -5393,7 +5253,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>168</v>
       </c>
@@ -5432,7 +5292,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>170</v>
       </c>
@@ -5471,7 +5331,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>172</v>
       </c>
@@ -5512,7 +5372,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>175</v>
       </c>
@@ -5551,7 +5411,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>168</v>
       </c>
@@ -5590,7 +5450,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>177</v>
       </c>
@@ -5629,7 +5489,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>179</v>
       </c>
@@ -5670,7 +5530,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>186</v>
       </c>
@@ -5711,7 +5571,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>187</v>
       </c>
@@ -5752,7 +5612,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>64</v>
       </c>
@@ -5793,7 +5653,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="43.5">
+    <row r="20" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -5834,7 +5694,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>196</v>
       </c>
@@ -5873,7 +5733,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -5912,7 +5772,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -5951,7 +5811,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -5990,7 +5850,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -6029,7 +5889,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -6068,7 +5928,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>61</v>
       </c>
@@ -6107,7 +5967,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>199</v>
       </c>
@@ -6146,7 +6006,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="29" spans="1:13">
+    <row r="29" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>199</v>
       </c>
@@ -6185,7 +6045,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="30" spans="1:13">
+    <row r="30" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>128</v>
       </c>
@@ -6224,7 +6084,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>61</v>
       </c>
@@ -6263,7 +6123,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:13">
+    <row r="32" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>61</v>
       </c>
@@ -6301,7 +6161,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>61</v>
       </c>
@@ -6339,7 +6199,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>203</v>
       </c>
@@ -6377,7 +6237,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>203</v>
       </c>
@@ -6415,7 +6275,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>203</v>
       </c>
@@ -6453,7 +6313,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>203</v>
       </c>
@@ -6491,7 +6351,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>203</v>
       </c>
@@ -6529,7 +6389,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>203</v>
       </c>
@@ -6567,7 +6427,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="15" customHeight="1">
+    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>203</v>
       </c>
@@ -6605,7 +6465,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="15" customHeight="1">
+    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>203</v>
       </c>
@@ -6643,7 +6503,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="15" customHeight="1">
+    <row r="42" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>203</v>
       </c>
@@ -6681,7 +6541,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="15" customHeight="1">
+    <row r="43" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>140</v>
       </c>
@@ -6720,7 +6580,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="15" customHeight="1">
+    <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>61</v>
       </c>
@@ -6759,67 +6619,67 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="15" customHeight="1">
+    <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L45" s="15"/>
     </row>
-    <row r="46" spans="1:13" ht="15" customHeight="1">
+    <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L46" s="15"/>
     </row>
-    <row r="47" spans="1:13" ht="15" customHeight="1">
+    <row r="47" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L47" s="15"/>
     </row>
-    <row r="48" spans="1:13" ht="15" customHeight="1">
+    <row r="48" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L48" s="15"/>
     </row>
-    <row r="49" spans="12:12" ht="15" customHeight="1">
+    <row r="49" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L49" s="15"/>
     </row>
-    <row r="50" spans="12:12" ht="15" customHeight="1">
+    <row r="50" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L50" s="15"/>
     </row>
-    <row r="51" spans="12:12" ht="15" customHeight="1">
+    <row r="51" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L51" s="15"/>
     </row>
-    <row r="52" spans="12:12" ht="15" customHeight="1">
+    <row r="52" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L52" s="15"/>
     </row>
-    <row r="53" spans="12:12" ht="15" customHeight="1">
+    <row r="53" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L53" s="15"/>
     </row>
-    <row r="54" spans="12:12" ht="15" customHeight="1">
+    <row r="54" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L54" s="15"/>
     </row>
-    <row r="55" spans="12:12" ht="15" customHeight="1">
+    <row r="55" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L55" s="15"/>
     </row>
-    <row r="56" spans="12:12" ht="15" customHeight="1">
+    <row r="56" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L56" s="15"/>
     </row>
-    <row r="57" spans="12:12" ht="15" customHeight="1">
+    <row r="57" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L57" s="15"/>
     </row>
-    <row r="58" spans="12:12" ht="15" customHeight="1">
+    <row r="58" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L58" s="15"/>
     </row>
-    <row r="59" spans="12:12" ht="15" customHeight="1">
+    <row r="59" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L59" s="15"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A44:F44 H44:K44">
-    <cfRule type="expression" dxfId="18" priority="15">
+    <cfRule type="expression" dxfId="5" priority="15">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A44:F44 H44:L44">
-    <cfRule type="expression" dxfId="17" priority="16">
+    <cfRule type="expression" dxfId="4" priority="16">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M44 A45:M59 A3:M9 A10:G15 I10:M15 A16:M43">
+  <conditionalFormatting sqref="A3:M9 A10:G15 I10:M15 A16:M43 M44 A45:M59">
     <cfRule type="expression" priority="17">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="18">
+    <cfRule type="expression" dxfId="3" priority="18">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6827,67 +6687,15 @@
     <cfRule type="expression" priority="13">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="14">
+    <cfRule type="expression" dxfId="2" priority="14">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
-    <cfRule type="expression" dxfId="14" priority="11">
+  <conditionalFormatting sqref="H10:H15">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
-    <cfRule type="expression" dxfId="13" priority="12">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H11">
-    <cfRule type="expression" dxfId="12" priority="9">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H11">
-    <cfRule type="expression" dxfId="11" priority="10">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H12">
-    <cfRule type="expression" dxfId="10" priority="7">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H12">
-    <cfRule type="expression" dxfId="9" priority="8">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H13">
-    <cfRule type="expression" dxfId="8" priority="5">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H13">
-    <cfRule type="expression" dxfId="7" priority="6">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H14">
-    <cfRule type="expression" dxfId="6" priority="3">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H14">
-    <cfRule type="expression" dxfId="5" priority="4">
-      <formula>ISODD(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H15">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H15">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6911,19 +6719,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66F9EB6D-6D2E-43F3-A79F-D2A5CF3A037E}">
   <dimension ref="A1:B47"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="1" max="1" width="46.109375" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>207</v>
       </c>
       <c r="B1" s="26"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -6931,7 +6739,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>209</v>
       </c>
@@ -6939,7 +6747,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>210</v>
       </c>
@@ -6947,7 +6755,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>211</v>
       </c>
@@ -6955,7 +6763,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>212</v>
       </c>
@@ -6963,7 +6771,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>213</v>
       </c>
@@ -6971,7 +6779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>214</v>
       </c>
@@ -6979,7 +6787,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>215</v>
       </c>
@@ -6987,7 +6795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>216</v>
       </c>
@@ -6995,7 +6803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>217</v>
       </c>
@@ -7003,7 +6811,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>218</v>
       </c>
@@ -7011,7 +6819,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>219</v>
       </c>
@@ -7019,7 +6827,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>220</v>
       </c>
@@ -7027,7 +6835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>221</v>
       </c>
@@ -7035,7 +6843,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>222</v>
       </c>
@@ -7043,7 +6851,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>223</v>
       </c>
@@ -7051,7 +6859,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>224</v>
       </c>
@@ -7059,7 +6867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>225</v>
       </c>
@@ -7067,7 +6875,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>226</v>
       </c>
@@ -7075,7 +6883,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>227</v>
       </c>
@@ -7083,7 +6891,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>228</v>
       </c>
@@ -7091,7 +6899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>229</v>
       </c>
@@ -7099,7 +6907,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>230</v>
       </c>
@@ -7107,7 +6915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>231</v>
       </c>
@@ -7115,7 +6923,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>232</v>
       </c>
@@ -7123,7 +6931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>233</v>
       </c>
@@ -7131,7 +6939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>234</v>
       </c>
@@ -7139,7 +6947,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>235</v>
       </c>
@@ -7147,7 +6955,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>236</v>
       </c>
@@ -7155,7 +6963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>237</v>
       </c>
@@ -7163,7 +6971,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>238</v>
       </c>
@@ -7171,7 +6979,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>239</v>
       </c>
@@ -7179,7 +6987,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>240</v>
       </c>
@@ -7187,7 +6995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>241</v>
       </c>
@@ -7195,7 +7003,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>242</v>
       </c>
@@ -7203,7 +7011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>243</v>
       </c>
@@ -7211,7 +7019,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>244</v>
       </c>
@@ -7219,7 +7027,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>245</v>
       </c>
@@ -7227,7 +7035,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>246</v>
       </c>
@@ -7235,7 +7043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>247</v>
       </c>
@@ -7243,7 +7051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>248</v>
       </c>
@@ -7251,7 +7059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>249</v>
       </c>
@@ -7259,7 +7067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>250</v>
       </c>
@@ -7267,7 +7075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>251</v>
       </c>
@@ -7275,7 +7083,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>252</v>
       </c>
@@ -7283,7 +7091,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>253</v>
       </c>

</xml_diff>

<commit_message>
sproc to insert into parts table -- backend support not finished
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucasja\git\Inventory-System\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\lucasja\Inventory-System\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1769F4D0-9B06-4025-9E21-BBB42E246945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39906191-F046-4C44-A76B-7AC87B711D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Ready To Donate" sheetId="2" r:id="rId4"/>
     <sheet name="Donated" sheetId="6" r:id="rId5"/>
     <sheet name="Parts" sheetId="3" r:id="rId6"/>
+    <sheet name="Tools" sheetId="12" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="257">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -670,45 +671,6 @@
     <t>Qty</t>
   </si>
   <si>
-    <t>2.5" SSDs</t>
-  </si>
-  <si>
-    <t>M.2 SSDs</t>
-  </si>
-  <si>
-    <t>1GB DDR3 SODIMM</t>
-  </si>
-  <si>
-    <t>2GB DDR4 SODIMM</t>
-  </si>
-  <si>
-    <t>2GB DDR3 SODIMM</t>
-  </si>
-  <si>
-    <t>8GB DDR4 SODIMM</t>
-  </si>
-  <si>
-    <t>8GB DDR3 SODIMM</t>
-  </si>
-  <si>
-    <t>4GB DDR4 SODIMM</t>
-  </si>
-  <si>
-    <t>4GB DDR3 SODIMM</t>
-  </si>
-  <si>
-    <t>8GB DDR4 DIMM</t>
-  </si>
-  <si>
-    <t>8GB DDR3 DIMM</t>
-  </si>
-  <si>
-    <t>16GB DDR4 DIMM</t>
-  </si>
-  <si>
-    <t>4GB DDR3 DIMM</t>
-  </si>
-  <si>
     <t>USB Keyboard</t>
   </si>
   <si>
@@ -806,6 +768,51 @@
   </si>
   <si>
     <t>Intel core i7-i8850H</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>SATA SSD</t>
+  </si>
+  <si>
+    <t>M.2 SSD</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>SODIMM</t>
+  </si>
+  <si>
+    <t>8GB DDR4</t>
+  </si>
+  <si>
+    <t>2GB DDR3</t>
+  </si>
+  <si>
+    <t>4GB DDR3</t>
+  </si>
+  <si>
+    <t>2GB DDR4</t>
+  </si>
+  <si>
+    <t>8GB DDR3</t>
+  </si>
+  <si>
+    <t>4GB DDR4</t>
+  </si>
+  <si>
+    <t>16GB DDR4</t>
+  </si>
+  <si>
+    <t>1GB DDR3</t>
+  </si>
+  <si>
+    <t>DIMM</t>
+  </si>
+  <si>
+    <t>TOOLS</t>
   </si>
 </sst>
 </file>
@@ -948,7 +955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1002,6 +1009,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1165,20 +1175,6 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1199,6 +1195,20 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1224,7 +1234,7 @@
     <tableColumn id="13" xr3:uid="{5BEE40AD-E450-4A13-BFB5-1D0CED084DB3}" name="ID"/>
     <tableColumn id="8" xr3:uid="{E9AB9B46-3541-4715-8E5B-024096D78342}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{F7DAC8DD-8096-40F1-8780-1DB9CB4EC72F}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="21"/>
     <tableColumn id="5" xr3:uid="{5338F6FB-43B0-44AF-AF8B-542FAC6CEDF0}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{64D6C993-8518-4A7C-9BDA-A54D7DBFBA8E}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{E5D987A3-C54A-4907-B710-79DB224E0008}" name="Current Status" totalsRowFunction="count"/>
@@ -1243,7 +1253,7 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F96A3CC8-25D1-4CF8-877D-2816B26B7DC4}" name="Item Name" totalsRowLabel="Total"/>
-    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="20"/>
     <tableColumn id="8" xr3:uid="{7D8F815E-A974-42A8-AC0B-AB8B951599A2}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{FEA94C75-B538-448A-A9F5-46F5A27E863D}" name="Year released"/>
     <tableColumn id="4" xr3:uid="{24998D92-36B7-4553-81E7-CB33711B31BB}" name="Special Reqs/Notes"/>
@@ -1265,7 +1275,7 @@
     <tableColumn id="13" xr3:uid="{EFFF3477-1A58-41CD-BFF3-45CE299505A7}" name="ID"/>
     <tableColumn id="8" xr3:uid="{C694899F-E385-4DE2-972A-7395A9633019}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{13C54556-A90A-4F9C-800D-3D838462DF46}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="19"/>
     <tableColumn id="5" xr3:uid="{6DE19FBC-9BD8-456E-9FC5-F633F61E4A34}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{68546225-0A78-43C1-A4F9-4D2E1DC008A3}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{0D7FD365-4F73-4A57-B8A1-CFAC47267923}" name="Current Status" totalsRowFunction="count"/>
@@ -1276,7 +1286,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="18">
   <autoFilter ref="A2:L33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{73648E04-2EA1-4ADB-8E24-E7DDE01C0462}" name="Item"/>
@@ -1288,8 +1298,8 @@
     <tableColumn id="2" xr3:uid="{C85B34EB-06B2-40A8-BBCB-B5F170EF3F82}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{A686D1B3-031E-4544-A98D-8F3144FA62B0}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{AB29939A-0AF4-4451-A6F4-2144F8957E73}" name="SSD/HDD"/>
-    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="16"/>
     <tableColumn id="12" xr3:uid="{67EC036F-98F6-4C6B-BDD7-99DB9B6ADF97}" name="ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1297,7 +1307,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="24">
   <autoFilter ref="A2:M59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{D71C6020-33AC-4F3C-BC88-69BADE52FD9C}" name="Item"/>
@@ -1309,9 +1319,9 @@
     <tableColumn id="13" xr3:uid="{D6E0079E-D628-428A-8C40-CC4B7F920E56}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{7319329B-DA0F-470E-AE1F-CAF023744072}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{96CAC308-4A56-4EA5-AF3F-FCAC656EEA09}" name="SSD/HDD"/>
-    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="23"/>
     <tableColumn id="12" xr3:uid="{04505084-FFBB-491E-B658-CE08D38C3E7B}" name="Notes"/>
-    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="22"/>
     <tableColumn id="2" xr3:uid="{45D6EFC2-97A5-4C00-9305-6B4ED43BEBB2}" name="Recipient"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1319,11 +1329,24 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}" name="Parts" displayName="Parts" ref="A2:B47" totalsRowShown="0">
-  <autoFilter ref="A2:B47" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{AE6A62C8-410E-43CA-9FCC-DB171FCD3CD1}" name="Item"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}" name="Parts" displayName="Parts" ref="A2:C15" totalsRowShown="0">
+  <autoFilter ref="A2:C15" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{AE6A62C8-410E-43CA-9FCC-DB171FCD3CD1}" name="Type"/>
+    <tableColumn id="3" xr3:uid="{8BE6192C-E1B9-4BD5-BEB2-D26E68C58775}" name="Description"/>
     <tableColumn id="2" xr3:uid="{675E5FD2-430E-4D35-9481-575A83791C4E}" name="Qty"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{42D1C34C-9303-4D46-A107-174D17AE2274}" name="Parts5" displayName="Parts5" ref="A2:C34" totalsRowShown="0">
+  <autoFilter ref="A2:C34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{C29E963F-354B-4750-B17F-22461F6DC5F4}" name="Type"/>
+    <tableColumn id="3" xr3:uid="{7C7B0B32-2D9C-4EDB-8E56-4C2ADECB5869}" name="Description"/>
+    <tableColumn id="2" xr3:uid="{1155C0CA-025A-4922-8B0E-F2A817B3BB60}" name="Qty"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4991,7 +5014,7 @@
         <v>2019</v>
       </c>
       <c r="D3" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E3" t="s">
         <v>137</v>
@@ -5030,7 +5053,7 @@
         <v>2019</v>
       </c>
       <c r="D4" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E4" t="s">
         <v>137</v>
@@ -5069,7 +5092,7 @@
         <v>2019</v>
       </c>
       <c r="D5" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E5" t="s">
         <v>137</v>
@@ -5108,7 +5131,7 @@
         <v>2019</v>
       </c>
       <c r="D6" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E6" t="s">
         <v>137</v>
@@ -5147,7 +5170,7 @@
         <v>2019</v>
       </c>
       <c r="D7" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E7" t="s">
         <v>137</v>
@@ -5186,7 +5209,7 @@
         <v>2019</v>
       </c>
       <c r="D8" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E8" t="s">
         <v>137</v>
@@ -5225,7 +5248,7 @@
         <v>2019</v>
       </c>
       <c r="D9" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="E9" t="s">
         <v>137</v>
@@ -6718,390 +6741,467 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66F9EB6D-6D2E-43F3-A79F-D2A5CF3A037E}">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.109375" customWidth="1"/>
-    <col min="2" max="2" width="10.109375" customWidth="1"/>
+    <col min="1" max="1" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="26"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" s="27"/>
+      <c r="C1" s="26"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B5" t="s">
+        <v>254</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>246</v>
+      </c>
+      <c r="B6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B9" t="s">
+        <v>251</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B10" t="s">
+        <v>252</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>246</v>
+      </c>
+      <c r="B11" t="s">
+        <v>249</v>
+      </c>
+      <c r="C11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>255</v>
+      </c>
+      <c r="B12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>255</v>
+      </c>
+      <c r="B13" t="s">
+        <v>251</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>255</v>
+      </c>
+      <c r="B14" t="s">
+        <v>253</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>255</v>
+      </c>
+      <c r="B15" t="s">
+        <v>249</v>
+      </c>
+      <c r="C15">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6AEFF60-27EE-498D-A491-C67356035C05}">
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="26"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>209</v>
       </c>
-      <c r="B3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>210</v>
       </c>
-      <c r="B4">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>211</v>
       </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>212</v>
       </c>
-      <c r="B6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>213</v>
       </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>214</v>
       </c>
-      <c r="B8">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>215</v>
       </c>
-      <c r="B9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>216</v>
       </c>
-      <c r="B10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>217</v>
       </c>
-      <c r="B11">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>218</v>
       </c>
-      <c r="B12">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>219</v>
       </c>
-      <c r="B13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>220</v>
       </c>
-      <c r="B14">
+      <c r="C14">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>221</v>
       </c>
-      <c r="B15">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>222</v>
       </c>
-      <c r="B16">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>223</v>
       </c>
-      <c r="B17">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>224</v>
       </c>
-      <c r="B18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>225</v>
       </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>226</v>
       </c>
-      <c r="B20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>227</v>
       </c>
-      <c r="B21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>228</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>229</v>
       </c>
-      <c r="B23">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>230</v>
       </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C24">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>231</v>
       </c>
-      <c r="B25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>232</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>233</v>
       </c>
-      <c r="B27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>234</v>
       </c>
-      <c r="B28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>235</v>
       </c>
-      <c r="B29">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>236</v>
       </c>
-      <c r="B30">
+      <c r="C30">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>237</v>
       </c>
-      <c r="B31">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>238</v>
       </c>
-      <c r="B32">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C32">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>239</v>
       </c>
-      <c r="B33">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C33">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>240</v>
       </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>241</v>
-      </c>
-      <c r="B35">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>242</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>243</v>
-      </c>
-      <c r="B37">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>244</v>
-      </c>
-      <c r="B38">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>245</v>
-      </c>
-      <c r="B39">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>246</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>247</v>
-      </c>
-      <c r="B41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>248</v>
-      </c>
-      <c r="B42">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>249</v>
-      </c>
-      <c r="B43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>250</v>
-      </c>
-      <c r="B44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>251</v>
-      </c>
-      <c r="B45">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>252</v>
-      </c>
-      <c r="B46">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>253</v>
-      </c>
-      <c r="B47">
+      <c r="C34">
         <v>6</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fixed PartType enum declarations and dependencies -- still actual import not implemented
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\lucasja\Inventory-System\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39906191-F046-4C44-A76B-7AC87B711D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843F4EDD-8E2F-4262-BF42-795457F9E7F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -776,9 +776,6 @@
     <t>SATA SSD</t>
   </si>
   <si>
-    <t>M.2 SSD</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -813,6 +810,9 @@
   </si>
   <si>
     <t>TOOLS</t>
+  </si>
+  <si>
+    <t>M2 SSD</t>
   </si>
 </sst>
 </file>
@@ -955,7 +955,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -999,19 +999,16 @@
     <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1175,6 +1172,20 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1195,20 +1206,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1234,7 +1231,7 @@
     <tableColumn id="13" xr3:uid="{5BEE40AD-E450-4A13-BFB5-1D0CED084DB3}" name="ID"/>
     <tableColumn id="8" xr3:uid="{E9AB9B46-3541-4715-8E5B-024096D78342}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{F7DAC8DD-8096-40F1-8780-1DB9CB4EC72F}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="24"/>
     <tableColumn id="5" xr3:uid="{5338F6FB-43B0-44AF-AF8B-542FAC6CEDF0}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{64D6C993-8518-4A7C-9BDA-A54D7DBFBA8E}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{E5D987A3-C54A-4907-B710-79DB224E0008}" name="Current Status" totalsRowFunction="count"/>
@@ -1253,7 +1250,7 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F96A3CC8-25D1-4CF8-877D-2816B26B7DC4}" name="Item Name" totalsRowLabel="Total"/>
-    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="20"/>
+    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="23"/>
     <tableColumn id="8" xr3:uid="{7D8F815E-A974-42A8-AC0B-AB8B951599A2}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{FEA94C75-B538-448A-A9F5-46F5A27E863D}" name="Year released"/>
     <tableColumn id="4" xr3:uid="{24998D92-36B7-4553-81E7-CB33711B31BB}" name="Special Reqs/Notes"/>
@@ -1275,7 +1272,7 @@
     <tableColumn id="13" xr3:uid="{EFFF3477-1A58-41CD-BFF3-45CE299505A7}" name="ID"/>
     <tableColumn id="8" xr3:uid="{C694899F-E385-4DE2-972A-7395A9633019}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{13C54556-A90A-4F9C-800D-3D838462DF46}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="22"/>
     <tableColumn id="5" xr3:uid="{6DE19FBC-9BD8-456E-9FC5-F633F61E4A34}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{68546225-0A78-43C1-A4F9-4D2E1DC008A3}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{0D7FD365-4F73-4A57-B8A1-CFAC47267923}" name="Current Status" totalsRowFunction="count"/>
@@ -1286,7 +1283,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="21">
   <autoFilter ref="A2:L33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{73648E04-2EA1-4ADB-8E24-E7DDE01C0462}" name="Item"/>
@@ -1298,8 +1295,8 @@
     <tableColumn id="2" xr3:uid="{C85B34EB-06B2-40A8-BBCB-B5F170EF3F82}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{A686D1B3-031E-4544-A98D-8F3144FA62B0}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{AB29939A-0AF4-4451-A6F4-2144F8957E73}" name="SSD/HDD"/>
-    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="19"/>
     <tableColumn id="12" xr3:uid="{67EC036F-98F6-4C6B-BDD7-99DB9B6ADF97}" name="ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1307,7 +1304,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="18">
   <autoFilter ref="A2:M59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{D71C6020-33AC-4F3C-BC88-69BADE52FD9C}" name="Item"/>
@@ -1319,9 +1316,9 @@
     <tableColumn id="13" xr3:uid="{D6E0079E-D628-428A-8C40-CC4B7F920E56}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{7319329B-DA0F-470E-AE1F-CAF023744072}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{96CAC308-4A56-4EA5-AF3F-FCAC656EEA09}" name="SSD/HDD"/>
-    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="17"/>
     <tableColumn id="12" xr3:uid="{04505084-FFBB-491E-B658-CE08D38C3E7B}" name="Notes"/>
-    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{45D6EFC2-97A5-4C00-9305-6B4ED43BEBB2}" name="Recipient"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1684,17 +1681,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -2397,15 +2394,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -3655,17 +3652,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -3886,20 +3883,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
     </row>
     <row r="2" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -6750,18 +6747,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="26"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>242</v>
       </c>
       <c r="B2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>208</v>
@@ -6777,7 +6774,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="C4">
         <v>9</v>
@@ -6785,10 +6782,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -6796,10 +6793,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C6">
         <v>10</v>
@@ -6807,10 +6804,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B7" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -6818,10 +6815,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B8" t="s">
         <v>246</v>
-      </c>
-      <c r="B8" t="s">
-        <v>247</v>
       </c>
       <c r="C8">
         <v>18</v>
@@ -6829,10 +6826,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C9">
         <v>4</v>
@@ -6840,10 +6837,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C10">
         <v>3</v>
@@ -6851,10 +6848,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C11">
         <v>16</v>
@@ -6862,10 +6859,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C12">
         <v>6</v>
@@ -6873,10 +6870,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C13">
         <v>3</v>
@@ -6884,10 +6881,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -6895,10 +6892,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B15" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C15">
         <v>11</v>
@@ -6926,18 +6923,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
-        <v>256</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="26"/>
+      <c r="A1" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>242</v>
       </c>
       <c r="B2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>208</v>

</xml_diff>

<commit_message>
finished import parts, fixed import donated devices
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\lucasja\Inventory-System\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/lucasja_rose-hulman_edu/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843F4EDD-8E2F-4262-BF42-795457F9E7F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3460" documentId="8_{A0F2C8DF-695D-4A53-BA74-C2F5D1F57A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73C00331-DB68-481F-98A9-F3303D7051BD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="4" activeTab="5" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
     <sheet name="Desktops" sheetId="7" r:id="rId2"/>
     <sheet name="Tablets" sheetId="10" r:id="rId3"/>
     <sheet name="Ready To Donate" sheetId="2" r:id="rId4"/>
-    <sheet name="Donated" sheetId="6" r:id="rId5"/>
-    <sheet name="Parts" sheetId="3" r:id="rId6"/>
-    <sheet name="Tools" sheetId="12" r:id="rId7"/>
+    <sheet name="Donated" sheetId="11" r:id="rId5"/>
+    <sheet name="Parts" sheetId="12" r:id="rId6"/>
+    <sheet name="Tools" sheetId="13" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="255">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -665,40 +665,133 @@
     <t>Wabash Activity Center</t>
   </si>
   <si>
-    <t>PARTS</t>
+    <t>y</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Description</t>
   </si>
   <si>
     <t>Qty</t>
   </si>
   <si>
-    <t>USB Keyboard</t>
-  </si>
-  <si>
-    <t>USB Mouse</t>
-  </si>
-  <si>
-    <t>Wireless Mouse</t>
-  </si>
-  <si>
-    <t>Wireless Keyboard/Mouse kit</t>
-  </si>
-  <si>
-    <t>iFixit Moray kit</t>
+    <t>Donated?</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>SATA SSD</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>M2 SSD</t>
+  </si>
+  <si>
+    <t>SODIMM</t>
+  </si>
+  <si>
+    <t>1GB DDR3</t>
+  </si>
+  <si>
+    <t>2GB DDR4</t>
+  </si>
+  <si>
+    <t>2GB DDR3</t>
+  </si>
+  <si>
+    <t>8GB DDR4</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>8GB DDR3</t>
+  </si>
+  <si>
+    <t>4GB DDR4</t>
+  </si>
+  <si>
+    <t>4GB DDR3</t>
+  </si>
+  <si>
+    <t>DIMM</t>
+  </si>
+  <si>
+    <t>16GB DDR4</t>
+  </si>
+  <si>
+    <t>GPU</t>
+  </si>
+  <si>
+    <t>Nvidia P1000</t>
+  </si>
+  <si>
+    <t>TOOLS</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Column2</t>
+  </si>
+  <si>
+    <t>Column3</t>
+  </si>
+  <si>
+    <t>iFixit Moray Kit (complete)</t>
+  </si>
+  <si>
+    <t>Screwdriver Kit</t>
+  </si>
+  <si>
+    <t>iFixit Pro Tech Toolkit (complete)</t>
   </si>
   <si>
     <t>iFixit Project Mat</t>
   </si>
   <si>
-    <t>iFixit Pro Tech Toolkit</t>
-  </si>
-  <si>
-    <t>Cleaning cloths</t>
-  </si>
-  <si>
-    <t>Thermal paste</t>
-  </si>
-  <si>
-    <t>Power Strips</t>
+    <t>Screw Organizer</t>
+  </si>
+  <si>
+    <t>Magnetic Parts Tray</t>
+  </si>
+  <si>
+    <t>Anker Power Strip</t>
+  </si>
+  <si>
+    <t>Power Strip</t>
+  </si>
+  <si>
+    <t>Generic Power Strip</t>
+  </si>
+  <si>
+    <t>USB A to Ethernet</t>
+  </si>
+  <si>
+    <t>Adapter</t>
+  </si>
+  <si>
+    <t>Duster</t>
+  </si>
+  <si>
+    <t>Miscellaneous</t>
+  </si>
+  <si>
+    <t>USB Drive</t>
+  </si>
+  <si>
+    <t>Goo Gone</t>
+  </si>
+  <si>
+    <t>Cleaning Supplies</t>
+  </si>
+  <si>
+    <t>Isopropyl Alcohol</t>
   </si>
   <si>
     <t>Monitors w/ HDMI</t>
@@ -713,106 +806,7 @@
     <t>Monitor Stands</t>
   </si>
   <si>
-    <t>4-in-1 monitor stand with Displayport monitors</t>
-  </si>
-  <si>
-    <t>USB A to Ethernet adapters</t>
-  </si>
-  <si>
-    <t>A3 Mesh bags (not in use)</t>
-  </si>
-  <si>
-    <t>A4 mesh bags (not in use)</t>
-  </si>
-  <si>
-    <t>Duster</t>
-  </si>
-  <si>
-    <t>AUX wired earbuds</t>
-  </si>
-  <si>
-    <t>Super Glue</t>
-  </si>
-  <si>
-    <t>USB drives</t>
-  </si>
-  <si>
-    <t>Sharpies</t>
-  </si>
-  <si>
-    <t>Dry Erase Markers</t>
-  </si>
-  <si>
-    <t>Goo Gone</t>
-  </si>
-  <si>
-    <t>Isopropyl Alcohol</t>
-  </si>
-  <si>
-    <t>Magnetic Parts Trays</t>
-  </si>
-  <si>
-    <t>30 Gallon Trash Bags (20/box)</t>
-  </si>
-  <si>
-    <t>Sandwich bags (200/box)</t>
-  </si>
-  <si>
-    <t>Mickey Mouse Power Cables</t>
-  </si>
-  <si>
-    <t>Ethernet cables</t>
-  </si>
-  <si>
     <t>WiFi Adapters</t>
-  </si>
-  <si>
-    <t>Intel core i7-i8850H</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>SATA SSD</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>SODIMM</t>
-  </si>
-  <si>
-    <t>8GB DDR4</t>
-  </si>
-  <si>
-    <t>2GB DDR3</t>
-  </si>
-  <si>
-    <t>4GB DDR3</t>
-  </si>
-  <si>
-    <t>2GB DDR4</t>
-  </si>
-  <si>
-    <t>8GB DDR3</t>
-  </si>
-  <si>
-    <t>4GB DDR4</t>
-  </si>
-  <si>
-    <t>16GB DDR4</t>
-  </si>
-  <si>
-    <t>1GB DDR3</t>
-  </si>
-  <si>
-    <t>DIMM</t>
-  </si>
-  <si>
-    <t>TOOLS</t>
-  </si>
-  <si>
-    <t>M2 SSD</t>
   </si>
 </sst>
 </file>
@@ -824,7 +818,7 @@
     <numFmt numFmtId="164" formatCode="00000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -955,7 +949,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -999,11 +993,8 @@
     <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1011,11 +1002,40 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="27">
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1069,6 +1089,19 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <fill>
@@ -1147,6 +1180,12 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="00000"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
@@ -1170,39 +1209,6 @@
           <color rgb="FF000000"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="00000"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1231,7 +1237,7 @@
     <tableColumn id="13" xr3:uid="{5BEE40AD-E450-4A13-BFB5-1D0CED084DB3}" name="ID"/>
     <tableColumn id="8" xr3:uid="{E9AB9B46-3541-4715-8E5B-024096D78342}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{F7DAC8DD-8096-40F1-8780-1DB9CB4EC72F}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="26"/>
     <tableColumn id="5" xr3:uid="{5338F6FB-43B0-44AF-AF8B-542FAC6CEDF0}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{64D6C993-8518-4A7C-9BDA-A54D7DBFBA8E}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{E5D987A3-C54A-4907-B710-79DB224E0008}" name="Current Status" totalsRowFunction="count"/>
@@ -1283,7 +1289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="13">
   <autoFilter ref="A2:L33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{73648E04-2EA1-4ADB-8E24-E7DDE01C0462}" name="Item"/>
@@ -1295,8 +1301,8 @@
     <tableColumn id="2" xr3:uid="{C85B34EB-06B2-40A8-BBCB-B5F170EF3F82}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{A686D1B3-031E-4544-A98D-8F3144FA62B0}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{AB29939A-0AF4-4451-A6F4-2144F8957E73}" name="SSD/HDD"/>
-    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="11"/>
     <tableColumn id="12" xr3:uid="{67EC036F-98F6-4C6B-BDD7-99DB9B6ADF97}" name="ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1304,46 +1310,52 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10100501-D05A-423B-A036-4B5D9B2ECD20}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="4">
   <autoFilter ref="A2:M59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{D71C6020-33AC-4F3C-BC88-69BADE52FD9C}" name="Item"/>
-    <tableColumn id="11" xr3:uid="{3694AE3D-BABD-4C86-8092-3A4D6CE18FE9}" name="Type of Device"/>
-    <tableColumn id="3" xr3:uid="{DBF01EDE-E989-4722-BA17-4F2F168FA1B7}" name="Est. Year"/>
-    <tableColumn id="4" xr3:uid="{8A83BF41-D4B3-47AF-9A4E-D470FED11493}" name="CPU"/>
-    <tableColumn id="5" xr3:uid="{5A855548-F141-4612-89D9-87C3C3042FDB}" name="OS"/>
-    <tableColumn id="6" xr3:uid="{7C6B1539-F50D-45A7-A8CD-94746983CE20}" name="RAM Amount"/>
-    <tableColumn id="13" xr3:uid="{D6E0079E-D628-428A-8C40-CC4B7F920E56}" name="RAM Generation"/>
-    <tableColumn id="7" xr3:uid="{7319329B-DA0F-470E-AE1F-CAF023744072}" name="Storage"/>
-    <tableColumn id="8" xr3:uid="{96CAC308-4A56-4EA5-AF3F-FCAC656EEA09}" name="SSD/HDD"/>
-    <tableColumn id="10" xr3:uid="{6EFEA34D-1A93-4407-A41E-DD47A214B1DA}" name="Est. Value" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{04505084-FFBB-491E-B658-CE08D38C3E7B}" name="Notes"/>
-    <tableColumn id="9" xr3:uid="{6814BC74-3E15-43D3-BC09-F23C9C777339}" name="Date Donated" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{45D6EFC2-97A5-4C00-9305-6B4ED43BEBB2}" name="Recipient"/>
+    <tableColumn id="1" xr3:uid="{549BC727-085C-45F5-9520-711A34B50F51}" name="Item"/>
+    <tableColumn id="11" xr3:uid="{3C98AC72-613E-4EC8-8310-F9E3ED18CC90}" name="Type of Device"/>
+    <tableColumn id="3" xr3:uid="{50863EE7-CAD0-400D-9B34-779EE33CD648}" name="Est. Year"/>
+    <tableColumn id="4" xr3:uid="{00F5359B-A50E-41FF-A2BF-D2260FFBD06C}" name="CPU"/>
+    <tableColumn id="5" xr3:uid="{B2D873F2-431E-43E8-96DC-0380E528EA00}" name="OS"/>
+    <tableColumn id="6" xr3:uid="{67FB40A4-BE9A-4206-AF76-C81A6385AAC3}" name="RAM Amount"/>
+    <tableColumn id="13" xr3:uid="{A9DF335A-A163-4AA9-8879-B5B359D716CC}" name="RAM Generation"/>
+    <tableColumn id="7" xr3:uid="{03AC00D8-5308-407D-9BAC-3303A2B380B3}" name="Storage"/>
+    <tableColumn id="8" xr3:uid="{CFFC1B93-1DA0-40C5-BC8E-01F5CAD8DB66}" name="SSD/HDD"/>
+    <tableColumn id="10" xr3:uid="{71AF2E6E-D071-4784-865B-CA65E73CD28D}" name="Est. Value" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{EFA4DB39-7CD3-4AA7-9335-2FEE3F14CF55}" name="Notes"/>
+    <tableColumn id="9" xr3:uid="{2DC095C6-494B-405F-9E1B-C8849C64E6F1}" name="Date Donated" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{77D1B06F-E180-45FD-ACE9-4BA0C5955E95}" name="Recipient"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}" name="Parts" displayName="Parts" ref="A2:C15" totalsRowShown="0">
-  <autoFilter ref="A2:C15" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{AE6A62C8-410E-43CA-9FCC-DB171FCD3CD1}" name="Type"/>
-    <tableColumn id="3" xr3:uid="{8BE6192C-E1B9-4BD5-BEB2-D26E68C58775}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{675E5FD2-430E-4D35-9481-575A83791C4E}" name="Qty"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5027EC0E-CEEE-4641-ADD0-AA27230F7EC3}" name="Parts5" displayName="Parts5" ref="A2:E19" totalsRowShown="0">
+  <autoFilter ref="A2:E19" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{A07F4B01-C838-4D46-AE29-85BAC951AA36}" name="Type"/>
+    <tableColumn id="3" xr3:uid="{9AC978C2-FD83-43AA-9C69-BC026B4E6411}" name="Description"/>
+    <tableColumn id="4" xr3:uid="{9B2129F6-659A-4DD2-94CF-8EC39B827718}" name="Qty"/>
+    <tableColumn id="5" xr3:uid="{C24221AA-BF54-4384-AC51-1C5D1D76BE99}" name="Donated?" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{1B36C5CD-E753-4327-9D04-48D37AAB944F}" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{42D1C34C-9303-4D46-A107-174D17AE2274}" name="Parts5" displayName="Parts5" ref="A2:C34" totalsRowShown="0">
-  <autoFilter ref="A2:C34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{C29E963F-354B-4750-B17F-22461F6DC5F4}" name="Type"/>
-    <tableColumn id="3" xr3:uid="{7C7B0B32-2D9C-4EDB-8E56-4C2ADECB5869}" name="Description"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1921E586-F6B8-46BF-BE64-CE91A4EEE8D6}" name="Parts56" displayName="Parts56" ref="A2:G34" totalsRowShown="0">
+  <autoFilter ref="A2:G34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{C29E963F-354B-4750-B17F-22461F6DC5F4}" name="Name"/>
+    <tableColumn id="3" xr3:uid="{7C7B0B32-2D9C-4EDB-8E56-4C2ADECB5869}" name="Type"/>
     <tableColumn id="2" xr3:uid="{1155C0CA-025A-4922-8B0E-F2A817B3BB60}" name="Qty"/>
+    <tableColumn id="8" xr3:uid="{D743202E-D377-4920-815B-09F9ED9CC36B}" name="Value" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{B4A0A0AC-4FD4-4A43-8591-ABD2EBAA117A}" name="Column1"/>
+    <tableColumn id="5" xr3:uid="{829B96B7-C10C-454A-A528-8575C5865BFA}" name="Column2"/>
+    <tableColumn id="6" xr3:uid="{DDBE87C8-7522-4C92-862B-558811DEBA9D}" name="Column3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1667,33 +1679,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5AA6A1-7D43-4966-8813-F497D895A5C2}">
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="33.33203125" customWidth="1"/>
-    <col min="2" max="2" width="6.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5546875" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="19.44140625" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1725,11 +1737,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="E3" s="1"/>
       <c r="I3" s="16"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1755,11 +1767,11 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="E5" s="1"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1785,7 +1797,7 @@
         <v>45673</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1812,7 +1824,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1836,7 +1848,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1860,7 +1872,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1884,7 +1896,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1908,7 +1920,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1932,7 +1944,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="28.9">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1958,7 +1970,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -1987,7 +1999,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="43.15">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -2013,7 +2025,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -2037,7 +2049,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="28.9">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2063,7 +2075,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -2087,7 +2099,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -2113,7 +2125,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -2137,7 +2149,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="28.9">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2166,11 +2178,11 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9">
       <c r="E22" s="1"/>
       <c r="I22" s="16"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2194,7 +2206,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2218,11 +2230,11 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9">
       <c r="E25" s="1"/>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -2248,7 +2260,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -2272,7 +2284,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -2296,7 +2308,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -2322,34 +2334,34 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:5">
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:5">
       <c r="E34" s="1"/>
     </row>
-    <row r="35" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:5">
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="5:5">
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="5:5">
       <c r="E37" s="1"/>
     </row>
-    <row r="38" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="5:5">
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="5:5">
       <c r="E39" s="1"/>
     </row>
   </sheetData>
@@ -2382,29 +2394,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DEA6183-B753-401C-B21E-C502785DFA3D}">
   <dimension ref="A1:G63"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="33.33203125" customWidth="1"/>
-    <col min="2" max="2" width="7.5546875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5546875" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.28515625" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" style="12" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2427,7 +2439,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
@@ -2448,7 +2460,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
         <v>57</v>
       </c>
@@ -2469,7 +2481,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="15" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>57</v>
       </c>
@@ -2492,7 +2504,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="43.15">
       <c r="A6" s="8" t="s">
         <v>57</v>
       </c>
@@ -2515,7 +2527,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
         <v>57</v>
       </c>
@@ -2536,7 +2548,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="28.9">
       <c r="A8" s="8" t="s">
         <v>57</v>
       </c>
@@ -2559,7 +2571,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
@@ -2580,7 +2592,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7">
       <c r="A10" s="8"/>
       <c r="B10" s="14"/>
       <c r="C10" s="9"/>
@@ -2589,7 +2601,7 @@
       <c r="F10" s="9"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" s="4" t="s">
         <v>57</v>
       </c>
@@ -2610,7 +2622,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="57.6">
       <c r="A12" s="8" t="s">
         <v>61</v>
       </c>
@@ -2633,7 +2645,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7">
       <c r="A13" s="8" t="s">
         <v>61</v>
       </c>
@@ -2656,7 +2668,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7">
       <c r="A14" s="4" t="s">
         <v>61</v>
       </c>
@@ -2677,7 +2689,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7">
       <c r="A15" s="8" t="s">
         <v>61</v>
       </c>
@@ -2698,7 +2710,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7">
       <c r="A16" s="4" t="s">
         <v>61</v>
       </c>
@@ -2719,7 +2731,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7">
       <c r="A17" s="4" t="s">
         <v>61</v>
       </c>
@@ -2740,7 +2752,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7">
       <c r="A18" s="4" t="s">
         <v>61</v>
       </c>
@@ -2761,7 +2773,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7">
       <c r="A19" s="8" t="s">
         <v>61</v>
       </c>
@@ -2782,7 +2794,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7">
       <c r="A20" s="4" t="s">
         <v>61</v>
       </c>
@@ -2803,7 +2815,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7">
       <c r="A21" s="8" t="s">
         <v>61</v>
       </c>
@@ -2824,7 +2836,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
         <v>64</v>
       </c>
@@ -2845,7 +2857,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7">
       <c r="A23" s="8" t="s">
         <v>65</v>
       </c>
@@ -2868,7 +2880,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
         <v>64</v>
       </c>
@@ -2889,7 +2901,7 @@
         <v>46052</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7">
       <c r="A25" s="8" t="s">
         <v>64</v>
       </c>
@@ -2908,7 +2920,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7">
       <c r="A26" s="4"/>
       <c r="B26" s="13"/>
       <c r="C26" s="5"/>
@@ -2917,7 +2929,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7">
       <c r="A27" s="8" t="s">
         <v>64</v>
       </c>
@@ -2940,7 +2952,7 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7">
       <c r="A28" s="4" t="s">
         <v>68</v>
       </c>
@@ -2961,7 +2973,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7">
       <c r="A29" s="8" t="s">
         <v>69</v>
       </c>
@@ -2984,7 +2996,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7">
       <c r="A30" s="8" t="s">
         <v>71</v>
       </c>
@@ -3007,7 +3019,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7">
       <c r="A31" s="8" t="s">
         <v>73</v>
       </c>
@@ -3028,7 +3040,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7">
       <c r="A32" s="8" t="s">
         <v>74</v>
       </c>
@@ -3049,7 +3061,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7">
       <c r="A33" s="8" t="s">
         <v>75</v>
       </c>
@@ -3070,7 +3082,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7">
       <c r="A34" s="8" t="s">
         <v>73</v>
       </c>
@@ -3091,7 +3103,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7">
       <c r="A35" s="8" t="s">
         <v>76</v>
       </c>
@@ -3112,7 +3124,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -3135,7 +3147,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>64</v>
       </c>
@@ -3158,7 +3170,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -3178,7 +3190,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -3198,7 +3210,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>64</v>
       </c>
@@ -3221,7 +3233,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -3244,10 +3256,10 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7">
       <c r="G42" s="16"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -3267,7 +3279,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>81</v>
       </c>
@@ -3287,7 +3299,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>81</v>
       </c>
@@ -3307,7 +3319,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>86</v>
       </c>
@@ -3330,7 +3342,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -3353,7 +3365,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -3373,7 +3385,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
         <v>89</v>
       </c>
@@ -3390,7 +3402,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>91</v>
       </c>
@@ -3410,7 +3422,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>92</v>
       </c>
@@ -3430,7 +3442,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>93</v>
       </c>
@@ -3450,7 +3462,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
         <v>94</v>
       </c>
@@ -3473,7 +3485,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>97</v>
       </c>
@@ -3493,7 +3505,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -3516,7 +3528,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>100</v>
       </c>
@@ -3536,7 +3548,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>91</v>
       </c>
@@ -3556,7 +3568,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -3576,7 +3588,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -3599,16 +3611,16 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7">
       <c r="G60" s="16"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7">
       <c r="G61" s="16"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7">
       <c r="G62" s="16"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7">
       <c r="G63" s="16"/>
     </row>
   </sheetData>
@@ -3616,10 +3628,10 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:G63">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3638,33 +3650,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F948288C-1730-49D1-BD4C-FC704F167D22}">
   <dimension ref="A1:I33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="33.33203125" customWidth="1"/>
-    <col min="2" max="2" width="6.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5546875" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5703125" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:9">
+      <c r="A1" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -3693,7 +3705,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>103</v>
       </c>
@@ -3722,7 +3734,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>103</v>
       </c>
@@ -3751,91 +3763,91 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9">
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9">
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9">
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9">
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9">
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9">
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9">
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9">
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9">
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9">
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9">
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9">
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:5">
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:5">
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:5">
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:5">
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:5">
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:5">
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:5">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="5:5">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="5:5">
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="5:5">
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="5:5">
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="5:5">
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="5:5">
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="5:5">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="5:5">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="5:5">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:5">
       <c r="E33" s="1"/>
     </row>
   </sheetData>
@@ -3867,38 +3879,38 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE86381-3E33-4CB8-A62B-E48A74AB9667}">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.28515625" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="17.109375" customWidth="1"/>
-    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.109375" customWidth="1"/>
-    <col min="10" max="10" width="18.6640625" style="19" customWidth="1"/>
-    <col min="11" max="11" width="21.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="19" customWidth="1"/>
+    <col min="11" max="11" width="21.28515625" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:12" ht="14.45">
+      <c r="A1" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-    </row>
-    <row r="2" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+    </row>
+    <row r="2" spans="1:12" ht="14.45">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -3936,7 +3948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="14.45">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -3972,7 +3984,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="14.45">
       <c r="A4" t="s">
         <v>125</v>
       </c>
@@ -4008,7 +4020,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="14.45">
       <c r="A5" t="s">
         <v>128</v>
       </c>
@@ -4044,10 +4056,10 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="14.45">
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="14.45">
       <c r="A7" t="s">
         <v>128</v>
       </c>
@@ -4083,7 +4095,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="14.45">
       <c r="A8" t="s">
         <v>84</v>
       </c>
@@ -4119,7 +4131,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="14.45">
       <c r="A9" t="s">
         <v>133</v>
       </c>
@@ -4155,10 +4167,10 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="14.45">
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="14.45">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -4194,7 +4206,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="14.45">
       <c r="A12" t="s">
         <v>138</v>
       </c>
@@ -4229,7 +4241,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="14.45">
       <c r="A13" t="s">
         <v>140</v>
       </c>
@@ -4265,7 +4277,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="15" customHeight="1">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -4301,7 +4313,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="15" customHeight="1">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -4337,7 +4349,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="15" customHeight="1">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -4373,7 +4385,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="15" customHeight="1">
       <c r="A17" t="s">
         <v>146</v>
       </c>
@@ -4409,7 +4421,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="15" customHeight="1">
       <c r="A18" t="s">
         <v>149</v>
       </c>
@@ -4445,7 +4457,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="15" customHeight="1">
       <c r="A19" t="s">
         <v>149</v>
       </c>
@@ -4481,7 +4493,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="15" customHeight="1">
       <c r="A20" t="s">
         <v>151</v>
       </c>
@@ -4517,7 +4529,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="15" customHeight="1">
       <c r="A21" t="s">
         <v>151</v>
       </c>
@@ -4553,7 +4565,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="15" customHeight="1">
       <c r="A22" t="s">
         <v>61</v>
       </c>
@@ -4589,7 +4601,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="15" customHeight="1">
       <c r="A23" t="s">
         <v>154</v>
       </c>
@@ -4625,7 +4637,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="15" customHeight="1">
       <c r="A24" t="s">
         <v>57</v>
       </c>
@@ -4661,7 +4673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="15" customHeight="1">
       <c r="A25" t="s">
         <v>128</v>
       </c>
@@ -4697,7 +4709,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="15" customHeight="1">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -4733,7 +4745,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="15" customHeight="1">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -4769,7 +4781,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="15" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>64</v>
       </c>
@@ -4805,7 +4817,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" ht="15" customHeight="1">
       <c r="A29" t="s">
         <v>159</v>
       </c>
@@ -4841,16 +4853,16 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" ht="15" customHeight="1">
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="15" customHeight="1">
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="15" customHeight="1">
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="11:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="11:11" ht="15" customHeight="1">
       <c r="K33" s="1"/>
     </row>
   </sheetData>
@@ -4858,36 +4870,36 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="A27:A28">
-    <cfRule type="expression" dxfId="13" priority="17">
+    <cfRule type="expression" dxfId="21" priority="17">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="18">
+    <cfRule type="expression" dxfId="20" priority="18">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:K9 A11:K14 A15:C15 E15:K15 A16:K25">
-    <cfRule type="expression" dxfId="11" priority="21">
+    <cfRule type="expression" dxfId="19" priority="21">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:L9 A11:L14 A15:C15 E15:L15 A16:L25">
-    <cfRule type="expression" dxfId="10" priority="22">
+    <cfRule type="expression" dxfId="18" priority="22">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G26:G29">
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="17" priority="9">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="16" priority="10">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26:H29">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4908,28 +4920,28 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19592962-4FD3-47C5-914B-6346C180BC2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1C144A-BB57-4446-B714-000D1D9FAB4A}">
   <dimension ref="A1:O59"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.33203125" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="16" customWidth="1"/>
-    <col min="13" max="13" width="29.109375" customWidth="1"/>
-    <col min="14" max="14" width="27.6640625" customWidth="1"/>
-    <col min="15" max="15" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="16" customWidth="1"/>
+    <col min="13" max="13" width="29.140625" customWidth="1"/>
+    <col min="14" max="14" width="27.7109375" customWidth="1"/>
+    <col min="15" max="15" width="28.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15" customHeight="1">
       <c r="B1" s="17" t="s">
         <v>161</v>
       </c>
@@ -4951,7 +4963,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="14.45">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -5000,7 +5012,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="14.45">
       <c r="A3" t="s">
         <v>166</v>
       </c>
@@ -5009,18 +5021,6 @@
       </c>
       <c r="C3">
         <v>2019</v>
-      </c>
-      <c r="D3" t="s">
-        <v>241</v>
-      </c>
-      <c r="E3" t="s">
-        <v>137</v>
-      </c>
-      <c r="F3">
-        <v>8</v>
-      </c>
-      <c r="G3" t="s">
-        <v>130</v>
       </c>
       <c r="H3">
         <v>256</v>
@@ -5039,7 +5039,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="14.45">
       <c r="A4" t="s">
         <v>166</v>
       </c>
@@ -5048,18 +5048,6 @@
       </c>
       <c r="C4">
         <v>2019</v>
-      </c>
-      <c r="D4" t="s">
-        <v>241</v>
-      </c>
-      <c r="E4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F4">
-        <v>8</v>
-      </c>
-      <c r="G4" t="s">
-        <v>130</v>
       </c>
       <c r="H4">
         <v>256</v>
@@ -5078,7 +5066,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="14.45">
       <c r="A5" t="s">
         <v>166</v>
       </c>
@@ -5087,18 +5075,6 @@
       </c>
       <c r="C5">
         <v>2019</v>
-      </c>
-      <c r="D5" t="s">
-        <v>241</v>
-      </c>
-      <c r="E5" t="s">
-        <v>137</v>
-      </c>
-      <c r="F5">
-        <v>8</v>
-      </c>
-      <c r="G5" t="s">
-        <v>130</v>
       </c>
       <c r="H5">
         <v>256</v>
@@ -5117,7 +5093,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="14.45">
       <c r="A6" t="s">
         <v>166</v>
       </c>
@@ -5126,18 +5102,6 @@
       </c>
       <c r="C6">
         <v>2019</v>
-      </c>
-      <c r="D6" t="s">
-        <v>241</v>
-      </c>
-      <c r="E6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F6">
-        <v>8</v>
-      </c>
-      <c r="G6" t="s">
-        <v>130</v>
       </c>
       <c r="H6">
         <v>256</v>
@@ -5156,7 +5120,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="14.45">
       <c r="A7" t="s">
         <v>166</v>
       </c>
@@ -5165,18 +5129,6 @@
       </c>
       <c r="C7">
         <v>2019</v>
-      </c>
-      <c r="D7" t="s">
-        <v>241</v>
-      </c>
-      <c r="E7" t="s">
-        <v>137</v>
-      </c>
-      <c r="F7">
-        <v>8</v>
-      </c>
-      <c r="G7" t="s">
-        <v>130</v>
       </c>
       <c r="H7">
         <v>256</v>
@@ -5195,7 +5147,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="14.45">
       <c r="A8" t="s">
         <v>166</v>
       </c>
@@ -5204,18 +5156,6 @@
       </c>
       <c r="C8">
         <v>2019</v>
-      </c>
-      <c r="D8" t="s">
-        <v>241</v>
-      </c>
-      <c r="E8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F8">
-        <v>8</v>
-      </c>
-      <c r="G8" t="s">
-        <v>130</v>
       </c>
       <c r="H8">
         <v>256</v>
@@ -5234,7 +5174,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="14.45">
       <c r="A9" t="s">
         <v>166</v>
       </c>
@@ -5243,18 +5183,6 @@
       </c>
       <c r="C9">
         <v>2019</v>
-      </c>
-      <c r="D9" t="s">
-        <v>241</v>
-      </c>
-      <c r="E9" t="s">
-        <v>137</v>
-      </c>
-      <c r="F9">
-        <v>8</v>
-      </c>
-      <c r="G9" t="s">
-        <v>130</v>
       </c>
       <c r="H9">
         <v>256</v>
@@ -5273,7 +5201,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="14.45">
       <c r="A10" t="s">
         <v>168</v>
       </c>
@@ -5312,7 +5240,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="14.45">
       <c r="A11" t="s">
         <v>170</v>
       </c>
@@ -5351,7 +5279,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="14.45">
       <c r="A12" t="s">
         <v>172</v>
       </c>
@@ -5392,7 +5320,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="14.45">
       <c r="A13" t="s">
         <v>175</v>
       </c>
@@ -5431,7 +5359,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="14.45">
       <c r="A14" t="s">
         <v>168</v>
       </c>
@@ -5470,7 +5398,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="14.45">
       <c r="A15" t="s">
         <v>177</v>
       </c>
@@ -5509,7 +5437,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="14.45">
       <c r="A16" t="s">
         <v>179</v>
       </c>
@@ -5550,7 +5478,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="14.45">
       <c r="A17" t="s">
         <v>186</v>
       </c>
@@ -5591,7 +5519,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="14.45">
       <c r="A18" t="s">
         <v>187</v>
       </c>
@@ -5632,7 +5560,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="14.45">
       <c r="A19" t="s">
         <v>64</v>
       </c>
@@ -5673,7 +5601,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="28.9">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -5714,7 +5642,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="14.45">
       <c r="A21" t="s">
         <v>196</v>
       </c>
@@ -5753,7 +5681,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="14.45">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -5792,7 +5720,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="14.45">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -5831,7 +5759,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="14.45">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -5870,7 +5798,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" ht="14.45">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -5909,7 +5837,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" ht="14.45">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -5948,7 +5876,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" ht="14.45">
       <c r="A27" t="s">
         <v>61</v>
       </c>
@@ -5987,7 +5915,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" ht="14.45">
       <c r="A28" t="s">
         <v>199</v>
       </c>
@@ -6026,7 +5954,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" ht="14.45">
       <c r="A29" t="s">
         <v>199</v>
       </c>
@@ -6065,7 +5993,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" ht="14.45">
       <c r="A30" t="s">
         <v>128</v>
       </c>
@@ -6104,7 +6032,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" ht="14.45">
       <c r="A31" s="8" t="s">
         <v>61</v>
       </c>
@@ -6143,7 +6071,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" ht="14.45">
       <c r="A32" t="s">
         <v>61</v>
       </c>
@@ -6181,7 +6109,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" ht="14.45">
       <c r="A33" t="s">
         <v>61</v>
       </c>
@@ -6219,7 +6147,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" ht="14.45">
       <c r="A34" t="s">
         <v>203</v>
       </c>
@@ -6257,7 +6185,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" ht="14.45">
       <c r="A35" t="s">
         <v>203</v>
       </c>
@@ -6295,7 +6223,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" ht="14.45">
       <c r="A36" t="s">
         <v>203</v>
       </c>
@@ -6333,7 +6261,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" ht="14.45">
       <c r="A37" t="s">
         <v>203</v>
       </c>
@@ -6371,7 +6299,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="14.45">
       <c r="A38" t="s">
         <v>203</v>
       </c>
@@ -6409,7 +6337,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" ht="14.45">
       <c r="A39" t="s">
         <v>203</v>
       </c>
@@ -6447,7 +6375,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" ht="15" customHeight="1">
       <c r="A40" t="s">
         <v>203</v>
       </c>
@@ -6485,7 +6413,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" ht="15" customHeight="1">
       <c r="A41" t="s">
         <v>203</v>
       </c>
@@ -6523,7 +6451,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" ht="15" customHeight="1">
       <c r="A42" t="s">
         <v>203</v>
       </c>
@@ -6561,7 +6489,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" ht="15" customHeight="1">
       <c r="A43" t="s">
         <v>140</v>
       </c>
@@ -6600,7 +6528,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" ht="15" customHeight="1">
       <c r="A44" s="4" t="s">
         <v>61</v>
       </c>
@@ -6639,94 +6567,94 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" ht="15" customHeight="1">
       <c r="L45" s="15"/>
     </row>
-    <row r="46" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" ht="15" customHeight="1">
       <c r="L46" s="15"/>
     </row>
-    <row r="47" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" ht="15" customHeight="1">
       <c r="L47" s="15"/>
     </row>
-    <row r="48" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" ht="15" customHeight="1">
       <c r="L48" s="15"/>
     </row>
-    <row r="49" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="12:12" ht="15" customHeight="1">
       <c r="L49" s="15"/>
     </row>
-    <row r="50" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="12:12" ht="15" customHeight="1">
       <c r="L50" s="15"/>
     </row>
-    <row r="51" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="12:12" ht="15" customHeight="1">
       <c r="L51" s="15"/>
     </row>
-    <row r="52" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="12:12" ht="15" customHeight="1">
       <c r="L52" s="15"/>
     </row>
-    <row r="53" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="12:12" ht="15" customHeight="1">
       <c r="L53" s="15"/>
     </row>
-    <row r="54" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="12:12" ht="15" customHeight="1">
       <c r="L54" s="15"/>
     </row>
-    <row r="55" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="12:12" ht="15" customHeight="1">
       <c r="L55" s="15"/>
     </row>
-    <row r="56" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="12:12" ht="15" customHeight="1">
       <c r="L56" s="15"/>
     </row>
-    <row r="57" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="12:12" ht="15" customHeight="1">
       <c r="L57" s="15"/>
     </row>
-    <row r="58" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="12:12" ht="15" customHeight="1">
       <c r="L58" s="15"/>
     </row>
-    <row r="59" spans="12:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="12:12" ht="15" customHeight="1">
       <c r="L59" s="15"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A44:F44 H44:K44">
-    <cfRule type="expression" dxfId="5" priority="15">
+    <cfRule type="expression" dxfId="10" priority="5">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A44:F44 H44:L44">
-    <cfRule type="expression" dxfId="4" priority="16">
+    <cfRule type="expression" dxfId="9" priority="6">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:M9 A10:G15 I10:M15 A16:M43 M44 A45:M59">
-    <cfRule type="expression" priority="17">
+    <cfRule type="expression" priority="7">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="18">
+    <cfRule type="expression" dxfId="8" priority="8">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G44">
-    <cfRule type="expression" priority="13">
+    <cfRule type="expression" priority="3">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="14">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H15">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B17 B19 B21:B29 B31:B42" xr:uid="{1DFA3251-7984-4A3C-A048-50097DB9AAD3}">
-      <formula1>"Desktop,Laptop,Tablet,All-In-One"</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1 L1:L42 L45:L1048576" xr:uid="{A67DFFE0-1B96-49B5-A6E2-5C17E92A136C}"/>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K32:K42" xr:uid="{BD4480FF-AB8D-4446-AB7A-01C4C2A99ADB}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K32:K42" xr:uid="{9E34EFD6-6288-43CE-B05D-35BC10E05685}">
       <formula1>1</formula1>
       <formula2>2000</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1 L1:L42 L45:L1048576" xr:uid="{A9EBE1C3-8923-4578-8214-596FAC33FDB8}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B17 B19 B21:B29 B31:B42" xr:uid="{C7FD23E6-3E08-4DF7-8556-C07E455C4835}">
+      <formula1>"Desktop,Laptop,Tablet,All-In-One"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6737,173 +6665,287 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66F9EB6D-6D2E-43F3-A79F-D2A5CF3A037E}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6146040A-3AF4-440D-9E03-57379B2EC394}">
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>242</v>
+        <v>208</v>
       </c>
       <c r="B2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+      <c r="C2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="C3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E3" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>215</v>
       </c>
       <c r="C4">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E4" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B5" t="s">
-        <v>253</v>
+        <v>217</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E5" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B6" t="s">
-        <v>249</v>
+        <v>218</v>
       </c>
       <c r="C6">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B7" t="s">
-        <v>247</v>
+        <v>219</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B8" t="s">
-        <v>246</v>
+        <v>220</v>
       </c>
       <c r="C8">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="E8" s="2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B9" t="s">
-        <v>250</v>
+        <v>222</v>
       </c>
       <c r="C9">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="E9" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B10" t="s">
-        <v>251</v>
+        <v>223</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E10" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>245</v>
+        <v>216</v>
       </c>
       <c r="B11" t="s">
-        <v>248</v>
+        <v>224</v>
       </c>
       <c r="C11">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E11" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="B12" t="s">
-        <v>246</v>
+        <v>220</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E12" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="B13" t="s">
-        <v>250</v>
+        <v>222</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E13" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="B14" t="s">
-        <v>252</v>
+        <v>226</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E14" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>254</v>
+        <v>225</v>
       </c>
       <c r="B15" t="s">
-        <v>248</v>
+        <v>224</v>
       </c>
       <c r="C15">
         <v>11</v>
       </c>
+      <c r="D15" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E15" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" customHeight="1">
+      <c r="A16" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="E16" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="4:4" ht="15" customHeight="1">
+      <c r="D17" s="23"/>
+    </row>
+    <row r="18" spans="4:4" ht="15" customHeight="1">
+      <c r="D18" s="23"/>
+    </row>
+    <row r="19" spans="4:4" ht="15" customHeight="1">
+      <c r="D19" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -6913,286 +6955,222 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6AEFF60-27EE-498D-A491-C67356035C05}">
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3F77F78-0898-4060-A2C7-C1A84336B28A}">
+  <dimension ref="A1:G34"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" customWidth="1"/>
+    <col min="1" max="1" width="33.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="19" customWidth="1"/>
+    <col min="5" max="5" width="41.5703125" customWidth="1"/>
+    <col min="6" max="6" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15">
+      <c r="A1" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="28"/>
+    </row>
+    <row r="2" spans="1:7" ht="15">
       <c r="A2" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="B2" t="s">
-        <v>244</v>
+        <v>208</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>210</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>233</v>
+      </c>
+      <c r="B3" t="s">
+        <v>234</v>
       </c>
       <c r="C3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>235</v>
+      </c>
+      <c r="B4" t="s">
+        <v>234</v>
       </c>
       <c r="C4">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15">
       <c r="A5" t="s">
-        <v>211</v>
+        <v>236</v>
+      </c>
+      <c r="B5" t="s">
+        <v>237</v>
       </c>
       <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15">
       <c r="A6" t="s">
-        <v>212</v>
+        <v>238</v>
+      </c>
+      <c r="B6" t="s">
+        <v>237</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="15">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>239</v>
+      </c>
+      <c r="B7" t="s">
+        <v>240</v>
       </c>
       <c r="C7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15">
       <c r="A8" t="s">
-        <v>214</v>
+        <v>241</v>
+      </c>
+      <c r="B8" t="s">
+        <v>240</v>
       </c>
       <c r="C8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15">
       <c r="A9" t="s">
-        <v>215</v>
+        <v>242</v>
+      </c>
+      <c r="B9" t="s">
+        <v>243</v>
       </c>
       <c r="C9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" t="s">
+        <v>245</v>
+      </c>
+      <c r="C10">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>216</v>
-      </c>
-      <c r="C10">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="15">
       <c r="A11" t="s">
-        <v>217</v>
+        <v>246</v>
+      </c>
+      <c r="B11" t="s">
+        <v>245</v>
       </c>
       <c r="C11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" t="s">
+        <v>247</v>
+      </c>
+      <c r="B12" t="s">
+        <v>248</v>
+      </c>
+      <c r="C12">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>218</v>
-      </c>
-      <c r="C12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="15">
       <c r="A13" t="s">
-        <v>219</v>
+        <v>249</v>
+      </c>
+      <c r="B13" t="s">
+        <v>248</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>220</v>
-      </c>
-      <c r="C14">
+      <c r="E13" t="s">
+        <v>250</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="E14" t="s">
+        <v>251</v>
+      </c>
+      <c r="G14">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>221</v>
-      </c>
-      <c r="C15">
+    <row r="15" spans="1:7" ht="15">
+      <c r="E15" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>222</v>
-      </c>
-      <c r="C16">
+    <row r="16" spans="1:7" ht="15">
+      <c r="E16" t="s">
+        <v>253</v>
+      </c>
+      <c r="G16">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>223</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>224</v>
-      </c>
-      <c r="C18">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>225</v>
-      </c>
-      <c r="C19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>226</v>
-      </c>
-      <c r="C20">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>227</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>228</v>
-      </c>
-      <c r="C22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>229</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>230</v>
-      </c>
-      <c r="C24">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>231</v>
-      </c>
-      <c r="C25">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>232</v>
-      </c>
-      <c r="C26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>233</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>234</v>
-      </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>235</v>
-      </c>
-      <c r="C29">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>236</v>
-      </c>
-      <c r="C30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>237</v>
-      </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>238</v>
-      </c>
-      <c r="C32">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>239</v>
-      </c>
-      <c r="C33">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>240</v>
-      </c>
-      <c r="C34">
+    <row r="17" ht="15"/>
+    <row r="18" ht="15"/>
+    <row r="19" ht="15"/>
+    <row r="20" ht="15"/>
+    <row r="21" ht="15"/>
+    <row r="22" ht="15"/>
+    <row r="23" ht="15"/>
+    <row r="24" ht="15"/>
+    <row r="25" ht="15"/>
+    <row r="26" ht="15"/>
+    <row r="27" ht="15"/>
+    <row r="28" ht="15"/>
+    <row r="29" ht="15"/>
+    <row r="30" ht="15"/>
+    <row r="31" ht="15"/>
+    <row r="32" ht="15"/>
+    <row r="33" spans="5:7" ht="15"/>
+    <row r="34" spans="5:7" ht="15">
+      <c r="E34" t="s">
+        <v>254</v>
+      </c>
+      <c r="G34">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated OldInventorySystem to cleaned version
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/lucasja_rose-hulman_edu/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3460" documentId="8_{A0F2C8DF-695D-4A53-BA74-C2F5D1F57A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73C00331-DB68-481F-98A9-F3303D7051BD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97CF21FA-E5B5-40B6-91B6-79617555DD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="4" activeTab="5" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="4" activeTab="6" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="249">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -737,12 +737,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Column2</t>
-  </si>
-  <si>
-    <t>Column3</t>
-  </si>
-  <si>
     <t>iFixit Moray Kit (complete)</t>
   </si>
   <si>
@@ -752,7 +746,7 @@
     <t>iFixit Pro Tech Toolkit (complete)</t>
   </si>
   <si>
-    <t>iFixit Project Mat</t>
+    <t>iFixit Magnetic Screw Organizer</t>
   </si>
   <si>
     <t>Screw Organizer</t>
@@ -794,19 +788,7 @@
     <t>Isopropyl Alcohol</t>
   </si>
   <si>
-    <t>Monitors w/ HDMI</t>
-  </si>
-  <si>
-    <t>Monitors w/ No HDMI but DisplayPort</t>
-  </si>
-  <si>
-    <t>Monitors w/No HDMI and no DisplayPort</t>
-  </si>
-  <si>
-    <t>Monitor Stands</t>
-  </si>
-  <si>
-    <t>WiFi Adapters</t>
+    <t>USB Wifi Adapter</t>
   </si>
 </sst>
 </file>
@@ -1346,16 +1328,13 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1921E586-F6B8-46BF-BE64-CE91A4EEE8D6}" name="Parts56" displayName="Parts56" ref="A2:G34" totalsRowShown="0">
-  <autoFilter ref="A2:G34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1921E586-F6B8-46BF-BE64-CE91A4EEE8D6}" name="Parts56" displayName="Parts56" ref="A2:D34" totalsRowShown="0">
+  <autoFilter ref="A2:D34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{C29E963F-354B-4750-B17F-22461F6DC5F4}" name="Name"/>
     <tableColumn id="3" xr3:uid="{7C7B0B32-2D9C-4EDB-8E56-4C2ADECB5869}" name="Type"/>
     <tableColumn id="2" xr3:uid="{1155C0CA-025A-4922-8B0E-F2A817B3BB60}" name="Qty"/>
     <tableColumn id="8" xr3:uid="{D743202E-D377-4920-815B-09F9ED9CC36B}" name="Value" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{B4A0A0AC-4FD4-4A43-8591-ABD2EBAA117A}" name="Column1"/>
-    <tableColumn id="5" xr3:uid="{829B96B7-C10C-454A-A528-8575C5865BFA}" name="Column2"/>
-    <tableColumn id="6" xr3:uid="{DDBE87C8-7522-4C92-862B-558811DEBA9D}" name="Column3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6956,18 +6935,16 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3F77F78-0898-4060-A2C7-C1A84336B28A}">
-  <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="33.140625" customWidth="1"/>
     <col min="2" max="2" width="15.28515625" customWidth="1"/>
     <col min="3" max="3" width="10.140625" customWidth="1"/>
     <col min="4" max="4" width="10.140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="41.5703125" customWidth="1"/>
-    <col min="6" max="6" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15">
+    <row r="1" spans="1:4">
       <c r="A1" s="26" t="s">
         <v>229</v>
       </c>
@@ -6975,7 +6952,7 @@
       <c r="C1" s="27"/>
       <c r="D1" s="28"/>
     </row>
-    <row r="2" spans="1:7" ht="15">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>230</v>
       </c>
@@ -6988,192 +6965,195 @@
       <c r="D2" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>231</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B3" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15">
-      <c r="A3" t="s">
-        <v>233</v>
-      </c>
-      <c r="B3" t="s">
-        <v>234</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="15">
+      <c r="D3" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="15">
+      <c r="D4" s="19">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="15">
+      <c r="D5" s="19">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="15">
+      <c r="D6" s="19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="15">
+      <c r="D7" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="15">
+      <c r="D8" s="19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B9" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C9">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="15">
+      <c r="D9" s="19">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="15">
+      <c r="D10" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B11" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C11">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="15">
+      <c r="D11" s="19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B12" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="15">
+      <c r="D12" s="19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B13" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="E13" t="s">
-        <v>250</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="15">
-      <c r="E14" t="s">
-        <v>251</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15">
-      <c r="E15" t="s">
-        <v>252</v>
-      </c>
-      <c r="G15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="15">
-      <c r="E16" t="s">
-        <v>253</v>
-      </c>
-      <c r="G16">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" ht="15"/>
-    <row r="18" ht="15"/>
-    <row r="19" ht="15"/>
-    <row r="20" ht="15"/>
-    <row r="21" ht="15"/>
-    <row r="22" ht="15"/>
-    <row r="23" ht="15"/>
-    <row r="24" ht="15"/>
-    <row r="25" ht="15"/>
-    <row r="26" ht="15"/>
-    <row r="27" ht="15"/>
-    <row r="28" ht="15"/>
-    <row r="29" ht="15"/>
-    <row r="30" ht="15"/>
-    <row r="31" ht="15"/>
-    <row r="32" ht="15"/>
-    <row r="33" spans="5:7" ht="15"/>
-    <row r="34" spans="5:7" ht="15">
-      <c r="E34" t="s">
-        <v>254</v>
-      </c>
-      <c r="G34">
+      <c r="D13" s="19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>248</v>
+      </c>
+      <c r="B14" t="s">
+        <v>241</v>
+      </c>
+      <c r="C14">
         <v>6</v>
       </c>
-    </row>
+      <c r="D14" s="19">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4"/>
+    <row r="16" spans="1:4"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
sprocs to import party, organization, persons -- connectivity not built yet
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/lucasja_rose-hulman_edu/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97CF21FA-E5B5-40B6-91B6-79617555DD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3566" documentId="8_{A0F2C8DF-695D-4A53-BA74-C2F5D1F57A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A467ED7A-F1D3-41C0-9B3D-00F5C1CAE948}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="4" activeTab="6" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="250">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -789,6 +789,9 @@
   </si>
   <si>
     <t>USB Wifi Adapter</t>
+  </si>
+  <si>
+    <t>Org?</t>
   </si>
 </sst>
 </file>
@@ -800,7 +803,7 @@
     <numFmt numFmtId="164" formatCode="00000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -978,10 +981,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -990,33 +990,26 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="28">
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -1046,16 +1039,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="4" tint="0.79998168889431442"/>
@@ -1071,19 +1054,6 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -1162,12 +1132,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="00000"/>
-    </dxf>
-    <dxf>
       <font>
         <color theme="1"/>
       </font>
@@ -1193,7 +1157,50 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="00000"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1238,7 +1245,7 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F96A3CC8-25D1-4CF8-877D-2816B26B7DC4}" name="Item Name" totalsRowLabel="Total"/>
-    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="25"/>
     <tableColumn id="8" xr3:uid="{7D8F815E-A974-42A8-AC0B-AB8B951599A2}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{FEA94C75-B538-448A-A9F5-46F5A27E863D}" name="Year released"/>
     <tableColumn id="4" xr3:uid="{24998D92-36B7-4553-81E7-CB33711B31BB}" name="Special Reqs/Notes"/>
@@ -1260,7 +1267,7 @@
     <tableColumn id="13" xr3:uid="{EFFF3477-1A58-41CD-BFF3-45CE299505A7}" name="ID"/>
     <tableColumn id="8" xr3:uid="{C694899F-E385-4DE2-972A-7395A9633019}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{13C54556-A90A-4F9C-800D-3D838462DF46}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="24"/>
     <tableColumn id="5" xr3:uid="{6DE19FBC-9BD8-456E-9FC5-F633F61E4A34}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{68546225-0A78-43C1-A4F9-4D2E1DC008A3}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{0D7FD365-4F73-4A57-B8A1-CFAC47267923}" name="Current Status" totalsRowFunction="count"/>
@@ -1271,7 +1278,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:L33" totalsRowShown="0" tableBorderDxfId="23">
   <autoFilter ref="A2:L33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{73648E04-2EA1-4ADB-8E24-E7DDE01C0462}" name="Item"/>
@@ -1283,8 +1290,8 @@
     <tableColumn id="2" xr3:uid="{C85B34EB-06B2-40A8-BBCB-B5F170EF3F82}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{A686D1B3-031E-4544-A98D-8F3144FA62B0}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{AB29939A-0AF4-4451-A6F4-2144F8957E73}" name="SSD/HDD"/>
-    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="21"/>
     <tableColumn id="12" xr3:uid="{67EC036F-98F6-4C6B-BDD7-99DB9B6ADF97}" name="ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1292,9 +1299,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10100501-D05A-423B-A036-4B5D9B2ECD20}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:M59" totalsRowShown="0" tableBorderDxfId="4">
-  <autoFilter ref="A2:M59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10100501-D05A-423B-A036-4B5D9B2ECD20}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:N59" totalsRowShown="0" tableBorderDxfId="20">
+  <autoFilter ref="A2:N59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{549BC727-085C-45F5-9520-711A34B50F51}" name="Item"/>
     <tableColumn id="11" xr3:uid="{3C98AC72-613E-4EC8-8310-F9E3ED18CC90}" name="Type of Device"/>
     <tableColumn id="3" xr3:uid="{50863EE7-CAD0-400D-9B34-779EE33CD648}" name="Est. Year"/>
@@ -1304,10 +1311,11 @@
     <tableColumn id="13" xr3:uid="{A9DF335A-A163-4AA9-8879-B5B359D716CC}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{03AC00D8-5308-407D-9BAC-3303A2B380B3}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{CFFC1B93-1DA0-40C5-BC8E-01F5CAD8DB66}" name="SSD/HDD"/>
-    <tableColumn id="10" xr3:uid="{71AF2E6E-D071-4784-865B-CA65E73CD28D}" name="Est. Value" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{71AF2E6E-D071-4784-865B-CA65E73CD28D}" name="Est. Value" dataDxfId="19"/>
     <tableColumn id="12" xr3:uid="{EFA4DB39-7CD3-4AA7-9335-2FEE3F14CF55}" name="Notes"/>
-    <tableColumn id="9" xr3:uid="{2DC095C6-494B-405F-9E1B-C8849C64E6F1}" name="Date Donated" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{77D1B06F-E180-45FD-ACE9-4BA0C5955E95}" name="Recipient"/>
+    <tableColumn id="9" xr3:uid="{2DC095C6-494B-405F-9E1B-C8849C64E6F1}" name="Date Donated" dataDxfId="18"/>
+    <tableColumn id="14" xr3:uid="{4D76F748-9FDA-4C94-B04F-D8250CE6CE08}" name="Recipient" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{77D1B06F-E180-45FD-ACE9-4BA0C5955E95}" name="Org?"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1320,7 +1328,7 @@
     <tableColumn id="1" xr3:uid="{A07F4B01-C838-4D46-AE29-85BAC951AA36}" name="Type"/>
     <tableColumn id="3" xr3:uid="{9AC978C2-FD83-43AA-9C69-BC026B4E6411}" name="Description"/>
     <tableColumn id="4" xr3:uid="{9B2129F6-659A-4DD2-94CF-8EC39B827718}" name="Qty"/>
-    <tableColumn id="5" xr3:uid="{C24221AA-BF54-4384-AC51-1C5D1D76BE99}" name="Donated?" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C24221AA-BF54-4384-AC51-1C5D1D76BE99}" name="Donated?" dataDxfId="17"/>
     <tableColumn id="2" xr3:uid="{1B36C5CD-E753-4327-9D04-48D37AAB944F}" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1334,7 +1342,7 @@
     <tableColumn id="1" xr3:uid="{C29E963F-354B-4750-B17F-22461F6DC5F4}" name="Name"/>
     <tableColumn id="3" xr3:uid="{7C7B0B32-2D9C-4EDB-8E56-4C2ADECB5869}" name="Type"/>
     <tableColumn id="2" xr3:uid="{1155C0CA-025A-4922-8B0E-F2A817B3BB60}" name="Qty"/>
-    <tableColumn id="8" xr3:uid="{D743202E-D377-4920-815B-09F9ED9CC36B}" name="Value" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{D743202E-D377-4920-815B-09F9ED9CC36B}" name="Value" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1658,33 +1666,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5AA6A1-7D43-4966-8813-F497D895A5C2}">
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1716,11 +1724,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E3" s="1"/>
       <c r="I3" s="16"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1746,11 +1754,11 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1776,7 +1784,7 @@
         <v>45673</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1803,7 +1811,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1827,7 +1835,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1851,7 +1859,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1875,7 +1883,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1899,7 +1907,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1923,7 +1931,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="28.9">
+    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1949,7 +1957,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -1978,7 +1986,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="43.15">
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -2004,7 +2012,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -2028,7 +2036,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28.9">
+    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2054,7 +2062,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -2078,7 +2086,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -2104,7 +2112,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -2128,7 +2136,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="28.9">
+    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2157,11 +2165,11 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E22" s="1"/>
       <c r="I22" s="16"/>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2185,7 +2193,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2209,11 +2217,11 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E25" s="1"/>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -2239,7 +2247,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -2263,7 +2271,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -2287,7 +2295,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -2313,34 +2321,34 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="5:5">
+    <row r="34" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E34" s="1"/>
     </row>
-    <row r="35" spans="5:5">
+    <row r="35" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="5:5">
+    <row r="36" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="5:5">
+    <row r="37" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E37" s="1"/>
     </row>
-    <row r="38" spans="5:5">
+    <row r="38" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="5:5">
+    <row r="39" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E39" s="1"/>
     </row>
   </sheetData>
@@ -2373,29 +2381,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DEA6183-B753-401C-B21E-C502785DFA3D}">
   <dimension ref="A1:G63"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" style="12" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.5546875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2418,7 +2426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
@@ -2439,7 +2447,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>57</v>
       </c>
@@ -2460,7 +2468,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1">
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>57</v>
       </c>
@@ -2483,7 +2491,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.15">
+    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>57</v>
       </c>
@@ -2506,7 +2514,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>57</v>
       </c>
@@ -2527,7 +2535,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="28.9">
+    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>57</v>
       </c>
@@ -2550,7 +2558,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
@@ -2571,7 +2579,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
       <c r="B10" s="14"/>
       <c r="C10" s="9"/>
@@ -2580,7 +2588,7 @@
       <c r="F10" s="9"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>57</v>
       </c>
@@ -2601,7 +2609,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="57.6">
+    <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>61</v>
       </c>
@@ -2624,7 +2632,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>61</v>
       </c>
@@ -2647,7 +2655,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>61</v>
       </c>
@@ -2668,7 +2676,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>61</v>
       </c>
@@ -2689,7 +2697,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>61</v>
       </c>
@@ -2710,7 +2718,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>61</v>
       </c>
@@ -2731,7 +2739,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>61</v>
       </c>
@@ -2752,7 +2760,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>61</v>
       </c>
@@ -2773,7 +2781,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>61</v>
       </c>
@@ -2794,7 +2802,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>61</v>
       </c>
@@ -2815,7 +2823,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>64</v>
       </c>
@@ -2836,7 +2844,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>65</v>
       </c>
@@ -2859,7 +2867,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>64</v>
       </c>
@@ -2880,7 +2888,7 @@
         <v>46052</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>64</v>
       </c>
@@ -2899,7 +2907,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="13"/>
       <c r="C26" s="5"/>
@@ -2908,7 +2916,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>64</v>
       </c>
@@ -2931,7 +2939,7 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>68</v>
       </c>
@@ -2952,7 +2960,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>69</v>
       </c>
@@ -2975,7 +2983,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>71</v>
       </c>
@@ -2998,7 +3006,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>73</v>
       </c>
@@ -3019,7 +3027,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>74</v>
       </c>
@@ -3040,7 +3048,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>75</v>
       </c>
@@ -3061,7 +3069,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>73</v>
       </c>
@@ -3082,7 +3090,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>76</v>
       </c>
@@ -3103,7 +3111,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -3126,7 +3134,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>64</v>
       </c>
@@ -3149,7 +3157,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -3169,7 +3177,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -3189,7 +3197,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>64</v>
       </c>
@@ -3212,7 +3220,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -3235,10 +3243,10 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G42" s="16"/>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -3258,7 +3266,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>81</v>
       </c>
@@ -3278,7 +3286,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>81</v>
       </c>
@@ -3298,7 +3306,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>86</v>
       </c>
@@ -3321,7 +3329,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -3344,7 +3352,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -3364,7 +3372,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>89</v>
       </c>
@@ -3381,7 +3389,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>91</v>
       </c>
@@ -3401,7 +3409,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>92</v>
       </c>
@@ -3421,7 +3429,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>93</v>
       </c>
@@ -3441,7 +3449,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>94</v>
       </c>
@@ -3464,7 +3472,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>97</v>
       </c>
@@ -3484,7 +3492,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -3507,7 +3515,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>100</v>
       </c>
@@ -3527,7 +3535,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>91</v>
       </c>
@@ -3547,7 +3555,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -3567,7 +3575,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -3590,16 +3598,16 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G60" s="16"/>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G61" s="16"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G62" s="16"/>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G63" s="16"/>
     </row>
   </sheetData>
@@ -3607,10 +3615,10 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:G63">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3629,33 +3637,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F948288C-1730-49D1-BD4C-FC704F167D22}">
   <dimension ref="A1:I33"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -3684,7 +3692,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>103</v>
       </c>
@@ -3713,7 +3721,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>103</v>
       </c>
@@ -3742,91 +3750,91 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="5:5">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="5:5">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="5:5">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="5:5">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="5:5">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="5:5">
+    <row r="22" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="5:5">
+    <row r="23" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="5:5">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="5:5">
+    <row r="25" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="5:5">
+    <row r="26" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="5:5">
+    <row r="27" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="5:5">
+    <row r="28" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="5:5">
+    <row r="29" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="5:5">
+    <row r="30" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="5:5">
+    <row r="31" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="5:5">
+    <row r="32" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="1"/>
     </row>
   </sheetData>
@@ -3858,38 +3866,38 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE86381-3E33-4CB8-A62B-E48A74AB9667}">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.33203125" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="17.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" style="19" customWidth="1"/>
-    <col min="11" max="11" width="21.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="19" customWidth="1"/>
+    <col min="11" max="11" width="21.33203125" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="14.45">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-    </row>
-    <row r="2" spans="1:12" ht="14.45">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+    </row>
+    <row r="2" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -3927,7 +3935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="14.45">
+    <row r="3" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -3963,7 +3971,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="14.45">
+    <row r="4" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>125</v>
       </c>
@@ -3999,7 +4007,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="14.45">
+    <row r="5" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>128</v>
       </c>
@@ -4035,10 +4043,10 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="14.45">
+    <row r="6" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:12" ht="14.45">
+    <row r="7" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>128</v>
       </c>
@@ -4074,7 +4082,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="14.45">
+    <row r="8" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>84</v>
       </c>
@@ -4110,7 +4118,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="14.45">
+    <row r="9" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>133</v>
       </c>
@@ -4146,10 +4154,10 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="14.45">
+    <row r="10" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:12" ht="14.45">
+    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -4185,7 +4193,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="14.45">
+    <row r="12" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>138</v>
       </c>
@@ -4220,7 +4228,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="14.45">
+    <row r="13" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>140</v>
       </c>
@@ -4256,7 +4264,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1">
+    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -4292,7 +4300,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1">
+    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -4328,7 +4336,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1">
+    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -4364,7 +4372,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15" customHeight="1">
+    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>146</v>
       </c>
@@ -4400,7 +4408,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15" customHeight="1">
+    <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>149</v>
       </c>
@@ -4436,7 +4444,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="15" customHeight="1">
+    <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>149</v>
       </c>
@@ -4472,7 +4480,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1">
+    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>151</v>
       </c>
@@ -4508,7 +4516,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15" customHeight="1">
+    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>151</v>
       </c>
@@ -4544,7 +4552,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15" customHeight="1">
+    <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>61</v>
       </c>
@@ -4580,7 +4588,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15" customHeight="1">
+    <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>154</v>
       </c>
@@ -4616,7 +4624,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15" customHeight="1">
+    <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>57</v>
       </c>
@@ -4652,7 +4660,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15" customHeight="1">
+    <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>128</v>
       </c>
@@ -4688,7 +4696,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="15" customHeight="1">
+    <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -4724,7 +4732,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="15" customHeight="1">
+    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -4760,7 +4768,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="15" customHeight="1">
+    <row r="28" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>64</v>
       </c>
@@ -4796,7 +4804,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="15" customHeight="1">
+    <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>159</v>
       </c>
@@ -4832,16 +4840,16 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="15" customHeight="1">
+    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:12" ht="15" customHeight="1">
+    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:12" ht="15" customHeight="1">
+    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="11:11" ht="15" customHeight="1">
+    <row r="33" spans="11:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K33" s="1"/>
     </row>
   </sheetData>
@@ -4849,36 +4857,36 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="A27:A28">
-    <cfRule type="expression" dxfId="21" priority="17">
+    <cfRule type="expression" dxfId="13" priority="17">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="18">
+    <cfRule type="expression" dxfId="12" priority="18">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:K9 A11:K14 A15:C15 E15:K15 A16:K25">
-    <cfRule type="expression" dxfId="19" priority="21">
+    <cfRule type="expression" dxfId="11" priority="21">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:L9 A11:L14 A15:C15 E15:L15 A16:L25">
-    <cfRule type="expression" dxfId="18" priority="22">
+    <cfRule type="expression" dxfId="10" priority="22">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G26:G29">
-    <cfRule type="expression" dxfId="17" priority="9">
+    <cfRule type="expression" dxfId="9" priority="9">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="10">
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26:H29">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4900,27 +4908,28 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1C144A-BB57-4446-B714-000D1D9FAB4A}">
-  <dimension ref="A1:O59"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:P59"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" customWidth="1"/>
-    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.28515625" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" style="16" customWidth="1"/>
-    <col min="13" max="13" width="29.140625" customWidth="1"/>
-    <col min="14" max="14" width="27.7109375" customWidth="1"/>
-    <col min="15" max="15" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.33203125" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" style="16" customWidth="1"/>
+    <col min="13" max="13" width="33.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="27.6640625" customWidth="1"/>
+    <col min="16" max="16" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15" customHeight="1">
+    <row r="1" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="17" t="s">
         <v>161</v>
       </c>
@@ -4934,15 +4943,16 @@
       <c r="J1" s="20"/>
       <c r="K1" s="18"/>
       <c r="L1" s="22"/>
-      <c r="M1" s="18"/>
-      <c r="N1" t="s">
+      <c r="M1" s="22"/>
+      <c r="N1" s="18"/>
+      <c r="O1" t="s">
         <v>162</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="14.45">
+    <row r="2" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -4979,19 +4989,22 @@
       <c r="L2" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" t="s">
+        <v>249</v>
+      </c>
+      <c r="O2" s="2">
         <f>SUM(J3:J38)</f>
         <v>9870</v>
       </c>
-      <c r="O2">
-        <f>COUNTIF(M3:M42,"*International*")</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="14.45">
+      <c r="P2">
+        <f>COUNTIF(N3:N42,"*International*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>166</v>
       </c>
@@ -5014,11 +5027,14 @@
       <c r="L3" s="15">
         <v>45970</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="14.45">
+      <c r="N3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>166</v>
       </c>
@@ -5041,11 +5057,14 @@
       <c r="L4" s="15">
         <v>45970</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="14.45">
+      <c r="N4" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>166</v>
       </c>
@@ -5068,11 +5087,14 @@
       <c r="L5" s="15">
         <v>45970</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" ht="14.45">
+      <c r="N5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>166</v>
       </c>
@@ -5095,11 +5117,14 @@
       <c r="L6" s="15">
         <v>45970</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M6" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="14.45">
+      <c r="N6" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>166</v>
       </c>
@@ -5122,11 +5147,14 @@
       <c r="L7" s="15">
         <v>45970</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" ht="14.45">
+      <c r="N7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>166</v>
       </c>
@@ -5149,11 +5177,14 @@
       <c r="L8" s="15">
         <v>45970</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="14.45">
+      <c r="N8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>166</v>
       </c>
@@ -5176,11 +5207,14 @@
       <c r="L9" s="15">
         <v>45970</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="14.45">
+      <c r="N9" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>168</v>
       </c>
@@ -5215,11 +5249,14 @@
       <c r="L10" s="15">
         <v>45999</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" ht="14.45">
+      <c r="N10" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>170</v>
       </c>
@@ -5254,11 +5291,14 @@
       <c r="L11" s="15">
         <v>45999</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" ht="14.45">
+      <c r="N11" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>172</v>
       </c>
@@ -5295,11 +5335,14 @@
       <c r="L12" s="15">
         <v>45999</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" ht="14.45">
+      <c r="N12" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>175</v>
       </c>
@@ -5334,11 +5377,14 @@
       <c r="L13" s="15">
         <v>45999</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" ht="14.45">
+      <c r="N13" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>168</v>
       </c>
@@ -5373,11 +5419,14 @@
       <c r="L14" s="15">
         <v>45999</v>
       </c>
-      <c r="M14" t="s">
+      <c r="M14" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" ht="14.45">
+      <c r="N14" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>177</v>
       </c>
@@ -5412,11 +5461,14 @@
       <c r="L15" s="15">
         <v>45999</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M15" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" ht="14.45">
+      <c r="N15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>179</v>
       </c>
@@ -5453,11 +5505,14 @@
       <c r="L16" s="15">
         <v>45999</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M16" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" ht="14.45">
+      <c r="N16" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>186</v>
       </c>
@@ -5494,11 +5549,14 @@
       <c r="L17" s="15">
         <v>45999</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="15" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" ht="14.45">
+      <c r="N17" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>187</v>
       </c>
@@ -5535,11 +5593,14 @@
       <c r="L18" s="16">
         <v>46043</v>
       </c>
-      <c r="M18" t="s">
+      <c r="M18" s="16" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" ht="14.45">
+      <c r="N18" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>64</v>
       </c>
@@ -5576,11 +5637,14 @@
       <c r="L19" s="16">
         <v>46043</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M19" s="16" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" ht="28.9">
+      <c r="N19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -5617,11 +5681,14 @@
       <c r="L20" s="15">
         <v>46056</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" ht="14.45">
+      <c r="N20" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>196</v>
       </c>
@@ -5656,11 +5723,14 @@
       <c r="L21" s="15">
         <v>46056</v>
       </c>
-      <c r="M21" t="s">
+      <c r="M21" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" ht="14.45">
+      <c r="N21" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -5695,11 +5765,14 @@
       <c r="L22" s="15">
         <v>46056</v>
       </c>
-      <c r="M22" t="s">
+      <c r="M22" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" ht="14.45">
+      <c r="N22" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -5734,11 +5807,14 @@
       <c r="L23" s="15">
         <v>46056</v>
       </c>
-      <c r="M23" t="s">
+      <c r="M23" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" ht="14.45">
+      <c r="N23" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -5773,11 +5849,14 @@
       <c r="L24" s="15">
         <v>46056</v>
       </c>
-      <c r="M24" t="s">
+      <c r="M24" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" ht="14.45">
+      <c r="N24" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -5812,11 +5891,14 @@
       <c r="L25" s="15">
         <v>46056</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M25" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" ht="14.45">
+      <c r="N25" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -5851,11 +5933,14 @@
       <c r="L26" s="15">
         <v>46056</v>
       </c>
-      <c r="M26" t="s">
+      <c r="M26" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" ht="14.45">
+      <c r="N26" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>61</v>
       </c>
@@ -5890,11 +5975,14 @@
       <c r="L27" s="15">
         <v>46056</v>
       </c>
-      <c r="M27" t="s">
+      <c r="M27" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" ht="14.45">
+      <c r="N27" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>199</v>
       </c>
@@ -5929,11 +6017,14 @@
       <c r="L28" s="15">
         <v>46056</v>
       </c>
-      <c r="M28" t="s">
+      <c r="M28" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" ht="14.45">
+      <c r="N28" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>199</v>
       </c>
@@ -5968,11 +6059,14 @@
       <c r="L29" s="15">
         <v>46056</v>
       </c>
-      <c r="M29" t="s">
+      <c r="M29" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" ht="14.45">
+      <c r="N29" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>128</v>
       </c>
@@ -6007,11 +6101,14 @@
       <c r="L30" s="15">
         <v>46056</v>
       </c>
-      <c r="M30" t="s">
+      <c r="M30" s="15" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" ht="14.45">
+      <c r="N30" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>61</v>
       </c>
@@ -6046,11 +6143,14 @@
       <c r="L31" s="16">
         <v>46058</v>
       </c>
-      <c r="M31" t="s">
+      <c r="M31" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" ht="14.45">
+      <c r="N31" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>61</v>
       </c>
@@ -6084,11 +6184,14 @@
       <c r="L32" s="16">
         <v>46058</v>
       </c>
-      <c r="M32" t="s">
+      <c r="M32" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" ht="14.45">
+      <c r="N32" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>61</v>
       </c>
@@ -6122,11 +6225,14 @@
       <c r="L33" s="16">
         <v>46058</v>
       </c>
-      <c r="M33" t="s">
+      <c r="M33" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" ht="14.45">
+      <c r="N33" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>203</v>
       </c>
@@ -6160,11 +6266,14 @@
       <c r="L34" s="16">
         <v>46058</v>
       </c>
-      <c r="M34" t="s">
+      <c r="M34" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" ht="14.45">
+      <c r="N34" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>203</v>
       </c>
@@ -6198,11 +6307,14 @@
       <c r="L35" s="16">
         <v>46058</v>
       </c>
-      <c r="M35" t="s">
+      <c r="M35" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" ht="14.45">
+      <c r="N35" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>203</v>
       </c>
@@ -6236,11 +6348,14 @@
       <c r="L36" s="16">
         <v>46058</v>
       </c>
-      <c r="M36" t="s">
+      <c r="M36" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" ht="14.45">
+      <c r="N36" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>203</v>
       </c>
@@ -6274,11 +6389,14 @@
       <c r="L37" s="16">
         <v>46058</v>
       </c>
-      <c r="M37" t="s">
+      <c r="M37" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" ht="14.45">
+      <c r="N37" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>203</v>
       </c>
@@ -6312,11 +6430,14 @@
       <c r="L38" s="16">
         <v>46058</v>
       </c>
-      <c r="M38" t="s">
+      <c r="M38" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" ht="14.45">
+      <c r="N38" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>203</v>
       </c>
@@ -6350,11 +6471,14 @@
       <c r="L39" s="16">
         <v>46058</v>
       </c>
-      <c r="M39" t="s">
+      <c r="M39" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" ht="15" customHeight="1">
+      <c r="N39" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>203</v>
       </c>
@@ -6388,11 +6512,14 @@
       <c r="L40" s="16">
         <v>46058</v>
       </c>
-      <c r="M40" t="s">
+      <c r="M40" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" ht="15" customHeight="1">
+      <c r="N40" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>203</v>
       </c>
@@ -6426,11 +6553,14 @@
       <c r="L41" s="16">
         <v>46058</v>
       </c>
-      <c r="M41" t="s">
+      <c r="M41" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" ht="15" customHeight="1">
+      <c r="N41" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>203</v>
       </c>
@@ -6464,11 +6594,14 @@
       <c r="L42" s="16">
         <v>46058</v>
       </c>
-      <c r="M42" t="s">
+      <c r="M42" s="16" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" ht="15" customHeight="1">
+      <c r="N42" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>140</v>
       </c>
@@ -6503,11 +6636,14 @@
       <c r="L43" s="16">
         <v>46078</v>
       </c>
-      <c r="M43" t="s">
+      <c r="M43" s="16" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" ht="15" customHeight="1">
+      <c r="N43" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>61</v>
       </c>
@@ -6542,71 +6678,89 @@
       <c r="L44" s="16">
         <v>46099</v>
       </c>
-      <c r="M44" t="s">
+      <c r="M44" s="16" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" ht="15" customHeight="1">
+      <c r="N44" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L45" s="15"/>
-    </row>
-    <row r="46" spans="1:13" ht="15" customHeight="1">
+      <c r="M45" s="15"/>
+    </row>
+    <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L46" s="15"/>
-    </row>
-    <row r="47" spans="1:13" ht="15" customHeight="1">
+      <c r="M46" s="15"/>
+    </row>
+    <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L47" s="15"/>
-    </row>
-    <row r="48" spans="1:13" ht="15" customHeight="1">
+      <c r="M47" s="15"/>
+    </row>
+    <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L48" s="15"/>
-    </row>
-    <row r="49" spans="12:12" ht="15" customHeight="1">
+      <c r="M48" s="15"/>
+    </row>
+    <row r="49" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L49" s="15"/>
-    </row>
-    <row r="50" spans="12:12" ht="15" customHeight="1">
+      <c r="M49" s="15"/>
+    </row>
+    <row r="50" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L50" s="15"/>
-    </row>
-    <row r="51" spans="12:12" ht="15" customHeight="1">
+      <c r="M50" s="15"/>
+    </row>
+    <row r="51" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L51" s="15"/>
-    </row>
-    <row r="52" spans="12:12" ht="15" customHeight="1">
+      <c r="M51" s="15"/>
+    </row>
+    <row r="52" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L52" s="15"/>
-    </row>
-    <row r="53" spans="12:12" ht="15" customHeight="1">
+      <c r="M52" s="15"/>
+    </row>
+    <row r="53" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L53" s="15"/>
-    </row>
-    <row r="54" spans="12:12" ht="15" customHeight="1">
+      <c r="M53" s="15"/>
+    </row>
+    <row r="54" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L54" s="15"/>
-    </row>
-    <row r="55" spans="12:12" ht="15" customHeight="1">
+      <c r="M54" s="15"/>
+    </row>
+    <row r="55" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L55" s="15"/>
-    </row>
-    <row r="56" spans="12:12" ht="15" customHeight="1">
+      <c r="M55" s="15"/>
+    </row>
+    <row r="56" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L56" s="15"/>
-    </row>
-    <row r="57" spans="12:12" ht="15" customHeight="1">
+      <c r="M56" s="15"/>
+    </row>
+    <row r="57" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L57" s="15"/>
-    </row>
-    <row r="58" spans="12:12" ht="15" customHeight="1">
+      <c r="M57" s="15"/>
+    </row>
+    <row r="58" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L58" s="15"/>
-    </row>
-    <row r="59" spans="12:12" ht="15" customHeight="1">
+      <c r="M58" s="15"/>
+    </row>
+    <row r="59" spans="12:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L59" s="15"/>
+      <c r="M59" s="15"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A44:F44 H44:K44">
-    <cfRule type="expression" dxfId="10" priority="5">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A44:F44 H44:L44">
-    <cfRule type="expression" dxfId="9" priority="6">
+  <conditionalFormatting sqref="A44:F44 H44:M44">
+    <cfRule type="expression" dxfId="4" priority="6">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:M9 A10:G15 I10:M15 A16:M43 M44 A45:M59">
+  <conditionalFormatting sqref="A3:N9 A10:G15 I10:N15 A16:N43 N44 A45:N59">
     <cfRule type="expression" priority="7">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6614,15 +6768,15 @@
     <cfRule type="expression" priority="3">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H15">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6631,7 +6785,7 @@
       <formula1>1</formula1>
       <formula2>2000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1 L1:L42 L45:L1048576" xr:uid="{A9EBE1C3-8923-4578-8214-596FAC33FDB8}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N1 L1:M42 L45:M1048576" xr:uid="{A9EBE1C3-8923-4578-8214-596FAC33FDB8}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B17 B19 B21:B29 B31:B42" xr:uid="{C7FD23E6-3E08-4DF7-8556-C07E455C4835}">
       <formula1>"Desktop,Laptop,Tablet,All-In-One"</formula1>
     </dataValidation>
@@ -6646,25 +6800,25 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6146040A-3AF4-440D-9E03-57379B2EC394}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+    </row>
+    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>208</v>
       </c>
@@ -6681,7 +6835,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>213</v>
       </c>
@@ -6695,7 +6849,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>215</v>
       </c>
@@ -6709,7 +6863,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>216</v>
       </c>
@@ -6726,7 +6880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>216</v>
       </c>
@@ -6743,7 +6897,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>216</v>
       </c>
@@ -6760,7 +6914,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>216</v>
       </c>
@@ -6777,7 +6931,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>216</v>
       </c>
@@ -6794,7 +6948,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>216</v>
       </c>
@@ -6811,7 +6965,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>216</v>
       </c>
@@ -6828,7 +6982,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>225</v>
       </c>
@@ -6845,7 +6999,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>225</v>
       </c>
@@ -6862,7 +7016,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>225</v>
       </c>
@@ -6879,7 +7033,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>225</v>
       </c>
@@ -6896,7 +7050,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1">
+    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>227</v>
       </c>
@@ -6913,13 +7067,13 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="4:4" ht="15" customHeight="1">
+    <row r="17" spans="4:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D17" s="23"/>
     </row>
-    <row r="18" spans="4:4" ht="15" customHeight="1">
+    <row r="18" spans="4:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D18" s="23"/>
     </row>
-    <row r="19" spans="4:4" ht="15" customHeight="1">
+    <row r="19" spans="4:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D19" s="23"/>
     </row>
   </sheetData>
@@ -6936,23 +7090,23 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3F77F78-0898-4060-A2C7-C1A84336B28A}">
   <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.140625" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="19" customWidth="1"/>
+    <col min="1" max="1" width="33.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
         <v>229</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="28"/>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="24"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>230</v>
       </c>
@@ -6966,7 +7120,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>231</v>
       </c>
@@ -6980,7 +7134,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>233</v>
       </c>
@@ -6994,7 +7148,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>234</v>
       </c>
@@ -7008,7 +7162,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>236</v>
       </c>
@@ -7022,7 +7176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>237</v>
       </c>
@@ -7036,7 +7190,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>239</v>
       </c>
@@ -7050,7 +7204,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>240</v>
       </c>
@@ -7064,7 +7218,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>242</v>
       </c>
@@ -7078,7 +7232,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>244</v>
       </c>
@@ -7092,7 +7246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>245</v>
       </c>
@@ -7106,7 +7260,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>247</v>
       </c>
@@ -7120,7 +7274,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>248</v>
       </c>
@@ -7134,26 +7288,26 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:4"/>
-    <row r="16" spans="1:4"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3"/>
+    <row r="17" x14ac:dyDescent="0.3"/>
+    <row r="18" x14ac:dyDescent="0.3"/>
+    <row r="19" x14ac:dyDescent="0.3"/>
+    <row r="20" x14ac:dyDescent="0.3"/>
+    <row r="21" x14ac:dyDescent="0.3"/>
+    <row r="22" x14ac:dyDescent="0.3"/>
+    <row r="23" x14ac:dyDescent="0.3"/>
+    <row r="24" x14ac:dyDescent="0.3"/>
+    <row r="25" x14ac:dyDescent="0.3"/>
+    <row r="26" x14ac:dyDescent="0.3"/>
+    <row r="27" x14ac:dyDescent="0.3"/>
+    <row r="28" x14ac:dyDescent="0.3"/>
+    <row r="29" x14ac:dyDescent="0.3"/>
+    <row r="30" x14ac:dyDescent="0.3"/>
+    <row r="31" x14ac:dyDescent="0.3"/>
+    <row r="32" x14ac:dyDescent="0.3"/>
+    <row r="33" x14ac:dyDescent="0.3"/>
+    <row r="34" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
importer still crashes but updated tool data without type and fixed typos in parts view
</commit_message>
<xml_diff>
--- a/data/OldInventorySystem.xlsx
+++ b/data/OldInventorySystem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rosehulman-my.sharepoint.com/personal/lucasja_rose-hulman_edu/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{556398BC-9AA0-4613-9E16-7C15B14402EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3822" documentId="8_{A0F2C8DF-695D-4A53-BA74-C2F5D1F57A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5D3BD5F-2075-44A1-91B0-CD25A0336B48}"/>
   <bookViews>
-    <workbookView xWindow="-315" yWindow="3510" windowWidth="19665" windowHeight="11055" firstSheet="1" activeTab="4" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="6" xr2:uid="{5168A3A3-41E7-40C2-87C5-8FD5FAD669C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Laptops" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="247">
   <si>
     <t>LAPTOPS</t>
   </si>
@@ -764,49 +764,31 @@
     <t>iFixit Moray Kit (complete)</t>
   </si>
   <si>
-    <t>Screwdriver Kit</t>
-  </si>
-  <si>
     <t>iFixit Pro Tech Toolkit (complete)</t>
   </si>
   <si>
     <t>iFixit Magnetic Screw Organizer</t>
   </si>
   <si>
-    <t>Screw Organizer</t>
-  </si>
-  <si>
     <t>Magnetic Parts Tray</t>
   </si>
   <si>
     <t>Anker Power Strip</t>
   </si>
   <si>
-    <t>Power Strip</t>
-  </si>
-  <si>
     <t>Generic Power Strip</t>
   </si>
   <si>
     <t>USB A to Ethernet</t>
   </si>
   <si>
-    <t>Adapter</t>
-  </si>
-  <si>
     <t>Duster</t>
   </si>
   <si>
-    <t>Miscellaneous</t>
-  </si>
-  <si>
     <t>USB Drive</t>
   </si>
   <si>
     <t>Goo Gone</t>
-  </si>
-  <si>
-    <t>Cleaning Supplies</t>
   </si>
   <si>
     <t>Isopropyl Alcohol</t>
@@ -824,7 +806,7 @@
     <numFmt numFmtId="164" formatCode="00000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -968,7 +950,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1026,6 +1008,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1038,41 +1022,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="30">
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1126,19 +1080,6 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -1242,12 +1183,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="00000"/>
-    </dxf>
-    <dxf>
       <font>
         <color theme="1"/>
       </font>
@@ -1273,7 +1208,50 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="00000"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1299,7 +1277,7 @@
     <tableColumn id="13" xr3:uid="{5BEE40AD-E450-4A13-BFB5-1D0CED084DB3}" name="ID"/>
     <tableColumn id="8" xr3:uid="{E9AB9B46-3541-4715-8E5B-024096D78342}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{F7DAC8DD-8096-40F1-8780-1DB9CB4EC72F}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{C5D14689-5BE8-4F27-9815-298E6CAC6990}" name="Special Reqs/Notes" dataDxfId="25"/>
     <tableColumn id="5" xr3:uid="{5338F6FB-43B0-44AF-AF8B-542FAC6CEDF0}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{64D6C993-8518-4A7C-9BDA-A54D7DBFBA8E}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{E5D987A3-C54A-4907-B710-79DB224E0008}" name="Current Status" totalsRowFunction="count"/>
@@ -1318,7 +1296,7 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F96A3CC8-25D1-4CF8-877D-2816B26B7DC4}" name="Item Name" totalsRowLabel="Total"/>
-    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{CC95B79B-E9C6-4478-8268-7B5E0708443A}" name="ID" dataDxfId="24"/>
     <tableColumn id="8" xr3:uid="{7D8F815E-A974-42A8-AC0B-AB8B951599A2}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{FEA94C75-B538-448A-A9F5-46F5A27E863D}" name="Year released"/>
     <tableColumn id="4" xr3:uid="{24998D92-36B7-4553-81E7-CB33711B31BB}" name="Special Reqs/Notes"/>
@@ -1340,7 +1318,7 @@
     <tableColumn id="13" xr3:uid="{EFFF3477-1A58-41CD-BFF3-45CE299505A7}" name="ID"/>
     <tableColumn id="8" xr3:uid="{C694899F-E385-4DE2-972A-7395A9633019}" name="Manufacturer"/>
     <tableColumn id="9" xr3:uid="{13C54556-A90A-4F9C-800D-3D838462DF46}" name="Year released"/>
-    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{EB0C81D5-20B7-428A-9A74-64C6C59A39B6}" name="Special Reqs/Notes" dataDxfId="23"/>
     <tableColumn id="5" xr3:uid="{6DE19FBC-9BD8-456E-9FC5-F633F61E4A34}" name="Charger"/>
     <tableColumn id="6" xr3:uid="{68546225-0A78-43C1-A4F9-4D2E1DC008A3}" name="Working Battery"/>
     <tableColumn id="7" xr3:uid="{0D7FD365-4F73-4A57-B8A1-CFAC47267923}" name="Current Status" totalsRowFunction="count"/>
@@ -1351,7 +1329,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:M33" totalsRowShown="0" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}" name="Ready_To_Donate7" displayName="Ready_To_Donate7" ref="A2:M33" totalsRowShown="0" tableBorderDxfId="22">
   <autoFilter ref="A2:M33" xr:uid="{D92D5D5D-191C-4D78-B08D-0ABFBE06D7B2}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{73648E04-2EA1-4ADB-8E24-E7DDE01C0462}" name="Item"/>
@@ -1364,8 +1342,8 @@
     <tableColumn id="2" xr3:uid="{C85B34EB-06B2-40A8-BBCB-B5F170EF3F82}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{A686D1B3-031E-4544-A98D-8F3144FA62B0}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{AB29939A-0AF4-4451-A6F4-2144F8957E73}" name="SSD/HDD"/>
-    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{80B69989-1A34-4B32-B100-006B113A12B3}" name="Est. Value" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{46DBF7E9-A65E-495E-A2E7-C18169DE9637}" name="Notes" dataDxfId="20"/>
     <tableColumn id="12" xr3:uid="{67EC036F-98F6-4C6B-BDD7-99DB9B6ADF97}" name="ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1373,7 +1351,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10100501-D05A-423B-A036-4B5D9B2ECD20}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:O59" totalsRowShown="0" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10100501-D05A-423B-A036-4B5D9B2ECD20}" name="Ready_To_Donate" displayName="Ready_To_Donate" ref="A2:O59" totalsRowShown="0" tableBorderDxfId="29">
   <autoFilter ref="A2:O59" xr:uid="{06396574-0271-4522-ADDB-9465953585FF}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{549BC727-085C-45F5-9520-711A34B50F51}" name="Item"/>
@@ -1386,10 +1364,10 @@
     <tableColumn id="13" xr3:uid="{A9DF335A-A163-4AA9-8879-B5B359D716CC}" name="RAM Generation"/>
     <tableColumn id="7" xr3:uid="{03AC00D8-5308-407D-9BAC-3303A2B380B3}" name="Storage"/>
     <tableColumn id="8" xr3:uid="{CFFC1B93-1DA0-40C5-BC8E-01F5CAD8DB66}" name="SSD/HDD"/>
-    <tableColumn id="10" xr3:uid="{71AF2E6E-D071-4784-865B-CA65E73CD28D}" name="Est. Value" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{71AF2E6E-D071-4784-865B-CA65E73CD28D}" name="Est. Value" dataDxfId="28"/>
     <tableColumn id="12" xr3:uid="{EFA4DB39-7CD3-4AA7-9335-2FEE3F14CF55}" name="Notes"/>
-    <tableColumn id="9" xr3:uid="{2DC095C6-494B-405F-9E1B-C8849C64E6F1}" name="Date Donated" dataDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{4D76F748-9FDA-4C94-B04F-D8250CE6CE08}" name="Recipient" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{2DC095C6-494B-405F-9E1B-C8849C64E6F1}" name="Date Donated" dataDxfId="27"/>
+    <tableColumn id="14" xr3:uid="{4D76F748-9FDA-4C94-B04F-D8250CE6CE08}" name="Recipient" dataDxfId="26"/>
     <tableColumn id="2" xr3:uid="{77D1B06F-E180-45FD-ACE9-4BA0C5955E95}" name="Org?"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1403,7 +1381,7 @@
     <tableColumn id="1" xr3:uid="{A07F4B01-C838-4D46-AE29-85BAC951AA36}" name="Type"/>
     <tableColumn id="3" xr3:uid="{9AC978C2-FD83-43AA-9C69-BC026B4E6411}" name="Description"/>
     <tableColumn id="4" xr3:uid="{9B2129F6-659A-4DD2-94CF-8EC39B827718}" name="Qty"/>
-    <tableColumn id="5" xr3:uid="{C24221AA-BF54-4384-AC51-1C5D1D76BE99}" name="Donated?" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C24221AA-BF54-4384-AC51-1C5D1D76BE99}" name="Donated?" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{1B36C5CD-E753-4327-9D04-48D37AAB944F}" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1411,13 +1389,12 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1921E586-F6B8-46BF-BE64-CE91A4EEE8D6}" name="Parts56" displayName="Parts56" ref="A2:D34" totalsRowShown="0">
-  <autoFilter ref="A2:D34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1921E586-F6B8-46BF-BE64-CE91A4EEE8D6}" name="Parts56" displayName="Parts56" ref="A2:C34" totalsRowShown="0">
+  <autoFilter ref="A2:C34" xr:uid="{56EE61A1-6164-4CDE-8E4E-0C4F2D11BFE3}"/>
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{C29E963F-354B-4750-B17F-22461F6DC5F4}" name="Name"/>
-    <tableColumn id="3" xr3:uid="{7C7B0B32-2D9C-4EDB-8E56-4C2ADECB5869}" name="Type"/>
     <tableColumn id="2" xr3:uid="{1155C0CA-025A-4922-8B0E-F2A817B3BB60}" name="Qty"/>
-    <tableColumn id="8" xr3:uid="{D743202E-D377-4920-815B-09F9ED9CC36B}" name="Value" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{D743202E-D377-4920-815B-09F9ED9CC36B}" name="Value" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1741,33 +1718,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5AA6A1-7D43-4966-8813-F497D895A5C2}">
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1799,11 +1776,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E3" s="1"/>
       <c r="I3" s="16"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1829,11 +1806,11 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1859,7 +1836,7 @@
         <v>45673</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1886,7 +1863,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1910,7 +1887,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1934,7 +1911,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -1958,7 +1935,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1982,7 +1959,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -2006,7 +1983,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30">
+    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -2032,7 +2009,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -2061,7 +2038,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="45">
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -2087,7 +2064,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -2111,7 +2088,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="30">
+    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2137,7 +2114,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="30">
+    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -2163,7 +2140,7 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="30">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -2189,7 +2166,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>46</v>
       </c>
@@ -2213,7 +2190,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="30">
+    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -2242,11 +2219,11 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E22" s="1"/>
       <c r="I22" s="16"/>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2275,11 +2252,11 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E25" s="1"/>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:9" ht="30">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -2305,7 +2282,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -2329,7 +2306,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -2353,7 +2330,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>55</v>
       </c>
@@ -2379,34 +2356,34 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="5:5">
+    <row r="34" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E34" s="1"/>
     </row>
-    <row r="35" spans="5:5">
+    <row r="35" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="5:5">
+    <row r="36" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="5:5">
+    <row r="37" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E37" s="1"/>
     </row>
-    <row r="38" spans="5:5">
+    <row r="38" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="5:5">
+    <row r="39" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E39" s="1"/>
     </row>
   </sheetData>
@@ -2439,29 +2416,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DEA6183-B753-401C-B21E-C502785DFA3D}">
   <dimension ref="A1:G63"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" style="12" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.5546875" style="12" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2484,7 +2461,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>59</v>
       </c>
@@ -2505,7 +2482,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>59</v>
       </c>
@@ -2526,7 +2503,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1">
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>59</v>
       </c>
@@ -2549,7 +2526,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="45">
+    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>59</v>
       </c>
@@ -2572,7 +2549,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>59</v>
       </c>
@@ -2593,7 +2570,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30">
+    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
@@ -2616,7 +2593,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>59</v>
       </c>
@@ -2637,7 +2614,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
       <c r="B10" s="14"/>
       <c r="C10" s="9"/>
@@ -2646,7 +2623,7 @@
       <c r="F10" s="9"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>59</v>
       </c>
@@ -2667,7 +2644,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="60">
+    <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>63</v>
       </c>
@@ -2690,7 +2667,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>63</v>
       </c>
@@ -2713,7 +2690,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>63</v>
       </c>
@@ -2734,7 +2711,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>63</v>
       </c>
@@ -2755,7 +2732,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>63</v>
       </c>
@@ -2776,7 +2753,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>63</v>
       </c>
@@ -2797,7 +2774,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>63</v>
       </c>
@@ -2818,7 +2795,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>63</v>
       </c>
@@ -2839,7 +2816,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>63</v>
       </c>
@@ -2860,7 +2837,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>63</v>
       </c>
@@ -2881,7 +2858,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>66</v>
       </c>
@@ -2902,7 +2879,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>67</v>
       </c>
@@ -2925,7 +2902,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>66</v>
       </c>
@@ -2946,7 +2923,7 @@
         <v>46052</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>66</v>
       </c>
@@ -2967,7 +2944,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="13"/>
       <c r="C26" s="5"/>
@@ -2976,7 +2953,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>66</v>
       </c>
@@ -2999,7 +2976,7 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>70</v>
       </c>
@@ -3020,7 +2997,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>71</v>
       </c>
@@ -3043,7 +3020,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>73</v>
       </c>
@@ -3064,7 +3041,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>74</v>
       </c>
@@ -3085,7 +3062,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>75</v>
       </c>
@@ -3106,7 +3083,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>73</v>
       </c>
@@ -3127,7 +3104,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>76</v>
       </c>
@@ -3148,7 +3125,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -3171,7 +3148,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>66</v>
       </c>
@@ -3194,7 +3171,7 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -3214,7 +3191,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -3234,7 +3211,7 @@
         <v>46031</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>66</v>
       </c>
@@ -3257,7 +3234,7 @@
         <v>46057</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -3280,10 +3257,10 @@
         <v>46122</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G42" s="16"/>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -3303,7 +3280,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>81</v>
       </c>
@@ -3323,7 +3300,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>81</v>
       </c>
@@ -3343,7 +3320,7 @@
         <v>46066</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>86</v>
       </c>
@@ -3366,7 +3343,7 @@
         <v>46073</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -3389,7 +3366,7 @@
         <v>46108</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -3409,7 +3386,7 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>89</v>
       </c>
@@ -3426,10 +3403,10 @@
         <v>46092</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G50" s="16"/>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>91</v>
       </c>
@@ -3449,7 +3426,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>92</v>
       </c>
@@ -3469,7 +3446,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>93</v>
       </c>
@@ -3492,7 +3469,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>95</v>
       </c>
@@ -3515,7 +3492,7 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>97</v>
       </c>
@@ -3538,7 +3515,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>99</v>
       </c>
@@ -3561,7 +3538,7 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>100</v>
       </c>
@@ -3581,7 +3558,7 @@
         <v>46094</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -3601,7 +3578,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>66</v>
       </c>
@@ -3624,7 +3601,7 @@
         <v>46115</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>102</v>
       </c>
@@ -3647,24 +3624,24 @@
         <v>46136</v>
       </c>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G61" s="16"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G62" s="16"/>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G63" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A3:G28 A30:G59 A61:G63 B60:G60">
-    <cfRule type="expression" dxfId="28" priority="1">
+  <conditionalFormatting sqref="A3:G28 A30:G59 B60:G60 A61:G63">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="2">
+    <cfRule type="expression" dxfId="16" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3684,33 +3661,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F948288C-1730-49D1-BD4C-FC704F167D22}">
   <dimension ref="A1:I33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -3739,7 +3716,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>105</v>
       </c>
@@ -3768,7 +3745,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>105</v>
       </c>
@@ -3797,91 +3774,91 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="5:5">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="5:5">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="5:5">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="5:5">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="5:5">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="5:5">
+    <row r="22" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="5:5">
+    <row r="23" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="5:5">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="5:5">
+    <row r="25" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="5:5">
+    <row r="26" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="5:5">
+    <row r="27" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="5:5">
+    <row r="28" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="5:5">
+    <row r="29" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="5:5">
+    <row r="30" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="5:5">
+    <row r="31" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="5:5">
+    <row r="32" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="5:5">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="1"/>
     </row>
   </sheetData>
@@ -3913,40 +3890,40 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE86381-3E33-4CB8-A62B-E48A74AB9667}">
   <dimension ref="A1:M36"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="17.140625" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" style="19" customWidth="1"/>
-    <col min="12" max="12" width="21.28515625" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" customWidth="1"/>
+    <col min="9" max="9" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" style="19" customWidth="1"/>
+    <col min="12" max="12" width="21.33203125" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+    </row>
+    <row r="2" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>109</v>
       </c>
@@ -3987,7 +3964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>120</v>
       </c>
@@ -4026,7 +4003,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>126</v>
       </c>
@@ -4065,7 +4042,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -4104,10 +4081,10 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>129</v>
       </c>
@@ -4146,7 +4123,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>84</v>
       </c>
@@ -4185,7 +4162,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>134</v>
       </c>
@@ -4224,10 +4201,10 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>136</v>
       </c>
@@ -4266,7 +4243,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -4304,7 +4281,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>141</v>
       </c>
@@ -4343,7 +4320,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="15" customHeight="1">
+    <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>129</v>
       </c>
@@ -4382,7 +4359,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15" customHeight="1">
+    <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>143</v>
       </c>
@@ -4421,7 +4398,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="15" customHeight="1">
+    <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>145</v>
       </c>
@@ -4460,7 +4437,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="15" customHeight="1">
+    <row r="17" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>147</v>
       </c>
@@ -4499,7 +4476,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="15" customHeight="1">
+    <row r="18" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>150</v>
       </c>
@@ -4538,7 +4515,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="15" customHeight="1">
+    <row r="19" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>150</v>
       </c>
@@ -4577,7 +4554,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="15" customHeight="1">
+    <row r="20" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>152</v>
       </c>
@@ -4616,7 +4593,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="15" customHeight="1">
+    <row r="21" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>152</v>
       </c>
@@ -4655,7 +4632,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="15" customHeight="1">
+    <row r="22" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -4694,7 +4671,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="15" customHeight="1">
+    <row r="23" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>155</v>
       </c>
@@ -4733,7 +4710,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="15" customHeight="1">
+    <row r="24" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>59</v>
       </c>
@@ -4772,7 +4749,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="15" customHeight="1">
+    <row r="25" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>129</v>
       </c>
@@ -4811,7 +4788,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="15" customHeight="1">
+    <row r="26" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>157</v>
       </c>
@@ -4850,7 +4827,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="15" customHeight="1">
+    <row r="27" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>47</v>
       </c>
@@ -4889,11 +4866,11 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="15" customHeight="1">
+    <row r="28" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="31" t="s">
         <v>28</v>
       </c>
       <c r="C28" t="s">
@@ -4928,7 +4905,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="15" customHeight="1">
+    <row r="29" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>160</v>
       </c>
@@ -4967,11 +4944,11 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="15" customHeight="1">
+    <row r="30" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="B30" t="s">
         <v>12</v>
       </c>
       <c r="C30" t="s">
@@ -5008,16 +4985,16 @@
         <v>127</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="15" customHeight="1">
+    <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L31" s="1"/>
     </row>
-    <row r="32" spans="1:13" ht="15" customHeight="1">
+    <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L32" s="1"/>
     </row>
-    <row r="33" spans="3:12" ht="15" customHeight="1">
+    <row r="33" spans="3:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L33" s="1"/>
     </row>
-    <row r="36" spans="3:12" ht="15" customHeight="1">
+    <row r="36" spans="3:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C36" s="26"/>
       <c r="D36" s="27"/>
       <c r="E36" s="28"/>
@@ -5031,44 +5008,44 @@
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <conditionalFormatting sqref="A27:B28 A30:B30">
-    <cfRule type="expression" dxfId="24" priority="21">
+    <cfRule type="expression" dxfId="15" priority="21">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="22">
+    <cfRule type="expression" dxfId="14" priority="22">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:L9 A11:L14 A15:D15 F15:L15 A16:L25">
-    <cfRule type="expression" dxfId="22" priority="25">
+    <cfRule type="expression" dxfId="13" priority="25">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:M9 A11:M14 A15:D15 F15:M15 A16:M25">
-    <cfRule type="expression" dxfId="21" priority="26">
+    <cfRule type="expression" dxfId="12" priority="26">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C36:I36">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H26:H29">
-    <cfRule type="expression" dxfId="18" priority="13">
+    <cfRule type="expression" dxfId="9" priority="13">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="14">
+    <cfRule type="expression" dxfId="8" priority="14">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26:I29">
-    <cfRule type="expression" dxfId="16" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5094,28 +5071,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1C144A-BB57-4446-B714-000D1D9FAB4A}">
   <dimension ref="A1:Q59"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.28515625" style="19" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.28515625" customWidth="1"/>
-    <col min="13" max="13" width="16.85546875" style="16" customWidth="1"/>
-    <col min="14" max="14" width="33.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.109375" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" style="19" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.33203125" customWidth="1"/>
+    <col min="13" max="13" width="16.88671875" style="16" customWidth="1"/>
+    <col min="14" max="14" width="33.33203125" style="16" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="27.7109375" customWidth="1"/>
-    <col min="17" max="17" width="28.28515625" customWidth="1"/>
+    <col min="16" max="16" width="27.6640625" customWidth="1"/>
+    <col min="17" max="17" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" customHeight="1">
+    <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C1" s="17" t="s">
         <v>164</v>
       </c>
@@ -5138,7 +5115,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>109</v>
       </c>
@@ -5193,7 +5170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>170</v>
       </c>
@@ -5226,7 +5203,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>170</v>
       </c>
@@ -5259,7 +5236,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>170</v>
       </c>
@@ -5292,7 +5269,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>170</v>
       </c>
@@ -5325,7 +5302,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>170</v>
       </c>
@@ -5358,7 +5335,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>170</v>
       </c>
@@ -5391,7 +5368,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>170</v>
       </c>
@@ -5424,7 +5401,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>174</v>
       </c>
@@ -5469,7 +5446,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>176</v>
       </c>
@@ -5514,7 +5491,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>178</v>
       </c>
@@ -5561,7 +5538,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>181</v>
       </c>
@@ -5606,7 +5583,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>174</v>
       </c>
@@ -5651,7 +5628,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>183</v>
       </c>
@@ -5696,7 +5673,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>185</v>
       </c>
@@ -5743,7 +5720,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>192</v>
       </c>
@@ -5790,7 +5767,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>102</v>
       </c>
@@ -5818,8 +5795,8 @@
       <c r="I18">
         <v>256</v>
       </c>
-      <c r="J18" t="s">
-        <v>125</v>
+      <c r="J18">
+        <v>256</v>
       </c>
       <c r="K18" s="19">
         <v>250</v>
@@ -5837,7 +5814,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>66</v>
       </c>
@@ -5884,7 +5861,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="43.5">
+    <row r="20" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>63</v>
       </c>
@@ -5931,7 +5908,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>202</v>
       </c>
@@ -5976,7 +5953,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>66</v>
       </c>
@@ -6021,7 +5998,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -6066,7 +6043,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -6111,7 +6088,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -6156,7 +6133,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>63</v>
       </c>
@@ -6201,7 +6178,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>63</v>
       </c>
@@ -6246,7 +6223,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>205</v>
       </c>
@@ -6291,7 +6268,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>205</v>
       </c>
@@ -6336,7 +6313,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>129</v>
       </c>
@@ -6381,11 +6358,11 @@
         <v>173</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="38" t="s">
+      <c r="B31" s="32" t="s">
         <v>28</v>
       </c>
       <c r="C31" t="s">
@@ -6426,7 +6403,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -6470,7 +6447,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>63</v>
       </c>
@@ -6514,7 +6491,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>209</v>
       </c>
@@ -6558,7 +6535,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>209</v>
       </c>
@@ -6602,7 +6579,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>209</v>
       </c>
@@ -6646,7 +6623,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>209</v>
       </c>
@@ -6690,7 +6667,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>209</v>
       </c>
@@ -6734,7 +6711,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
+    <row r="39" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>209</v>
       </c>
@@ -6778,7 +6755,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="15" customHeight="1">
+    <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>209</v>
       </c>
@@ -6822,7 +6799,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="15" customHeight="1">
+    <row r="41" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>209</v>
       </c>
@@ -6866,7 +6843,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="15" customHeight="1">
+    <row r="42" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>209</v>
       </c>
@@ -6910,7 +6887,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="15" customHeight="1">
+    <row r="43" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>141</v>
       </c>
@@ -6955,11 +6932,11 @@
         <v>196</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="15" customHeight="1">
+    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B44" s="36" t="s">
+      <c r="B44" s="31" t="s">
         <v>28</v>
       </c>
       <c r="C44" t="s">
@@ -7000,82 +6977,82 @@
         <v>196</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="15" customHeight="1">
+    <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M45" s="15"/>
       <c r="N45" s="15"/>
     </row>
-    <row r="46" spans="1:15" ht="15" customHeight="1">
+    <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M46" s="15"/>
       <c r="N46" s="15"/>
     </row>
-    <row r="47" spans="1:15" ht="15" customHeight="1">
+    <row r="47" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M47" s="15"/>
       <c r="N47" s="15"/>
     </row>
-    <row r="48" spans="1:15" ht="15" customHeight="1">
+    <row r="48" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M48" s="15"/>
       <c r="N48" s="15"/>
     </row>
-    <row r="49" spans="13:14" ht="15" customHeight="1">
+    <row r="49" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M49" s="15"/>
       <c r="N49" s="15"/>
     </row>
-    <row r="50" spans="13:14" ht="15" customHeight="1">
+    <row r="50" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M50" s="15"/>
       <c r="N50" s="15"/>
     </row>
-    <row r="51" spans="13:14" ht="15" customHeight="1">
+    <row r="51" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M51" s="15"/>
       <c r="N51" s="15"/>
     </row>
-    <row r="52" spans="13:14" ht="15" customHeight="1">
+    <row r="52" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M52" s="15"/>
       <c r="N52" s="15"/>
     </row>
-    <row r="53" spans="13:14" ht="15" customHeight="1">
+    <row r="53" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M53" s="15"/>
       <c r="N53" s="15"/>
     </row>
-    <row r="54" spans="13:14" ht="15" customHeight="1">
+    <row r="54" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M54" s="15"/>
       <c r="N54" s="15"/>
     </row>
-    <row r="55" spans="13:14" ht="15" customHeight="1">
+    <row r="55" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M55" s="15"/>
       <c r="N55" s="15"/>
     </row>
-    <row r="56" spans="13:14" ht="15" customHeight="1">
+    <row r="56" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M56" s="15"/>
       <c r="N56" s="15"/>
     </row>
-    <row r="57" spans="13:14" ht="15" customHeight="1">
+    <row r="57" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M57" s="15"/>
       <c r="N57" s="15"/>
     </row>
-    <row r="58" spans="13:14" ht="15" customHeight="1">
+    <row r="58" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M58" s="15"/>
       <c r="N58" s="15"/>
     </row>
-    <row r="59" spans="13:14" ht="15" customHeight="1">
+    <row r="59" spans="13:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="M59" s="15"/>
       <c r="N59" s="15"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A44:G44 I44:L44">
-    <cfRule type="expression" dxfId="11" priority="5">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A44:G44 I44:N44">
-    <cfRule type="expression" dxfId="10" priority="6">
+    <cfRule type="expression" dxfId="4" priority="6">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:O9 A10:H15 J10:O15 O44 A45:O59 A16:O43">
+  <conditionalFormatting sqref="A3:O9 A10:H15 J10:O15 A16:O43 O44 A45:O59">
     <cfRule type="expression" priority="7">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="8">
+    <cfRule type="expression" dxfId="3" priority="8">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7083,15 +7060,15 @@
     <cfRule type="expression" priority="3">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:I15">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7115,25 +7092,25 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6146040A-3AF4-440D-9E03-57379B2EC394}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+    </row>
+    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>214</v>
       </c>
@@ -7150,7 +7127,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>219</v>
       </c>
@@ -7164,7 +7141,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>220</v>
       </c>
@@ -7178,7 +7155,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>221</v>
       </c>
@@ -7195,7 +7172,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>221</v>
       </c>
@@ -7212,7 +7189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>221</v>
       </c>
@@ -7229,7 +7206,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>221</v>
       </c>
@@ -7246,7 +7223,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>221</v>
       </c>
@@ -7263,7 +7240,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>221</v>
       </c>
@@ -7280,7 +7257,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>221</v>
       </c>
@@ -7297,7 +7274,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>229</v>
       </c>
@@ -7314,7 +7291,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>229</v>
       </c>
@@ -7331,7 +7308,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>229</v>
       </c>
@@ -7348,7 +7325,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>229</v>
       </c>
@@ -7365,7 +7342,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1">
+    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>231</v>
       </c>
@@ -7382,13 +7359,13 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="4:4" ht="15" customHeight="1">
+    <row r="17" spans="4:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D17" s="23"/>
     </row>
-    <row r="18" spans="4:4" ht="15" customHeight="1">
+    <row r="18" spans="4:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D18" s="23"/>
     </row>
-    <row r="19" spans="4:4" ht="15" customHeight="1">
+    <row r="19" spans="4:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D19" s="23"/>
     </row>
   </sheetData>
@@ -7404,208 +7381,167 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3F77F78-0898-4060-A2C7-C1A84336B28A}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.140625" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="19" customWidth="1"/>
+    <col min="1" max="1" width="33.109375" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" customHeight="1">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="35" t="s">
         <v>233</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="24"/>
-    </row>
-    <row r="2" spans="1:4" ht="15" customHeight="1">
+      <c r="B1" s="36"/>
+      <c r="C1" s="24"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>234</v>
       </c>
-      <c r="B2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="C2" s="21" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" customHeight="1">
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>235</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>236</v>
       </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3" s="19">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="19">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>237</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" s="19">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>238</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>239</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" s="19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9" s="19">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" s="19">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15" customHeight="1">
-      <c r="A4" t="s">
-        <v>237</v>
-      </c>
-      <c r="B4" t="s">
-        <v>236</v>
-      </c>
-      <c r="C4">
+    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>243</v>
+      </c>
+      <c r="B11">
+        <v>14</v>
+      </c>
+      <c r="C11" s="19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12">
         <v>1</v>
       </c>
-      <c r="D4" s="19">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" customHeight="1">
-      <c r="A5" t="s">
-        <v>238</v>
-      </c>
-      <c r="B5" t="s">
-        <v>239</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5" s="19">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" customHeight="1">
-      <c r="A6" t="s">
-        <v>240</v>
-      </c>
-      <c r="B6" t="s">
-        <v>239</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6" s="19">
+      <c r="C12" s="19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>245</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" s="19">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15" customHeight="1">
-      <c r="A7" t="s">
-        <v>241</v>
-      </c>
-      <c r="B7" t="s">
-        <v>242</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7" s="19">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1">
-      <c r="A8" t="s">
-        <v>243</v>
-      </c>
-      <c r="B8" t="s">
-        <v>242</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8" s="19">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" customHeight="1">
-      <c r="A9" t="s">
-        <v>244</v>
-      </c>
-      <c r="B9" t="s">
-        <v>245</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="D9" s="19">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" customHeight="1">
-      <c r="A10" t="s">
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>246</v>
       </c>
-      <c r="B10" t="s">
-        <v>247</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10" s="19">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1">
-      <c r="A11" t="s">
-        <v>248</v>
-      </c>
-      <c r="B11" t="s">
-        <v>247</v>
-      </c>
-      <c r="C11">
-        <v>14</v>
-      </c>
-      <c r="D11" s="19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" customHeight="1">
-      <c r="A12" t="s">
-        <v>249</v>
-      </c>
-      <c r="B12" t="s">
-        <v>250</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12" s="19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15" customHeight="1">
-      <c r="A13" t="s">
-        <v>251</v>
-      </c>
-      <c r="B13" t="s">
-        <v>250</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13" s="19">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15" customHeight="1">
-      <c r="A14" t="s">
-        <v>252</v>
-      </c>
-      <c r="B14" t="s">
-        <v>245</v>
-      </c>
-      <c r="C14">
+      <c r="B14">
         <v>6</v>
       </c>
-      <c r="D14" s="19">
+      <c r="C14" s="19">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>